<commit_message>
Treatments: add missing treatments to xlsx, repoint footer aliases
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/content/treatments.xlsx
+++ b/src/content/treatments.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="105">
   <si>
     <t>Title</t>
   </si>
@@ -214,6 +214,54 @@
   </si>
   <si>
     <t>joint-prp</t>
+  </si>
+  <si>
+    <t>Co2</t>
+  </si>
+  <si>
+    <t>co2</t>
+  </si>
+  <si>
+    <t>Miim Laser</t>
+  </si>
+  <si>
+    <t>miim-laser</t>
+  </si>
+  <si>
+    <t>Agnes</t>
+  </si>
+  <si>
+    <t>agnes</t>
+  </si>
+  <si>
+    <t>Noblex</t>
+  </si>
+  <si>
+    <t>noblex</t>
+  </si>
+  <si>
+    <t>Scarlet</t>
+  </si>
+  <si>
+    <t>scarlet</t>
+  </si>
+  <si>
+    <t>Shrink</t>
+  </si>
+  <si>
+    <t>shrink</t>
+  </si>
+  <si>
+    <t>V-Zet</t>
+  </si>
+  <si>
+    <t>v-zet</t>
+  </si>
+  <si>
+    <t>PDO Threads</t>
+  </si>
+  <si>
+    <t>pdo-threads</t>
   </si>
   <si>
     <t>Name</t>
@@ -1066,1887 +1114,1959 @@
       <c r="D29" s="2"/>
       <c r="G29" s="2"/>
     </row>
-    <row r="30" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>67</v>
+      </c>
+      <c r="B30" t="s">
+        <v>68</v>
+      </c>
+      <c r="C30" t="s">
+        <v>41</v>
+      </c>
       <c r="D30" s="2"/>
       <c r="G30" s="2"/>
     </row>
-    <row r="31" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>69</v>
+      </c>
+      <c r="B31" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" t="s">
+        <v>41</v>
+      </c>
       <c r="D31" s="2"/>
       <c r="G31" s="2"/>
     </row>
-    <row r="32" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>71</v>
+      </c>
+      <c r="B32" t="s">
+        <v>72</v>
+      </c>
+      <c r="C32" t="s">
+        <v>41</v>
+      </c>
       <c r="D32" s="2"/>
       <c r="G32" s="2"/>
     </row>
-    <row r="33" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>73</v>
+      </c>
+      <c r="B33" t="s">
+        <v>74</v>
+      </c>
+      <c r="C33" t="s">
+        <v>41</v>
+      </c>
       <c r="D33" s="2"/>
       <c r="G33" s="2"/>
     </row>
-    <row r="34" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>75</v>
+      </c>
+      <c r="B34" t="s">
+        <v>76</v>
+      </c>
+      <c r="C34" t="s">
+        <v>41</v>
+      </c>
       <c r="D34" s="2"/>
       <c r="G34" s="2"/>
     </row>
-    <row r="35" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>77</v>
+      </c>
+      <c r="B35" t="s">
+        <v>78</v>
+      </c>
+      <c r="C35" t="s">
+        <v>41</v>
+      </c>
       <c r="D35" s="2"/>
       <c r="G35" s="2"/>
     </row>
-    <row r="36" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" t="s">
+        <v>80</v>
+      </c>
+      <c r="C36" t="s">
+        <v>41</v>
+      </c>
       <c r="D36" s="2"/>
       <c r="G36" s="2"/>
     </row>
-    <row r="37" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>81</v>
+      </c>
+      <c r="B37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C37" t="s">
+        <v>22</v>
+      </c>
       <c r="D37" s="2"/>
       <c r="G37" s="2"/>
     </row>
-    <row r="38" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="38" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D38" s="2"/>
       <c r="G38" s="2"/>
     </row>
-    <row r="39" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="39" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D39" s="2"/>
       <c r="G39" s="2"/>
     </row>
-    <row r="40" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="40" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D40" s="2"/>
       <c r="G40" s="2"/>
     </row>
-    <row r="41" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="41" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D41" s="2"/>
       <c r="G41" s="2"/>
     </row>
-    <row r="42" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="42" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D42" s="2"/>
       <c r="G42" s="2"/>
     </row>
-    <row r="43" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="43" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D43" s="2"/>
       <c r="G43" s="2"/>
     </row>
-    <row r="44" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="44" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D44" s="2"/>
       <c r="G44" s="2"/>
     </row>
-    <row r="45" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="45" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D45" s="2"/>
       <c r="G45" s="2"/>
     </row>
-    <row r="46" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="46" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D46" s="2"/>
       <c r="G46" s="2"/>
     </row>
-    <row r="47" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="47" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D47" s="2"/>
       <c r="G47" s="2"/>
     </row>
-    <row r="48" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="48" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D48" s="2"/>
       <c r="G48" s="2"/>
     </row>
-    <row r="49" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D49" s="2"/>
       <c r="G49" s="2"/>
     </row>
-    <row r="50" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="50" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D50" s="2"/>
       <c r="G50" s="2"/>
     </row>
-    <row r="51" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="51" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D51" s="2"/>
       <c r="G51" s="2"/>
     </row>
-    <row r="52" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="52" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D52" s="2"/>
       <c r="G52" s="2"/>
     </row>
-    <row r="53" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="53" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D53" s="2"/>
       <c r="G53" s="2"/>
     </row>
-    <row r="54" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="54" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D54" s="2"/>
       <c r="G54" s="2"/>
     </row>
-    <row r="55" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="55" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D55" s="2"/>
       <c r="G55" s="2"/>
     </row>
-    <row r="56" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="56" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D56" s="2"/>
       <c r="G56" s="2"/>
     </row>
-    <row r="57" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="57" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D57" s="2"/>
       <c r="G57" s="2"/>
     </row>
-    <row r="58" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="58" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D58" s="2"/>
       <c r="G58" s="2"/>
     </row>
-    <row r="59" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="59" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D59" s="2"/>
       <c r="G59" s="2"/>
     </row>
-    <row r="60" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="60" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D60" s="2"/>
       <c r="G60" s="2"/>
     </row>
-    <row r="61" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="61" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D61" s="2"/>
       <c r="G61" s="2"/>
     </row>
-    <row r="62" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="62" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D62" s="2"/>
       <c r="G62" s="2"/>
     </row>
-    <row r="63" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="63" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D63" s="2"/>
       <c r="G63" s="2"/>
     </row>
-    <row r="64" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="64" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D64" s="2"/>
       <c r="G64" s="2"/>
     </row>
-    <row r="65" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="65" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D65" s="2"/>
       <c r="G65" s="2"/>
     </row>
-    <row r="66" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="66" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D66" s="2"/>
       <c r="G66" s="2"/>
     </row>
-    <row r="67" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="67" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D67" s="2"/>
       <c r="G67" s="2"/>
     </row>
-    <row r="68" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="68" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D68" s="2"/>
       <c r="G68" s="2"/>
     </row>
-    <row r="69" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="69" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D69" s="2"/>
       <c r="G69" s="2"/>
     </row>
-    <row r="70" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="70" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D70" s="2"/>
       <c r="G70" s="2"/>
     </row>
-    <row r="71" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="71" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D71" s="2"/>
       <c r="G71" s="2"/>
     </row>
-    <row r="72" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="72" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D72" s="2"/>
       <c r="G72" s="2"/>
     </row>
-    <row r="73" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="73" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D73" s="2"/>
       <c r="G73" s="2"/>
     </row>
-    <row r="74" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="74" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D74" s="2"/>
       <c r="G74" s="2"/>
     </row>
-    <row r="75" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="75" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D75" s="2"/>
       <c r="G75" s="2"/>
     </row>
-    <row r="76" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="76" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D76" s="2"/>
       <c r="G76" s="2"/>
     </row>
-    <row r="77" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="77" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D77" s="2"/>
       <c r="G77" s="2"/>
     </row>
-    <row r="78" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="78" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D78" s="2"/>
       <c r="G78" s="2"/>
     </row>
-    <row r="79" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="79" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D79" s="2"/>
       <c r="G79" s="2"/>
     </row>
-    <row r="80" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="80" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D80" s="2"/>
       <c r="G80" s="2"/>
     </row>
-    <row r="81" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="81" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D81" s="2"/>
       <c r="G81" s="2"/>
     </row>
-    <row r="82" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="82" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D82" s="2"/>
       <c r="G82" s="2"/>
     </row>
-    <row r="83" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="83" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D83" s="2"/>
       <c r="G83" s="2"/>
     </row>
-    <row r="84" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="84" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D84" s="2"/>
       <c r="G84" s="2"/>
     </row>
-    <row r="85" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="85" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D85" s="2"/>
       <c r="G85" s="2"/>
     </row>
-    <row r="86" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="86" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D86" s="2"/>
       <c r="G86" s="2"/>
     </row>
-    <row r="87" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="87" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D87" s="2"/>
       <c r="G87" s="2"/>
     </row>
-    <row r="88" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="88" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D88" s="2"/>
       <c r="G88" s="2"/>
     </row>
-    <row r="89" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="89" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D89" s="2"/>
       <c r="G89" s="2"/>
     </row>
-    <row r="90" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="90" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D90" s="2"/>
       <c r="G90" s="2"/>
     </row>
-    <row r="91" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="91" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D91" s="2"/>
       <c r="G91" s="2"/>
     </row>
-    <row r="92" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="92" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D92" s="2"/>
       <c r="G92" s="2"/>
     </row>
-    <row r="93" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="93" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D93" s="2"/>
       <c r="G93" s="2"/>
     </row>
-    <row r="94" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="94" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D94" s="2"/>
       <c r="G94" s="2"/>
     </row>
-    <row r="95" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="95" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D95" s="2"/>
       <c r="G95" s="2"/>
     </row>
-    <row r="96" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="96" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D96" s="2"/>
       <c r="G96" s="2"/>
     </row>
-    <row r="97" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="97" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D97" s="2"/>
       <c r="G97" s="2"/>
     </row>
-    <row r="98" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="98" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D98" s="2"/>
       <c r="G98" s="2"/>
     </row>
-    <row r="99" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="99" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D99" s="2"/>
       <c r="G99" s="2"/>
     </row>
-    <row r="100" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="100" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D100" s="2"/>
       <c r="G100" s="2"/>
     </row>
-    <row r="101" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="101" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D101" s="2"/>
       <c r="G101" s="2"/>
     </row>
-    <row r="102" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="102" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D102" s="2"/>
       <c r="G102" s="2"/>
     </row>
-    <row r="103" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="103" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D103" s="2"/>
       <c r="G103" s="2"/>
     </row>
-    <row r="104" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="104" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D104" s="2"/>
       <c r="G104" s="2"/>
     </row>
-    <row r="105" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="105" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D105" s="2"/>
       <c r="G105" s="2"/>
     </row>
-    <row r="106" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="106" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D106" s="2"/>
       <c r="G106" s="2"/>
     </row>
-    <row r="107" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="107" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D107" s="2"/>
       <c r="G107" s="2"/>
     </row>
-    <row r="108" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="108" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D108" s="2"/>
       <c r="G108" s="2"/>
     </row>
-    <row r="109" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="109" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D109" s="2"/>
       <c r="G109" s="2"/>
     </row>
-    <row r="110" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="110" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D110" s="2"/>
       <c r="G110" s="2"/>
     </row>
-    <row r="111" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="111" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D111" s="2"/>
       <c r="G111" s="2"/>
     </row>
-    <row r="112" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="112" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D112" s="2"/>
       <c r="G112" s="2"/>
     </row>
-    <row r="113" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="113" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D113" s="2"/>
       <c r="G113" s="2"/>
     </row>
-    <row r="114" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="114" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D114" s="2"/>
       <c r="G114" s="2"/>
     </row>
-    <row r="115" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="115" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D115" s="2"/>
       <c r="G115" s="2"/>
     </row>
-    <row r="116" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="116" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D116" s="2"/>
       <c r="G116" s="2"/>
     </row>
-    <row r="117" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="117" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D117" s="2"/>
       <c r="G117" s="2"/>
     </row>
-    <row r="118" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="118" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D118" s="2"/>
       <c r="G118" s="2"/>
     </row>
-    <row r="119" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="119" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D119" s="2"/>
       <c r="G119" s="2"/>
     </row>
-    <row r="120" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="120" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D120" s="2"/>
       <c r="G120" s="2"/>
     </row>
-    <row r="121" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="121" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D121" s="2"/>
       <c r="G121" s="2"/>
     </row>
-    <row r="122" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="122" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D122" s="2"/>
       <c r="G122" s="2"/>
     </row>
-    <row r="123" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="123" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D123" s="2"/>
       <c r="G123" s="2"/>
     </row>
-    <row r="124" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="124" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D124" s="2"/>
       <c r="G124" s="2"/>
     </row>
-    <row r="125" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="125" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D125" s="2"/>
       <c r="G125" s="2"/>
     </row>
-    <row r="126" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="126" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D126" s="2"/>
       <c r="G126" s="2"/>
     </row>
-    <row r="127" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="127" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D127" s="2"/>
       <c r="G127" s="2"/>
     </row>
-    <row r="128" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="128" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D128" s="2"/>
       <c r="G128" s="2"/>
     </row>
-    <row r="129" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="129" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D129" s="2"/>
       <c r="G129" s="2"/>
     </row>
-    <row r="130" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="130" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D130" s="2"/>
       <c r="G130" s="2"/>
     </row>
-    <row r="131" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="131" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D131" s="2"/>
       <c r="G131" s="2"/>
     </row>
-    <row r="132" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="132" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D132" s="2"/>
       <c r="G132" s="2"/>
     </row>
-    <row r="133" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="133" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D133" s="2"/>
       <c r="G133" s="2"/>
     </row>
-    <row r="134" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="134" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D134" s="2"/>
       <c r="G134" s="2"/>
     </row>
-    <row r="135" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="135" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D135" s="2"/>
       <c r="G135" s="2"/>
     </row>
-    <row r="136" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="136" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D136" s="2"/>
       <c r="G136" s="2"/>
     </row>
-    <row r="137" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="137" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D137" s="2"/>
       <c r="G137" s="2"/>
     </row>
-    <row r="138" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="138" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D138" s="2"/>
       <c r="G138" s="2"/>
     </row>
-    <row r="139" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="139" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D139" s="2"/>
       <c r="G139" s="2"/>
     </row>
-    <row r="140" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="140" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D140" s="2"/>
       <c r="G140" s="2"/>
     </row>
-    <row r="141" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="141" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D141" s="2"/>
       <c r="G141" s="2"/>
     </row>
-    <row r="142" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="142" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D142" s="2"/>
       <c r="G142" s="2"/>
     </row>
-    <row r="143" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="143" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D143" s="2"/>
       <c r="G143" s="2"/>
     </row>
-    <row r="144" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="144" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D144" s="2"/>
       <c r="G144" s="2"/>
     </row>
-    <row r="145" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="145" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D145" s="2"/>
       <c r="G145" s="2"/>
     </row>
-    <row r="146" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="146" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D146" s="2"/>
       <c r="G146" s="2"/>
     </row>
-    <row r="147" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="147" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D147" s="2"/>
       <c r="G147" s="2"/>
     </row>
-    <row r="148" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="148" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D148" s="2"/>
       <c r="G148" s="2"/>
     </row>
-    <row r="149" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="149" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D149" s="2"/>
       <c r="G149" s="2"/>
     </row>
-    <row r="150" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="150" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D150" s="2"/>
       <c r="G150" s="2"/>
     </row>
-    <row r="151" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="151" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D151" s="2"/>
       <c r="G151" s="2"/>
     </row>
-    <row r="152" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="152" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D152" s="2"/>
       <c r="G152" s="2"/>
     </row>
-    <row r="153" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="153" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D153" s="2"/>
       <c r="G153" s="2"/>
     </row>
-    <row r="154" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="154" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D154" s="2"/>
       <c r="G154" s="2"/>
     </row>
-    <row r="155" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="155" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D155" s="2"/>
       <c r="G155" s="2"/>
     </row>
-    <row r="156" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="156" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D156" s="2"/>
       <c r="G156" s="2"/>
     </row>
-    <row r="157" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="157" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D157" s="2"/>
       <c r="G157" s="2"/>
     </row>
-    <row r="158" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="158" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D158" s="2"/>
       <c r="G158" s="2"/>
     </row>
-    <row r="159" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="159" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D159" s="2"/>
       <c r="G159" s="2"/>
     </row>
-    <row r="160" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="160" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D160" s="2"/>
       <c r="G160" s="2"/>
     </row>
-    <row r="161" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="161" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D161" s="2"/>
       <c r="G161" s="2"/>
     </row>
-    <row r="162" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="162" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D162" s="2"/>
       <c r="G162" s="2"/>
     </row>
-    <row r="163" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="163" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D163" s="2"/>
       <c r="G163" s="2"/>
     </row>
-    <row r="164" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="164" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D164" s="2"/>
       <c r="G164" s="2"/>
     </row>
-    <row r="165" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="165" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D165" s="2"/>
       <c r="G165" s="2"/>
     </row>
-    <row r="166" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="166" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D166" s="2"/>
       <c r="G166" s="2"/>
     </row>
-    <row r="167" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="167" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D167" s="2"/>
       <c r="G167" s="2"/>
     </row>
-    <row r="168" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="168" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D168" s="2"/>
       <c r="G168" s="2"/>
     </row>
-    <row r="169" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="169" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D169" s="2"/>
       <c r="G169" s="2"/>
     </row>
-    <row r="170" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="170" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D170" s="2"/>
       <c r="G170" s="2"/>
     </row>
-    <row r="171" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="171" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D171" s="2"/>
       <c r="G171" s="2"/>
     </row>
-    <row r="172" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="172" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D172" s="2"/>
       <c r="G172" s="2"/>
     </row>
-    <row r="173" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="173" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D173" s="2"/>
       <c r="G173" s="2"/>
     </row>
-    <row r="174" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="174" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D174" s="2"/>
       <c r="G174" s="2"/>
     </row>
-    <row r="175" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="175" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D175" s="2"/>
       <c r="G175" s="2"/>
     </row>
-    <row r="176" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="176" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D176" s="2"/>
       <c r="G176" s="2"/>
     </row>
-    <row r="177" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="177" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D177" s="2"/>
       <c r="G177" s="2"/>
     </row>
-    <row r="178" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="178" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D178" s="2"/>
       <c r="G178" s="2"/>
     </row>
-    <row r="179" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="179" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D179" s="2"/>
       <c r="G179" s="2"/>
     </row>
-    <row r="180" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="180" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D180" s="2"/>
       <c r="G180" s="2"/>
     </row>
-    <row r="181" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="181" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D181" s="2"/>
       <c r="G181" s="2"/>
     </row>
-    <row r="182" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="182" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D182" s="2"/>
       <c r="G182" s="2"/>
     </row>
-    <row r="183" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="183" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D183" s="2"/>
       <c r="G183" s="2"/>
     </row>
-    <row r="184" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="184" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D184" s="2"/>
       <c r="G184" s="2"/>
     </row>
-    <row r="185" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="185" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D185" s="2"/>
       <c r="G185" s="2"/>
     </row>
-    <row r="186" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="186" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D186" s="2"/>
       <c r="G186" s="2"/>
     </row>
-    <row r="187" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="187" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D187" s="2"/>
       <c r="G187" s="2"/>
     </row>
-    <row r="188" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="188" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D188" s="2"/>
       <c r="G188" s="2"/>
     </row>
-    <row r="189" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="189" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D189" s="2"/>
       <c r="G189" s="2"/>
     </row>
-    <row r="190" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="190" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D190" s="2"/>
       <c r="G190" s="2"/>
     </row>
-    <row r="191" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="191" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D191" s="2"/>
       <c r="G191" s="2"/>
     </row>
-    <row r="192" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="192" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D192" s="2"/>
       <c r="G192" s="2"/>
     </row>
-    <row r="193" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="193" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D193" s="2"/>
       <c r="G193" s="2"/>
     </row>
-    <row r="194" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="194" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D194" s="2"/>
       <c r="G194" s="2"/>
     </row>
-    <row r="195" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="195" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D195" s="2"/>
       <c r="G195" s="2"/>
     </row>
-    <row r="196" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="196" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D196" s="2"/>
       <c r="G196" s="2"/>
     </row>
-    <row r="197" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="197" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D197" s="2"/>
       <c r="G197" s="2"/>
     </row>
-    <row r="198" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="198" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D198" s="2"/>
       <c r="G198" s="2"/>
     </row>
-    <row r="199" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="199" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D199" s="2"/>
       <c r="G199" s="2"/>
     </row>
-    <row r="200" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="200" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D200" s="2"/>
       <c r="G200" s="2"/>
     </row>
-    <row r="201" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="201" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D201" s="2"/>
       <c r="G201" s="2"/>
     </row>
-    <row r="202" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="202" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D202" s="2"/>
       <c r="G202" s="2"/>
     </row>
-    <row r="203" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="203" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D203" s="2"/>
       <c r="G203" s="2"/>
     </row>
-    <row r="204" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="204" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D204" s="2"/>
       <c r="G204" s="2"/>
     </row>
-    <row r="205" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="205" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D205" s="2"/>
       <c r="G205" s="2"/>
     </row>
-    <row r="206" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="206" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D206" s="2"/>
       <c r="G206" s="2"/>
     </row>
-    <row r="207" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="207" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D207" s="2"/>
       <c r="G207" s="2"/>
     </row>
-    <row r="208" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="208" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D208" s="2"/>
       <c r="G208" s="2"/>
     </row>
-    <row r="209" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="209" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D209" s="2"/>
       <c r="G209" s="2"/>
     </row>
-    <row r="210" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="210" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D210" s="2"/>
       <c r="G210" s="2"/>
     </row>
-    <row r="211" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="211" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D211" s="2"/>
       <c r="G211" s="2"/>
     </row>
-    <row r="212" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="212" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D212" s="2"/>
       <c r="G212" s="2"/>
     </row>
-    <row r="213" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="213" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D213" s="2"/>
       <c r="G213" s="2"/>
     </row>
-    <row r="214" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="214" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D214" s="2"/>
       <c r="G214" s="2"/>
     </row>
-    <row r="215" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="215" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D215" s="2"/>
       <c r="G215" s="2"/>
     </row>
-    <row r="216" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="216" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D216" s="2"/>
       <c r="G216" s="2"/>
     </row>
-    <row r="217" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="217" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D217" s="2"/>
       <c r="G217" s="2"/>
     </row>
-    <row r="218" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="218" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D218" s="2"/>
       <c r="G218" s="2"/>
     </row>
-    <row r="219" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="219" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D219" s="2"/>
       <c r="G219" s="2"/>
     </row>
-    <row r="220" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="220" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D220" s="2"/>
       <c r="G220" s="2"/>
     </row>
-    <row r="221" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="221" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D221" s="2"/>
       <c r="G221" s="2"/>
     </row>
-    <row r="222" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="222" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D222" s="2"/>
       <c r="G222" s="2"/>
     </row>
-    <row r="223" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="223" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D223" s="2"/>
       <c r="G223" s="2"/>
     </row>
-    <row r="224" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="224" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D224" s="2"/>
       <c r="G224" s="2"/>
     </row>
-    <row r="225" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="225" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D225" s="2"/>
       <c r="G225" s="2"/>
     </row>
-    <row r="226" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="226" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D226" s="2"/>
       <c r="G226" s="2"/>
     </row>
-    <row r="227" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="227" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D227" s="2"/>
       <c r="G227" s="2"/>
     </row>
-    <row r="228" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="228" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D228" s="2"/>
       <c r="G228" s="2"/>
     </row>
-    <row r="229" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="229" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D229" s="2"/>
       <c r="G229" s="2"/>
     </row>
-    <row r="230" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="230" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D230" s="2"/>
       <c r="G230" s="2"/>
     </row>
-    <row r="231" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="231" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D231" s="2"/>
       <c r="G231" s="2"/>
     </row>
-    <row r="232" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="232" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D232" s="2"/>
       <c r="G232" s="2"/>
     </row>
-    <row r="233" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="233" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D233" s="2"/>
       <c r="G233" s="2"/>
     </row>
-    <row r="234" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="234" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D234" s="2"/>
       <c r="G234" s="2"/>
     </row>
-    <row r="235" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="235" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D235" s="2"/>
       <c r="G235" s="2"/>
     </row>
-    <row r="236" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="236" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D236" s="2"/>
       <c r="G236" s="2"/>
     </row>
-    <row r="237" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="237" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D237" s="2"/>
       <c r="G237" s="2"/>
     </row>
-    <row r="238" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="238" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D238" s="2"/>
       <c r="G238" s="2"/>
     </row>
-    <row r="239" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="239" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D239" s="2"/>
       <c r="G239" s="2"/>
     </row>
-    <row r="240" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="240" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D240" s="2"/>
       <c r="G240" s="2"/>
     </row>
-    <row r="241" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="241" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D241" s="2"/>
       <c r="G241" s="2"/>
     </row>
-    <row r="242" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="242" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D242" s="2"/>
       <c r="G242" s="2"/>
     </row>
-    <row r="243" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="243" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D243" s="2"/>
       <c r="G243" s="2"/>
     </row>
-    <row r="244" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="244" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D244" s="2"/>
       <c r="G244" s="2"/>
     </row>
-    <row r="245" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="245" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D245" s="2"/>
       <c r="G245" s="2"/>
     </row>
-    <row r="246" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="246" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D246" s="2"/>
       <c r="G246" s="2"/>
     </row>
-    <row r="247" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="247" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D247" s="2"/>
       <c r="G247" s="2"/>
     </row>
-    <row r="248" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="248" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D248" s="2"/>
       <c r="G248" s="2"/>
     </row>
-    <row r="249" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="249" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D249" s="2"/>
       <c r="G249" s="2"/>
     </row>
-    <row r="250" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="250" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D250" s="2"/>
       <c r="G250" s="2"/>
     </row>
-    <row r="251" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="251" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D251" s="2"/>
       <c r="G251" s="2"/>
     </row>
-    <row r="252" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="252" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D252" s="2"/>
       <c r="G252" s="2"/>
     </row>
-    <row r="253" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="253" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D253" s="2"/>
       <c r="G253" s="2"/>
     </row>
-    <row r="254" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="254" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D254" s="2"/>
       <c r="G254" s="2"/>
     </row>
-    <row r="255" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="255" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D255" s="2"/>
       <c r="G255" s="2"/>
     </row>
-    <row r="256" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="256" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D256" s="2"/>
       <c r="G256" s="2"/>
     </row>
-    <row r="257" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="257" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D257" s="2"/>
       <c r="G257" s="2"/>
     </row>
-    <row r="258" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="258" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D258" s="2"/>
       <c r="G258" s="2"/>
     </row>
-    <row r="259" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="259" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D259" s="2"/>
       <c r="G259" s="2"/>
     </row>
-    <row r="260" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="260" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D260" s="2"/>
       <c r="G260" s="2"/>
     </row>
-    <row r="261" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="261" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D261" s="2"/>
       <c r="G261" s="2"/>
     </row>
-    <row r="262" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="262" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D262" s="2"/>
       <c r="G262" s="2"/>
     </row>
-    <row r="263" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="263" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D263" s="2"/>
       <c r="G263" s="2"/>
     </row>
-    <row r="264" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="264" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D264" s="2"/>
       <c r="G264" s="2"/>
     </row>
-    <row r="265" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="265" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D265" s="2"/>
       <c r="G265" s="2"/>
     </row>
-    <row r="266" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="266" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D266" s="2"/>
       <c r="G266" s="2"/>
     </row>
-    <row r="267" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="267" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D267" s="2"/>
       <c r="G267" s="2"/>
     </row>
-    <row r="268" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="268" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D268" s="2"/>
       <c r="G268" s="2"/>
     </row>
-    <row r="269" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="269" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D269" s="2"/>
       <c r="G269" s="2"/>
     </row>
-    <row r="270" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="270" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D270" s="2"/>
       <c r="G270" s="2"/>
     </row>
-    <row r="271" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="271" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D271" s="2"/>
       <c r="G271" s="2"/>
     </row>
-    <row r="272" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="272" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D272" s="2"/>
       <c r="G272" s="2"/>
     </row>
-    <row r="273" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="273" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D273" s="2"/>
       <c r="G273" s="2"/>
     </row>
-    <row r="274" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="274" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D274" s="2"/>
       <c r="G274" s="2"/>
     </row>
-    <row r="275" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="275" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D275" s="2"/>
       <c r="G275" s="2"/>
     </row>
-    <row r="276" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="276" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D276" s="2"/>
       <c r="G276" s="2"/>
     </row>
-    <row r="277" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="277" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D277" s="2"/>
       <c r="G277" s="2"/>
     </row>
-    <row r="278" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="278" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D278" s="2"/>
       <c r="G278" s="2"/>
     </row>
-    <row r="279" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="279" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D279" s="2"/>
       <c r="G279" s="2"/>
     </row>
-    <row r="280" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="280" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D280" s="2"/>
       <c r="G280" s="2"/>
     </row>
-    <row r="281" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="281" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D281" s="2"/>
       <c r="G281" s="2"/>
     </row>
-    <row r="282" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="282" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D282" s="2"/>
       <c r="G282" s="2"/>
     </row>
-    <row r="283" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="283" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D283" s="2"/>
       <c r="G283" s="2"/>
     </row>
-    <row r="284" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="284" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D284" s="2"/>
       <c r="G284" s="2"/>
     </row>
-    <row r="285" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="285" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D285" s="2"/>
       <c r="G285" s="2"/>
     </row>
-    <row r="286" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="286" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D286" s="2"/>
       <c r="G286" s="2"/>
     </row>
-    <row r="287" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="287" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D287" s="2"/>
       <c r="G287" s="2"/>
     </row>
-    <row r="288" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="288" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D288" s="2"/>
       <c r="G288" s="2"/>
     </row>
-    <row r="289" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="289" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D289" s="2"/>
       <c r="G289" s="2"/>
     </row>
-    <row r="290" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="290" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D290" s="2"/>
       <c r="G290" s="2"/>
     </row>
-    <row r="291" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="291" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D291" s="2"/>
       <c r="G291" s="2"/>
     </row>
-    <row r="292" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="292" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D292" s="2"/>
       <c r="G292" s="2"/>
     </row>
-    <row r="293" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="293" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D293" s="2"/>
       <c r="G293" s="2"/>
     </row>
-    <row r="294" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="294" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D294" s="2"/>
       <c r="G294" s="2"/>
     </row>
-    <row r="295" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="295" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D295" s="2"/>
       <c r="G295" s="2"/>
     </row>
-    <row r="296" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="296" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D296" s="2"/>
       <c r="G296" s="2"/>
     </row>
-    <row r="297" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="297" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D297" s="2"/>
       <c r="G297" s="2"/>
     </row>
-    <row r="298" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="298" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D298" s="2"/>
       <c r="G298" s="2"/>
     </row>
-    <row r="299" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="299" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D299" s="2"/>
       <c r="G299" s="2"/>
     </row>
-    <row r="300" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="300" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D300" s="2"/>
       <c r="G300" s="2"/>
     </row>
-    <row r="301" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="301" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D301" s="2"/>
       <c r="G301" s="2"/>
     </row>
-    <row r="302" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="302" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D302" s="2"/>
       <c r="G302" s="2"/>
     </row>
-    <row r="303" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="303" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D303" s="2"/>
       <c r="G303" s="2"/>
     </row>
-    <row r="304" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="304" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D304" s="2"/>
       <c r="G304" s="2"/>
     </row>
-    <row r="305" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="305" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D305" s="2"/>
       <c r="G305" s="2"/>
     </row>
-    <row r="306" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="306" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D306" s="2"/>
       <c r="G306" s="2"/>
     </row>
-    <row r="307" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="307" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D307" s="2"/>
       <c r="G307" s="2"/>
     </row>
-    <row r="308" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="308" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D308" s="2"/>
       <c r="G308" s="2"/>
     </row>
-    <row r="309" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="309" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D309" s="2"/>
       <c r="G309" s="2"/>
     </row>
-    <row r="310" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="310" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D310" s="2"/>
       <c r="G310" s="2"/>
     </row>
-    <row r="311" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="311" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D311" s="2"/>
       <c r="G311" s="2"/>
     </row>
-    <row r="312" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="312" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D312" s="2"/>
       <c r="G312" s="2"/>
     </row>
-    <row r="313" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="313" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D313" s="2"/>
       <c r="G313" s="2"/>
     </row>
-    <row r="314" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="314" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D314" s="2"/>
       <c r="G314" s="2"/>
     </row>
-    <row r="315" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="315" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D315" s="2"/>
       <c r="G315" s="2"/>
     </row>
-    <row r="316" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="316" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D316" s="2"/>
       <c r="G316" s="2"/>
     </row>
-    <row r="317" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="317" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D317" s="2"/>
       <c r="G317" s="2"/>
     </row>
-    <row r="318" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="318" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D318" s="2"/>
       <c r="G318" s="2"/>
     </row>
-    <row r="319" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="319" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D319" s="2"/>
       <c r="G319" s="2"/>
     </row>
-    <row r="320" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="320" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D320" s="2"/>
       <c r="G320" s="2"/>
     </row>
-    <row r="321" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="321" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D321" s="2"/>
       <c r="G321" s="2"/>
     </row>
-    <row r="322" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="322" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D322" s="2"/>
       <c r="G322" s="2"/>
     </row>
-    <row r="323" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="323" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D323" s="2"/>
       <c r="G323" s="2"/>
     </row>
-    <row r="324" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="324" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D324" s="2"/>
       <c r="G324" s="2"/>
     </row>
-    <row r="325" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="325" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D325" s="2"/>
       <c r="G325" s="2"/>
     </row>
-    <row r="326" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="326" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D326" s="2"/>
       <c r="G326" s="2"/>
     </row>
-    <row r="327" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="327" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D327" s="2"/>
       <c r="G327" s="2"/>
     </row>
-    <row r="328" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="328" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D328" s="2"/>
       <c r="G328" s="2"/>
     </row>
-    <row r="329" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="329" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D329" s="2"/>
       <c r="G329" s="2"/>
     </row>
-    <row r="330" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="330" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D330" s="2"/>
       <c r="G330" s="2"/>
     </row>
-    <row r="331" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="331" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D331" s="2"/>
       <c r="G331" s="2"/>
     </row>
-    <row r="332" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="332" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D332" s="2"/>
       <c r="G332" s="2"/>
     </row>
-    <row r="333" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="333" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D333" s="2"/>
       <c r="G333" s="2"/>
     </row>
-    <row r="334" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="334" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D334" s="2"/>
       <c r="G334" s="2"/>
     </row>
-    <row r="335" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="335" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D335" s="2"/>
       <c r="G335" s="2"/>
     </row>
-    <row r="336" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="336" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D336" s="2"/>
       <c r="G336" s="2"/>
     </row>
-    <row r="337" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="337" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D337" s="2"/>
       <c r="G337" s="2"/>
     </row>
-    <row r="338" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="338" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D338" s="2"/>
       <c r="G338" s="2"/>
     </row>
-    <row r="339" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="339" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D339" s="2"/>
       <c r="G339" s="2"/>
     </row>
-    <row r="340" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="340" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D340" s="2"/>
       <c r="G340" s="2"/>
     </row>
-    <row r="341" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="341" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D341" s="2"/>
       <c r="G341" s="2"/>
     </row>
-    <row r="342" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="342" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D342" s="2"/>
       <c r="G342" s="2"/>
     </row>
-    <row r="343" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="343" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D343" s="2"/>
       <c r="G343" s="2"/>
     </row>
-    <row r="344" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="344" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D344" s="2"/>
       <c r="G344" s="2"/>
     </row>
-    <row r="345" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="345" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D345" s="2"/>
       <c r="G345" s="2"/>
     </row>
-    <row r="346" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="346" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D346" s="2"/>
       <c r="G346" s="2"/>
     </row>
-    <row r="347" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="347" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D347" s="2"/>
       <c r="G347" s="2"/>
     </row>
-    <row r="348" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="348" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D348" s="2"/>
       <c r="G348" s="2"/>
     </row>
-    <row r="349" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="349" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D349" s="2"/>
       <c r="G349" s="2"/>
     </row>
-    <row r="350" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="350" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D350" s="2"/>
       <c r="G350" s="2"/>
     </row>
-    <row r="351" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="351" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D351" s="2"/>
       <c r="G351" s="2"/>
     </row>
-    <row r="352" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="352" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D352" s="2"/>
       <c r="G352" s="2"/>
     </row>
-    <row r="353" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="353" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D353" s="2"/>
       <c r="G353" s="2"/>
     </row>
-    <row r="354" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="354" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D354" s="2"/>
       <c r="G354" s="2"/>
     </row>
-    <row r="355" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="355" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D355" s="2"/>
       <c r="G355" s="2"/>
     </row>
-    <row r="356" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="356" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D356" s="2"/>
       <c r="G356" s="2"/>
     </row>
-    <row r="357" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="357" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D357" s="2"/>
       <c r="G357" s="2"/>
     </row>
-    <row r="358" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="358" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D358" s="2"/>
       <c r="G358" s="2"/>
     </row>
-    <row r="359" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="359" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D359" s="2"/>
       <c r="G359" s="2"/>
     </row>
-    <row r="360" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="360" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D360" s="2"/>
       <c r="G360" s="2"/>
     </row>
-    <row r="361" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="361" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D361" s="2"/>
       <c r="G361" s="2"/>
     </row>
-    <row r="362" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="362" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D362" s="2"/>
       <c r="G362" s="2"/>
     </row>
-    <row r="363" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="363" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D363" s="2"/>
       <c r="G363" s="2"/>
     </row>
-    <row r="364" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="364" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D364" s="2"/>
       <c r="G364" s="2"/>
     </row>
-    <row r="365" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="365" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D365" s="2"/>
       <c r="G365" s="2"/>
     </row>
-    <row r="366" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="366" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D366" s="2"/>
       <c r="G366" s="2"/>
     </row>
-    <row r="367" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="367" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D367" s="2"/>
       <c r="G367" s="2"/>
     </row>
-    <row r="368" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="368" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D368" s="2"/>
       <c r="G368" s="2"/>
     </row>
-    <row r="369" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="369" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D369" s="2"/>
       <c r="G369" s="2"/>
     </row>
-    <row r="370" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="370" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D370" s="2"/>
       <c r="G370" s="2"/>
     </row>
-    <row r="371" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="371" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D371" s="2"/>
       <c r="G371" s="2"/>
     </row>
-    <row r="372" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="372" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D372" s="2"/>
       <c r="G372" s="2"/>
     </row>
-    <row r="373" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="373" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D373" s="2"/>
       <c r="G373" s="2"/>
     </row>
-    <row r="374" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="374" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D374" s="2"/>
       <c r="G374" s="2"/>
     </row>
-    <row r="375" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="375" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D375" s="2"/>
       <c r="G375" s="2"/>
     </row>
-    <row r="376" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="376" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D376" s="2"/>
       <c r="G376" s="2"/>
     </row>
-    <row r="377" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="377" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D377" s="2"/>
       <c r="G377" s="2"/>
     </row>
-    <row r="378" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="378" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D378" s="2"/>
       <c r="G378" s="2"/>
     </row>
-    <row r="379" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="379" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D379" s="2"/>
       <c r="G379" s="2"/>
     </row>
-    <row r="380" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="380" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D380" s="2"/>
       <c r="G380" s="2"/>
     </row>
-    <row r="381" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="381" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D381" s="2"/>
       <c r="G381" s="2"/>
     </row>
-    <row r="382" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="382" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D382" s="2"/>
       <c r="G382" s="2"/>
     </row>
-    <row r="383" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="383" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D383" s="2"/>
       <c r="G383" s="2"/>
     </row>
-    <row r="384" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="384" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D384" s="2"/>
       <c r="G384" s="2"/>
     </row>
-    <row r="385" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="385" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D385" s="2"/>
       <c r="G385" s="2"/>
     </row>
-    <row r="386" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="386" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D386" s="2"/>
       <c r="G386" s="2"/>
     </row>
-    <row r="387" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="387" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D387" s="2"/>
       <c r="G387" s="2"/>
     </row>
-    <row r="388" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="388" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D388" s="2"/>
       <c r="G388" s="2"/>
     </row>
-    <row r="389" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="389" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D389" s="2"/>
       <c r="G389" s="2"/>
     </row>
-    <row r="390" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="390" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D390" s="2"/>
       <c r="G390" s="2"/>
     </row>
-    <row r="391" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="391" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D391" s="2"/>
       <c r="G391" s="2"/>
     </row>
-    <row r="392" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="392" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D392" s="2"/>
       <c r="G392" s="2"/>
     </row>
-    <row r="393" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="393" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D393" s="2"/>
       <c r="G393" s="2"/>
     </row>
-    <row r="394" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="394" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D394" s="2"/>
       <c r="G394" s="2"/>
     </row>
-    <row r="395" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="395" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D395" s="2"/>
       <c r="G395" s="2"/>
     </row>
-    <row r="396" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="396" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D396" s="2"/>
       <c r="G396" s="2"/>
     </row>
-    <row r="397" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="397" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D397" s="2"/>
       <c r="G397" s="2"/>
     </row>
-    <row r="398" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="398" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D398" s="2"/>
       <c r="G398" s="2"/>
     </row>
-    <row r="399" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="399" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D399" s="2"/>
       <c r="G399" s="2"/>
     </row>
-    <row r="400" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="400" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D400" s="2"/>
       <c r="G400" s="2"/>
     </row>
-    <row r="401" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="401" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D401" s="2"/>
       <c r="G401" s="2"/>
     </row>
-    <row r="402" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="402" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D402" s="2"/>
       <c r="G402" s="2"/>
     </row>
-    <row r="403" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="403" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D403" s="2"/>
       <c r="G403" s="2"/>
     </row>
-    <row r="404" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="404" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D404" s="2"/>
       <c r="G404" s="2"/>
     </row>
-    <row r="405" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="405" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D405" s="2"/>
       <c r="G405" s="2"/>
     </row>
-    <row r="406" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="406" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D406" s="2"/>
       <c r="G406" s="2"/>
     </row>
-    <row r="407" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="407" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D407" s="2"/>
       <c r="G407" s="2"/>
     </row>
-    <row r="408" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="408" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D408" s="2"/>
       <c r="G408" s="2"/>
     </row>
-    <row r="409" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="409" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D409" s="2"/>
       <c r="G409" s="2"/>
     </row>
-    <row r="410" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="410" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D410" s="2"/>
       <c r="G410" s="2"/>
     </row>
-    <row r="411" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="411" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D411" s="2"/>
       <c r="G411" s="2"/>
     </row>
-    <row r="412" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="412" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D412" s="2"/>
       <c r="G412" s="2"/>
     </row>
-    <row r="413" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="413" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D413" s="2"/>
       <c r="G413" s="2"/>
     </row>
-    <row r="414" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="414" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D414" s="2"/>
       <c r="G414" s="2"/>
     </row>
-    <row r="415" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="415" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D415" s="2"/>
       <c r="G415" s="2"/>
     </row>
-    <row r="416" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="416" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D416" s="2"/>
       <c r="G416" s="2"/>
     </row>
-    <row r="417" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="417" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D417" s="2"/>
       <c r="G417" s="2"/>
     </row>
-    <row r="418" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="418" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D418" s="2"/>
       <c r="G418" s="2"/>
     </row>
-    <row r="419" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="419" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D419" s="2"/>
       <c r="G419" s="2"/>
     </row>
-    <row r="420" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="420" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D420" s="2"/>
       <c r="G420" s="2"/>
     </row>
-    <row r="421" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="421" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D421" s="2"/>
       <c r="G421" s="2"/>
     </row>
-    <row r="422" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="422" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D422" s="2"/>
       <c r="G422" s="2"/>
     </row>
-    <row r="423" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="423" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D423" s="2"/>
       <c r="G423" s="2"/>
     </row>
-    <row r="424" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="424" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D424" s="2"/>
       <c r="G424" s="2"/>
     </row>
-    <row r="425" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="425" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D425" s="2"/>
       <c r="G425" s="2"/>
     </row>
-    <row r="426" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="426" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D426" s="2"/>
       <c r="G426" s="2"/>
     </row>
-    <row r="427" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="427" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D427" s="2"/>
       <c r="G427" s="2"/>
     </row>
-    <row r="428" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="428" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D428" s="2"/>
       <c r="G428" s="2"/>
     </row>
-    <row r="429" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="429" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D429" s="2"/>
       <c r="G429" s="2"/>
     </row>
-    <row r="430" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="430" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D430" s="2"/>
       <c r="G430" s="2"/>
     </row>
-    <row r="431" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="431" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D431" s="2"/>
       <c r="G431" s="2"/>
     </row>
-    <row r="432" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="432" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D432" s="2"/>
       <c r="G432" s="2"/>
     </row>
-    <row r="433" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="433" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D433" s="2"/>
       <c r="G433" s="2"/>
     </row>
-    <row r="434" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="434" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D434" s="2"/>
       <c r="G434" s="2"/>
     </row>
-    <row r="435" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="435" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D435" s="2"/>
       <c r="G435" s="2"/>
     </row>
-    <row r="436" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="436" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D436" s="2"/>
       <c r="G436" s="2"/>
     </row>
-    <row r="437" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="437" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D437" s="2"/>
       <c r="G437" s="2"/>
     </row>
-    <row r="438" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="438" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D438" s="2"/>
       <c r="G438" s="2"/>
     </row>
-    <row r="439" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="439" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D439" s="2"/>
       <c r="G439" s="2"/>
     </row>
-    <row r="440" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="440" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D440" s="2"/>
       <c r="G440" s="2"/>
     </row>
-    <row r="441" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="441" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D441" s="2"/>
       <c r="G441" s="2"/>
     </row>
-    <row r="442" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="442" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D442" s="2"/>
       <c r="G442" s="2"/>
     </row>
-    <row r="443" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="443" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D443" s="2"/>
       <c r="G443" s="2"/>
     </row>
-    <row r="444" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="444" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D444" s="2"/>
       <c r="G444" s="2"/>
     </row>
-    <row r="445" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="445" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D445" s="2"/>
       <c r="G445" s="2"/>
     </row>
-    <row r="446" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="446" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D446" s="2"/>
       <c r="G446" s="2"/>
     </row>
-    <row r="447" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="447" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D447" s="2"/>
       <c r="G447" s="2"/>
     </row>
-    <row r="448" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="448" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D448" s="2"/>
       <c r="G448" s="2"/>
     </row>
-    <row r="449" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="449" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D449" s="2"/>
       <c r="G449" s="2"/>
     </row>
-    <row r="450" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="450" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D450" s="2"/>
       <c r="G450" s="2"/>
     </row>
-    <row r="451" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="451" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D451" s="2"/>
       <c r="G451" s="2"/>
     </row>
-    <row r="452" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="452" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D452" s="2"/>
       <c r="G452" s="2"/>
     </row>
-    <row r="453" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="453" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D453" s="2"/>
       <c r="G453" s="2"/>
     </row>
-    <row r="454" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="454" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D454" s="2"/>
       <c r="G454" s="2"/>
     </row>
-    <row r="455" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="455" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D455" s="2"/>
       <c r="G455" s="2"/>
     </row>
-    <row r="456" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="456" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D456" s="2"/>
       <c r="G456" s="2"/>
     </row>
-    <row r="457" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="457" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D457" s="2"/>
       <c r="G457" s="2"/>
     </row>
-    <row r="458" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="458" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D458" s="2"/>
       <c r="G458" s="2"/>
     </row>
-    <row r="459" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="459" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D459" s="2"/>
       <c r="G459" s="2"/>
     </row>
-    <row r="460" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="460" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D460" s="2"/>
       <c r="G460" s="2"/>
     </row>
-    <row r="461" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="461" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D461" s="2"/>
       <c r="G461" s="2"/>
     </row>
-    <row r="462" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="462" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D462" s="2"/>
       <c r="G462" s="2"/>
     </row>
-    <row r="463" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="463" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D463" s="2"/>
       <c r="G463" s="2"/>
     </row>
-    <row r="464" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="464" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D464" s="2"/>
       <c r="G464" s="2"/>
     </row>
-    <row r="465" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="465" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D465" s="2"/>
       <c r="G465" s="2"/>
     </row>
-    <row r="466" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="466" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D466" s="2"/>
       <c r="G466" s="2"/>
     </row>
-    <row r="467" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="467" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D467" s="2"/>
       <c r="G467" s="2"/>
     </row>
-    <row r="468" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="468" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D468" s="2"/>
       <c r="G468" s="2"/>
     </row>
-    <row r="469" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="469" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D469" s="2"/>
       <c r="G469" s="2"/>
     </row>
-    <row r="470" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="470" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D470" s="2"/>
       <c r="G470" s="2"/>
     </row>
-    <row r="471" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="471" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D471" s="2"/>
       <c r="G471" s="2"/>
     </row>
-    <row r="472" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="472" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D472" s="2"/>
       <c r="G472" s="2"/>
     </row>
-    <row r="473" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="473" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D473" s="2"/>
       <c r="G473" s="2"/>
     </row>
-    <row r="474" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="474" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D474" s="2"/>
       <c r="G474" s="2"/>
     </row>
-    <row r="475" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="475" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D475" s="2"/>
       <c r="G475" s="2"/>
     </row>
-    <row r="476" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="476" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D476" s="2"/>
       <c r="G476" s="2"/>
     </row>
-    <row r="477" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="477" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D477" s="2"/>
       <c r="G477" s="2"/>
     </row>
-    <row r="478" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="478" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D478" s="2"/>
       <c r="G478" s="2"/>
     </row>
-    <row r="479" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="479" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D479" s="2"/>
       <c r="G479" s="2"/>
     </row>
-    <row r="480" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="480" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D480" s="2"/>
       <c r="G480" s="2"/>
     </row>
-    <row r="481" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="481" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D481" s="2"/>
       <c r="G481" s="2"/>
     </row>
-    <row r="482" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="482" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D482" s="2"/>
       <c r="G482" s="2"/>
     </row>
-    <row r="483" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="483" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D483" s="2"/>
       <c r="G483" s="2"/>
     </row>
-    <row r="484" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="484" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D484" s="2"/>
       <c r="G484" s="2"/>
     </row>
-    <row r="485" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="485" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D485" s="2"/>
       <c r="G485" s="2"/>
     </row>
-    <row r="486" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="486" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D486" s="2"/>
       <c r="G486" s="2"/>
     </row>
-    <row r="487" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="487" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D487" s="2"/>
       <c r="G487" s="2"/>
     </row>
-    <row r="488" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="488" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D488" s="2"/>
       <c r="G488" s="2"/>
     </row>
-    <row r="489" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="489" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D489" s="2"/>
       <c r="G489" s="2"/>
     </row>
-    <row r="490" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="490" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D490" s="2"/>
       <c r="G490" s="2"/>
     </row>
-    <row r="491" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="491" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D491" s="2"/>
       <c r="G491" s="2"/>
     </row>
-    <row r="492" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="492" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D492" s="2"/>
       <c r="G492" s="2"/>
     </row>
-    <row r="493" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="493" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D493" s="2"/>
       <c r="G493" s="2"/>
     </row>
-    <row r="494" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="494" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D494" s="2"/>
       <c r="G494" s="2"/>
     </row>
-    <row r="495" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="495" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D495" s="2"/>
       <c r="G495" s="2"/>
     </row>
-    <row r="496" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="496" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D496" s="2"/>
       <c r="G496" s="2"/>
     </row>
-    <row r="497" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="497" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D497" s="2"/>
       <c r="G497" s="2"/>
     </row>
-    <row r="498" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="498" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D498" s="2"/>
       <c r="G498" s="2"/>
     </row>
-    <row r="499" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="499" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D499" s="2"/>
       <c r="G499" s="2"/>
     </row>
-    <row r="500" spans="3:7" x14ac:dyDescent="0.25">
+    <row r="500" spans="4:7" x14ac:dyDescent="0.25">
       <c r="D500" s="2"/>
       <c r="G500" s="2"/>
     </row>
@@ -2960,7 +3080,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -2975,10 +3095,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2986,7 +3106,7 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2994,7 +3114,7 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>86</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -3002,7 +3122,7 @@
         <v>41</v>
       </c>
       <c r="B4" t="s">
-        <v>71</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -3010,12 +3130,12 @@
         <v>60</v>
       </c>
       <c r="B5" t="s">
-        <v>72</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -3029,96 +3149,96 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>73</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>76</v>
+        <v>92</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>77</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>80</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>81</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>82</v>
+        <v>98</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>99</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>84</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>101</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>102</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>74</v>
+        <v>90</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>87</v>
+        <v>103</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>88</v>
+        <v>104</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Treatments: fill placeholder blurbs (20-30 words lorem ipsum)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/content/treatments.xlsx
+++ b/src/content/treatments.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="141">
   <si>
     <t>Title</t>
   </si>
@@ -45,36 +45,54 @@
     <t>FACIAL &amp; PEELING</t>
   </si>
   <si>
+    <t>Adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris.</t>
+  </si>
+  <si>
     <t>Lhala Peel</t>
   </si>
   <si>
     <t>lhala-peel</t>
   </si>
   <si>
+    <t>Do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure.</t>
+  </si>
+  <si>
     <t>Enzyme Peel</t>
   </si>
   <si>
     <t>enzyme-peel</t>
   </si>
   <si>
+    <t>Incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute.</t>
+  </si>
+  <si>
     <t>24K Gold Therapy</t>
   </si>
   <si>
     <t>gold-therapy</t>
   </si>
   <si>
+    <t>Et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis.</t>
+  </si>
+  <si>
     <t>Acne Care Facial</t>
   </si>
   <si>
     <t>acne-care-facial</t>
   </si>
   <si>
+    <t>Aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum.</t>
+  </si>
+  <si>
     <t>Lymphatic Facial</t>
   </si>
   <si>
     <t>lymphatic-facial</t>
   </si>
   <si>
+    <t>Ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse.</t>
+  </si>
+  <si>
     <t>Neurotoxin</t>
   </si>
   <si>
@@ -84,54 +102,81 @@
     <t>INJECTABLES &amp; REGENERATIVE</t>
   </si>
   <si>
+    <t>Quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit.</t>
+  </si>
+  <si>
     <t>Dermal Filler</t>
   </si>
   <si>
     <t>dermal-filler</t>
   </si>
   <si>
+    <t>Ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor.</t>
+  </si>
+  <si>
     <t>Sculptra® • Radiesse®</t>
   </si>
   <si>
     <t>sculptra-radiesse</t>
   </si>
   <si>
+    <t>Ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum.</t>
+  </si>
+  <si>
     <t>Thread Lift</t>
   </si>
   <si>
     <t>thread-lift</t>
   </si>
   <si>
+    <t>Ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem.</t>
+  </si>
+  <si>
     <t>Skin Booster</t>
   </si>
   <si>
     <t>skin-booster</t>
   </si>
   <si>
+    <t>Duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod.</t>
+  </si>
+  <si>
     <t>PRP (Platelet-Rich Plasma)</t>
   </si>
   <si>
     <t>prp</t>
   </si>
   <si>
+    <t>Dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do.</t>
+  </si>
+  <si>
     <t>Cell Factor</t>
   </si>
   <si>
     <t>cell-factor</t>
   </si>
   <si>
+    <t>In voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut.</t>
+  </si>
+  <si>
     <t>Regenerative Skin Therapy</t>
   </si>
   <si>
     <t>regenerative-skin-therapy</t>
   </si>
   <si>
+    <t>Esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua.</t>
+  </si>
+  <si>
     <t>Fat Dissolving Injection</t>
   </si>
   <si>
     <t>fat-dissolving-injection</t>
   </si>
   <si>
+    <t>Eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna.</t>
+  </si>
+  <si>
     <t>Ultherapy PRIME®</t>
   </si>
   <si>
@@ -141,54 +186,81 @@
     <t>LASER &amp; ENERGY</t>
   </si>
   <si>
+    <t>Pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco.</t>
+  </si>
+  <si>
     <t>Thermage FLX®</t>
   </si>
   <si>
     <t>thermage-flx</t>
   </si>
   <si>
+    <t>Dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation.</t>
+  </si>
+  <si>
     <t>InMode (MiniFX / BodyFX / Forma)</t>
   </si>
   <si>
     <t>inmode-minifx</t>
   </si>
   <si>
+    <t>Consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud.</t>
+  </si>
+  <si>
     <t>Onda Pro</t>
   </si>
   <si>
     <t>onda-pro</t>
   </si>
   <si>
+    <t>Sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat.</t>
+  </si>
+  <si>
     <t>Eve Titan</t>
   </si>
   <si>
     <t>eve-titan</t>
   </si>
   <si>
+    <t>Tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo.</t>
+  </si>
+  <si>
     <t>Potenza® RF Microneedling</t>
   </si>
   <si>
     <t>potenza-rf</t>
   </si>
   <si>
+    <t>Labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea.</t>
+  </si>
+  <si>
     <t>PicoSure® Pro</t>
   </si>
   <si>
     <t>picosure-pro</t>
   </si>
   <si>
+    <t>Magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate.</t>
+  </si>
+  <si>
     <t>XERF (Sérf)</t>
   </si>
   <si>
     <t>xerf</t>
   </si>
   <si>
+    <t>Enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in.</t>
+  </si>
+  <si>
     <t>Plasma</t>
   </si>
   <si>
     <t>plasma</t>
   </si>
   <si>
+    <t>Veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem.</t>
+  </si>
+  <si>
     <t>Medical Weight Management</t>
   </si>
   <si>
@@ -198,70 +270,106 @@
     <t>WELLNESS</t>
   </si>
   <si>
+    <t>Exercitation ullamco laboris nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur.</t>
+  </si>
+  <si>
     <t>IV Therapy</t>
   </si>
   <si>
     <t>iv-therapy</t>
   </si>
   <si>
+    <t>Nisi ut aliquip ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla.</t>
+  </si>
+  <si>
     <t>Hair Restoration</t>
   </si>
   <si>
     <t>hair-restoration</t>
   </si>
   <si>
+    <t>Ex ea commodo consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed.</t>
+  </si>
+  <si>
     <t>Joint PRP / PRF</t>
   </si>
   <si>
     <t>joint-prp</t>
   </si>
   <si>
+    <t>Consequat duis aute irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit.</t>
+  </si>
+  <si>
     <t>Co2</t>
   </si>
   <si>
     <t>co2</t>
   </si>
   <si>
+    <t>Irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing.</t>
+  </si>
+  <si>
     <t>Miim Laser</t>
   </si>
   <si>
     <t>miim-laser</t>
   </si>
   <si>
+    <t>Reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore.</t>
+  </si>
+  <si>
     <t>Agnes</t>
   </si>
   <si>
     <t>agnes</t>
   </si>
   <si>
+    <t>Velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et.</t>
+  </si>
+  <si>
     <t>Noblex</t>
   </si>
   <si>
     <t>noblex</t>
   </si>
   <si>
+    <t>Dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore.</t>
+  </si>
+  <si>
     <t>Scarlet</t>
   </si>
   <si>
     <t>scarlet</t>
   </si>
   <si>
+    <t>Nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis.</t>
+  </si>
+  <si>
     <t>Shrink</t>
   </si>
   <si>
     <t>shrink</t>
   </si>
   <si>
+    <t>Ipsum dolor sit amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam.</t>
+  </si>
+  <si>
     <t>V-Zet</t>
   </si>
   <si>
     <t>v-zet</t>
   </si>
   <si>
+    <t>Amet consectetur adipiscing elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex ea.</t>
+  </si>
+  <si>
     <t>PDO Threads</t>
   </si>
   <si>
     <t>pdo-threads</t>
+  </si>
+  <si>
+    <t>Elit sed do eiusmod tempor incididunt ut labore et dolore magna aliqua ut enim ad minim veniam quis nostrud exercitation ullamco laboris nisi ut aliquip ex.</t>
   </si>
   <si>
     <t>Name</t>
@@ -760,462 +868,534 @@
       <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2"/>
+      <c r="D2" s="2" t="s">
+        <v>10</v>
+      </c>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
       </c>
-      <c r="D3" s="2"/>
+      <c r="D3" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="G3" s="2"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="2"/>
+      <c r="D4" s="2" t="s">
+        <v>16</v>
+      </c>
       <c r="G4" s="2"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="2"/>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="G5" s="2"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="D6" s="2"/>
+      <c r="D6" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="G6" s="2"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B7" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
         <v>9</v>
       </c>
-      <c r="D7" s="2"/>
+      <c r="D7" s="2" t="s">
+        <v>25</v>
+      </c>
       <c r="G7" s="2"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c r="B8" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="C8" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="G8" s="2"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="C9" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="G9" s="2"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="C10" t="s">
-        <v>22</v>
-      </c>
-      <c r="D10" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="G10" s="2"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="B11" t="s">
+        <v>37</v>
+      </c>
+      <c r="C11" t="s">
         <v>28</v>
       </c>
-      <c r="C11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="2"/>
+      <c r="D11" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="G11" s="2"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="C12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="G12" s="2"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>31</v>
+        <v>42</v>
       </c>
       <c r="B13" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="G13" s="2"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>33</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C14" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="G14" s="2"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C15" t="s">
-        <v>22</v>
-      </c>
-      <c r="D15" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>37</v>
+        <v>51</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>52</v>
       </c>
       <c r="C16" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="G16" s="2"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>39</v>
+        <v>54</v>
       </c>
       <c r="B17" t="s">
-        <v>40</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
-        <v>41</v>
-      </c>
-      <c r="D17" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="G17" s="2"/>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="B18" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
-      </c>
-      <c r="D18" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="G18" s="2"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="B19" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="C19" t="s">
-        <v>41</v>
-      </c>
-      <c r="D19" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>63</v>
+      </c>
       <c r="G19" s="2"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>46</v>
+        <v>64</v>
       </c>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>65</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
-      </c>
-      <c r="D20" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>66</v>
+      </c>
       <c r="G20" s="2"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
-      </c>
-      <c r="D21" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>69</v>
+      </c>
       <c r="G21" s="2"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>51</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
-        <v>41</v>
-      </c>
-      <c r="D22" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>72</v>
+      </c>
       <c r="G22" s="2"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>52</v>
+        <v>73</v>
       </c>
       <c r="B23" t="s">
-        <v>53</v>
+        <v>74</v>
       </c>
       <c r="C23" t="s">
-        <v>41</v>
-      </c>
-      <c r="D23" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>75</v>
+      </c>
       <c r="G23" s="2"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>54</v>
+        <v>76</v>
       </c>
       <c r="B24" t="s">
-        <v>55</v>
+        <v>77</v>
       </c>
       <c r="C24" t="s">
-        <v>41</v>
-      </c>
-      <c r="D24" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="G24" s="2"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
         <v>56</v>
       </c>
-      <c r="B25" t="s">
-        <v>57</v>
-      </c>
-      <c r="C25" t="s">
-        <v>41</v>
-      </c>
-      <c r="D25" s="2"/>
+      <c r="D25" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="G25" s="2"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="B26" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>85</v>
+      </c>
       <c r="G26" s="2"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>61</v>
+        <v>86</v>
       </c>
       <c r="B27" t="s">
-        <v>62</v>
+        <v>87</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="G27" s="2"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="B28" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
-      </c>
-      <c r="D28" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>91</v>
+      </c>
       <c r="G28" s="2"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>65</v>
+        <v>92</v>
       </c>
       <c r="B29" t="s">
-        <v>66</v>
+        <v>93</v>
       </c>
       <c r="C29" t="s">
-        <v>60</v>
-      </c>
-      <c r="D29" s="2"/>
+        <v>84</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>94</v>
+      </c>
       <c r="G29" s="2"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>67</v>
+        <v>95</v>
       </c>
       <c r="B30" t="s">
-        <v>68</v>
+        <v>96</v>
       </c>
       <c r="C30" t="s">
-        <v>41</v>
-      </c>
-      <c r="D30" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="G30" s="2"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>69</v>
+        <v>98</v>
       </c>
       <c r="B31" t="s">
-        <v>70</v>
+        <v>99</v>
       </c>
       <c r="C31" t="s">
-        <v>41</v>
-      </c>
-      <c r="D31" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>100</v>
+      </c>
       <c r="G31" s="2"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>71</v>
+        <v>101</v>
       </c>
       <c r="B32" t="s">
-        <v>72</v>
+        <v>102</v>
       </c>
       <c r="C32" t="s">
-        <v>41</v>
-      </c>
-      <c r="D32" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>103</v>
+      </c>
       <c r="G32" s="2"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="B33" t="s">
-        <v>74</v>
+        <v>105</v>
       </c>
       <c r="C33" t="s">
-        <v>41</v>
-      </c>
-      <c r="D33" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>106</v>
+      </c>
       <c r="G33" s="2"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>107</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>108</v>
       </c>
       <c r="C34" t="s">
-        <v>41</v>
-      </c>
-      <c r="D34" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>109</v>
+      </c>
       <c r="G34" s="2"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="B35" t="s">
-        <v>78</v>
+        <v>111</v>
       </c>
       <c r="C35" t="s">
-        <v>41</v>
-      </c>
-      <c r="D35" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="G35" s="2"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>79</v>
+        <v>113</v>
       </c>
       <c r="B36" t="s">
-        <v>80</v>
+        <v>114</v>
       </c>
       <c r="C36" t="s">
-        <v>41</v>
-      </c>
-      <c r="D36" s="2"/>
+        <v>56</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>115</v>
+      </c>
       <c r="G36" s="2"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>81</v>
+        <v>116</v>
       </c>
       <c r="B37" t="s">
-        <v>82</v>
+        <v>117</v>
       </c>
       <c r="C37" t="s">
-        <v>22</v>
-      </c>
-      <c r="D37" s="2"/>
+        <v>28</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="G37" s="2"/>
     </row>
     <row r="38" spans="4:7" x14ac:dyDescent="0.25">
@@ -3095,10 +3275,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>83</v>
+        <v>119</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>84</v>
+        <v>120</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -3106,31 +3286,31 @@
         <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>85</v>
+        <v>121</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="B3" t="s">
-        <v>86</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>56</v>
       </c>
       <c r="B4" t="s">
-        <v>87</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="B5" t="s">
-        <v>88</v>
+        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -3149,92 +3329,92 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>89</v>
+        <v>125</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>128</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>93</v>
+        <v>129</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>94</v>
+        <v>130</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>95</v>
+        <v>131</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>96</v>
+        <v>132</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>98</v>
+        <v>134</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>135</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>136</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>101</v>
+        <v>137</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>138</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>104</v>
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Treatments: single before/after image, add What It Treats and Benefit
Columns are now matched by header name so they can be reordered.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/content/treatments.xlsx
+++ b/src/content/treatments.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="146">
   <si>
     <t>Title</t>
   </si>
@@ -27,10 +27,13 @@
     <t>Blurb (max 50 words)</t>
   </si>
   <si>
-    <t>Before Image</t>
-  </si>
-  <si>
-    <t>After Image</t>
+    <t>Before &amp; After Image</t>
+  </si>
+  <si>
+    <t>What It Treats</t>
+  </si>
+  <si>
+    <t>Benefit</t>
   </si>
   <si>
     <t>How It Works (Markdown)</t>
@@ -436,6 +439,18 @@
   </si>
   <si>
     <t>After saving, re-upload the file to src/content/treatments.xlsx and leave a note about what changed.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Before &amp; After Image (optional): ONE image file name showing before and after together, e.g. "hydrafacial-before-after.jpg". Files go in src/assets/images/treatments/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • What It Treats (optional): plain text. Line breaks are kept (one concern per line works well).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Benefit (optional): plain text. Line breaks are kept.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  • Optional sections are hidden on the page when left empty. Columns are matched by their header names, so you may reorder columns but do not rename the headers.</t>
   </si>
 </sst>
 </file>
@@ -824,18 +839,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G500"/>
+  <dimension ref="A1:H500"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="4" width="60" customWidth="1"/>
-    <col min="5" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="60" customWidth="1"/>
+    <col min="5" max="5" width="30" customWidth="1"/>
+    <col min="6" max="7" width="50" customWidth="1"/>
+    <col min="8" max="8" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -857,2398 +873,3399 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H1" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" t="s">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s">
         <v>10</v>
       </c>
-      <c r="G2" s="2"/>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
       <c r="D3" s="2" t="s">
-        <v>13</v>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="F3" s="2"/>
       <c r="G3" s="2"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>16</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>19</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="F5" s="2"/>
       <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B6" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>22</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>25</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="F7" s="2"/>
       <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
         <v>29</v>
       </c>
-      <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>30</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>28</v>
-      </c>
       <c r="D9" s="2" t="s">
-        <v>32</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H9" s="2"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>35</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="F10" s="2"/>
       <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B11" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C11" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>38</v>
-      </c>
+        <v>39</v>
+      </c>
+      <c r="F11" s="2"/>
       <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B12" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>41</v>
-      </c>
+        <v>42</v>
+      </c>
+      <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B13" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C13" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>44</v>
-      </c>
+        <v>45</v>
+      </c>
+      <c r="F13" s="2"/>
       <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B14" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C14" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>47</v>
-      </c>
+        <v>48</v>
+      </c>
+      <c r="F14" s="2"/>
       <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H14" s="2"/>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C15" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>50</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B16" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>53</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="F16" s="2"/>
       <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B17" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D17" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>59</v>
+      </c>
+      <c r="B18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C18" t="s">
         <v>57</v>
       </c>
-      <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>58</v>
-      </c>
-      <c r="B18" t="s">
-        <v>59</v>
-      </c>
-      <c r="C18" t="s">
-        <v>56</v>
-      </c>
       <c r="D18" s="2" t="s">
-        <v>60</v>
-      </c>
+        <v>61</v>
+      </c>
+      <c r="F18" s="2"/>
       <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B19" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C19" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>63</v>
-      </c>
+        <v>64</v>
+      </c>
+      <c r="F19" s="2"/>
       <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B20" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C20" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>67</v>
+      </c>
+      <c r="F20" s="2"/>
       <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H20" s="2"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B21" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C21" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>69</v>
-      </c>
+        <v>70</v>
+      </c>
+      <c r="F21" s="2"/>
       <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B22" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>72</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="F22" s="2"/>
       <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C23" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>75</v>
-      </c>
+        <v>76</v>
+      </c>
+      <c r="F23" s="2"/>
       <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B24" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C24" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>78</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="F24" s="2"/>
       <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H24" s="2"/>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C25" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>81</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="F25" s="2"/>
       <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H25" s="2"/>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B26" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C26" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D26" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F26" s="2"/>
+      <c r="G26" s="2"/>
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>87</v>
+      </c>
+      <c r="B27" t="s">
+        <v>88</v>
+      </c>
+      <c r="C27" t="s">
         <v>85</v>
       </c>
-      <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>86</v>
-      </c>
-      <c r="B27" t="s">
-        <v>87</v>
-      </c>
-      <c r="C27" t="s">
-        <v>84</v>
-      </c>
       <c r="D27" s="2" t="s">
-        <v>88</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="F27" s="2"/>
       <c r="G27" s="2"/>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C28" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>91</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="F28" s="2"/>
       <c r="G28" s="2"/>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C29" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>94</v>
-      </c>
+        <v>95</v>
+      </c>
+      <c r="F29" s="2"/>
       <c r="G29" s="2"/>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H29" s="2"/>
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B30" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>97</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="F30" s="2"/>
       <c r="G30" s="2"/>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B31" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C31" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>100</v>
-      </c>
+        <v>101</v>
+      </c>
+      <c r="F31" s="2"/>
       <c r="G31" s="2"/>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B32" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C32" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>103</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="F32" s="2"/>
       <c r="G32" s="2"/>
-    </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H32" s="2"/>
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B33" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C33" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>106</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="F33" s="2"/>
       <c r="G33" s="2"/>
-    </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B34" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C34" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>109</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="F34" s="2"/>
       <c r="G34" s="2"/>
-    </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H34" s="2"/>
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B35" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C35" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>112</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="F35" s="2"/>
       <c r="G35" s="2"/>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H35" s="2"/>
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B36" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C36" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>115</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="F36" s="2"/>
       <c r="G36" s="2"/>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H36" s="2"/>
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="B37" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C37" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>118</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="F37" s="2"/>
       <c r="G37" s="2"/>
-    </row>
-    <row r="38" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H37" s="2"/>
+    </row>
+    <row r="38" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D38" s="2"/>
+      <c r="F38" s="2"/>
       <c r="G38" s="2"/>
-    </row>
-    <row r="39" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H38" s="2"/>
+    </row>
+    <row r="39" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D39" s="2"/>
+      <c r="F39" s="2"/>
       <c r="G39" s="2"/>
-    </row>
-    <row r="40" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H39" s="2"/>
+    </row>
+    <row r="40" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D40" s="2"/>
+      <c r="F40" s="2"/>
       <c r="G40" s="2"/>
-    </row>
-    <row r="41" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D41" s="2"/>
+      <c r="F41" s="2"/>
       <c r="G41" s="2"/>
-    </row>
-    <row r="42" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D42" s="2"/>
+      <c r="F42" s="2"/>
       <c r="G42" s="2"/>
-    </row>
-    <row r="43" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H42" s="2"/>
+    </row>
+    <row r="43" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D43" s="2"/>
+      <c r="F43" s="2"/>
       <c r="G43" s="2"/>
-    </row>
-    <row r="44" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D44" s="2"/>
+      <c r="F44" s="2"/>
       <c r="G44" s="2"/>
-    </row>
-    <row r="45" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H44" s="2"/>
+    </row>
+    <row r="45" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D45" s="2"/>
+      <c r="F45" s="2"/>
       <c r="G45" s="2"/>
-    </row>
-    <row r="46" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H45" s="2"/>
+    </row>
+    <row r="46" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D46" s="2"/>
+      <c r="F46" s="2"/>
       <c r="G46" s="2"/>
-    </row>
-    <row r="47" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H46" s="2"/>
+    </row>
+    <row r="47" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D47" s="2"/>
+      <c r="F47" s="2"/>
       <c r="G47" s="2"/>
-    </row>
-    <row r="48" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H47" s="2"/>
+    </row>
+    <row r="48" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D48" s="2"/>
+      <c r="F48" s="2"/>
       <c r="G48" s="2"/>
-    </row>
-    <row r="49" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H48" s="2"/>
+    </row>
+    <row r="49" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D49" s="2"/>
+      <c r="F49" s="2"/>
       <c r="G49" s="2"/>
-    </row>
-    <row r="50" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H49" s="2"/>
+    </row>
+    <row r="50" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D50" s="2"/>
+      <c r="F50" s="2"/>
       <c r="G50" s="2"/>
-    </row>
-    <row r="51" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H50" s="2"/>
+    </row>
+    <row r="51" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D51" s="2"/>
+      <c r="F51" s="2"/>
       <c r="G51" s="2"/>
-    </row>
-    <row r="52" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H51" s="2"/>
+    </row>
+    <row r="52" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D52" s="2"/>
+      <c r="F52" s="2"/>
       <c r="G52" s="2"/>
-    </row>
-    <row r="53" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H52" s="2"/>
+    </row>
+    <row r="53" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D53" s="2"/>
+      <c r="F53" s="2"/>
       <c r="G53" s="2"/>
-    </row>
-    <row r="54" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H53" s="2"/>
+    </row>
+    <row r="54" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D54" s="2"/>
+      <c r="F54" s="2"/>
       <c r="G54" s="2"/>
-    </row>
-    <row r="55" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H54" s="2"/>
+    </row>
+    <row r="55" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D55" s="2"/>
+      <c r="F55" s="2"/>
       <c r="G55" s="2"/>
-    </row>
-    <row r="56" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H55" s="2"/>
+    </row>
+    <row r="56" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D56" s="2"/>
+      <c r="F56" s="2"/>
       <c r="G56" s="2"/>
-    </row>
-    <row r="57" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H56" s="2"/>
+    </row>
+    <row r="57" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D57" s="2"/>
+      <c r="F57" s="2"/>
       <c r="G57" s="2"/>
-    </row>
-    <row r="58" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D58" s="2"/>
+      <c r="F58" s="2"/>
       <c r="G58" s="2"/>
-    </row>
-    <row r="59" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H58" s="2"/>
+    </row>
+    <row r="59" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D59" s="2"/>
+      <c r="F59" s="2"/>
       <c r="G59" s="2"/>
-    </row>
-    <row r="60" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H59" s="2"/>
+    </row>
+    <row r="60" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D60" s="2"/>
+      <c r="F60" s="2"/>
       <c r="G60" s="2"/>
-    </row>
-    <row r="61" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H60" s="2"/>
+    </row>
+    <row r="61" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D61" s="2"/>
+      <c r="F61" s="2"/>
       <c r="G61" s="2"/>
-    </row>
-    <row r="62" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H61" s="2"/>
+    </row>
+    <row r="62" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D62" s="2"/>
+      <c r="F62" s="2"/>
       <c r="G62" s="2"/>
-    </row>
-    <row r="63" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H62" s="2"/>
+    </row>
+    <row r="63" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D63" s="2"/>
+      <c r="F63" s="2"/>
       <c r="G63" s="2"/>
-    </row>
-    <row r="64" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H63" s="2"/>
+    </row>
+    <row r="64" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D64" s="2"/>
+      <c r="F64" s="2"/>
       <c r="G64" s="2"/>
-    </row>
-    <row r="65" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H64" s="2"/>
+    </row>
+    <row r="65" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D65" s="2"/>
+      <c r="F65" s="2"/>
       <c r="G65" s="2"/>
-    </row>
-    <row r="66" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H65" s="2"/>
+    </row>
+    <row r="66" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D66" s="2"/>
+      <c r="F66" s="2"/>
       <c r="G66" s="2"/>
-    </row>
-    <row r="67" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H66" s="2"/>
+    </row>
+    <row r="67" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D67" s="2"/>
+      <c r="F67" s="2"/>
       <c r="G67" s="2"/>
-    </row>
-    <row r="68" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H67" s="2"/>
+    </row>
+    <row r="68" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D68" s="2"/>
+      <c r="F68" s="2"/>
       <c r="G68" s="2"/>
-    </row>
-    <row r="69" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H68" s="2"/>
+    </row>
+    <row r="69" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D69" s="2"/>
+      <c r="F69" s="2"/>
       <c r="G69" s="2"/>
-    </row>
-    <row r="70" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H69" s="2"/>
+    </row>
+    <row r="70" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D70" s="2"/>
+      <c r="F70" s="2"/>
       <c r="G70" s="2"/>
-    </row>
-    <row r="71" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H70" s="2"/>
+    </row>
+    <row r="71" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D71" s="2"/>
+      <c r="F71" s="2"/>
       <c r="G71" s="2"/>
-    </row>
-    <row r="72" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H71" s="2"/>
+    </row>
+    <row r="72" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D72" s="2"/>
+      <c r="F72" s="2"/>
       <c r="G72" s="2"/>
-    </row>
-    <row r="73" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H72" s="2"/>
+    </row>
+    <row r="73" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D73" s="2"/>
+      <c r="F73" s="2"/>
       <c r="G73" s="2"/>
-    </row>
-    <row r="74" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H73" s="2"/>
+    </row>
+    <row r="74" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D74" s="2"/>
+      <c r="F74" s="2"/>
       <c r="G74" s="2"/>
-    </row>
-    <row r="75" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H74" s="2"/>
+    </row>
+    <row r="75" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D75" s="2"/>
+      <c r="F75" s="2"/>
       <c r="G75" s="2"/>
-    </row>
-    <row r="76" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H75" s="2"/>
+    </row>
+    <row r="76" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D76" s="2"/>
+      <c r="F76" s="2"/>
       <c r="G76" s="2"/>
-    </row>
-    <row r="77" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H76" s="2"/>
+    </row>
+    <row r="77" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D77" s="2"/>
+      <c r="F77" s="2"/>
       <c r="G77" s="2"/>
-    </row>
-    <row r="78" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H77" s="2"/>
+    </row>
+    <row r="78" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D78" s="2"/>
+      <c r="F78" s="2"/>
       <c r="G78" s="2"/>
-    </row>
-    <row r="79" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H78" s="2"/>
+    </row>
+    <row r="79" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D79" s="2"/>
+      <c r="F79" s="2"/>
       <c r="G79" s="2"/>
-    </row>
-    <row r="80" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H79" s="2"/>
+    </row>
+    <row r="80" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D80" s="2"/>
+      <c r="F80" s="2"/>
       <c r="G80" s="2"/>
-    </row>
-    <row r="81" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H80" s="2"/>
+    </row>
+    <row r="81" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D81" s="2"/>
+      <c r="F81" s="2"/>
       <c r="G81" s="2"/>
-    </row>
-    <row r="82" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H81" s="2"/>
+    </row>
+    <row r="82" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D82" s="2"/>
+      <c r="F82" s="2"/>
       <c r="G82" s="2"/>
-    </row>
-    <row r="83" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H82" s="2"/>
+    </row>
+    <row r="83" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D83" s="2"/>
+      <c r="F83" s="2"/>
       <c r="G83" s="2"/>
-    </row>
-    <row r="84" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H83" s="2"/>
+    </row>
+    <row r="84" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D84" s="2"/>
+      <c r="F84" s="2"/>
       <c r="G84" s="2"/>
-    </row>
-    <row r="85" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H84" s="2"/>
+    </row>
+    <row r="85" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D85" s="2"/>
+      <c r="F85" s="2"/>
       <c r="G85" s="2"/>
-    </row>
-    <row r="86" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H85" s="2"/>
+    </row>
+    <row r="86" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D86" s="2"/>
+      <c r="F86" s="2"/>
       <c r="G86" s="2"/>
-    </row>
-    <row r="87" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H86" s="2"/>
+    </row>
+    <row r="87" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D87" s="2"/>
+      <c r="F87" s="2"/>
       <c r="G87" s="2"/>
-    </row>
-    <row r="88" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H87" s="2"/>
+    </row>
+    <row r="88" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D88" s="2"/>
+      <c r="F88" s="2"/>
       <c r="G88" s="2"/>
-    </row>
-    <row r="89" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H88" s="2"/>
+    </row>
+    <row r="89" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D89" s="2"/>
+      <c r="F89" s="2"/>
       <c r="G89" s="2"/>
-    </row>
-    <row r="90" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H89" s="2"/>
+    </row>
+    <row r="90" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D90" s="2"/>
+      <c r="F90" s="2"/>
       <c r="G90" s="2"/>
-    </row>
-    <row r="91" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H90" s="2"/>
+    </row>
+    <row r="91" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D91" s="2"/>
+      <c r="F91" s="2"/>
       <c r="G91" s="2"/>
-    </row>
-    <row r="92" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H91" s="2"/>
+    </row>
+    <row r="92" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D92" s="2"/>
+      <c r="F92" s="2"/>
       <c r="G92" s="2"/>
-    </row>
-    <row r="93" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H92" s="2"/>
+    </row>
+    <row r="93" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D93" s="2"/>
+      <c r="F93" s="2"/>
       <c r="G93" s="2"/>
-    </row>
-    <row r="94" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H93" s="2"/>
+    </row>
+    <row r="94" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D94" s="2"/>
+      <c r="F94" s="2"/>
       <c r="G94" s="2"/>
-    </row>
-    <row r="95" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H94" s="2"/>
+    </row>
+    <row r="95" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D95" s="2"/>
+      <c r="F95" s="2"/>
       <c r="G95" s="2"/>
-    </row>
-    <row r="96" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H95" s="2"/>
+    </row>
+    <row r="96" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D96" s="2"/>
+      <c r="F96" s="2"/>
       <c r="G96" s="2"/>
-    </row>
-    <row r="97" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H96" s="2"/>
+    </row>
+    <row r="97" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D97" s="2"/>
+      <c r="F97" s="2"/>
       <c r="G97" s="2"/>
-    </row>
-    <row r="98" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H97" s="2"/>
+    </row>
+    <row r="98" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D98" s="2"/>
+      <c r="F98" s="2"/>
       <c r="G98" s="2"/>
-    </row>
-    <row r="99" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H98" s="2"/>
+    </row>
+    <row r="99" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D99" s="2"/>
+      <c r="F99" s="2"/>
       <c r="G99" s="2"/>
-    </row>
-    <row r="100" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H99" s="2"/>
+    </row>
+    <row r="100" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D100" s="2"/>
+      <c r="F100" s="2"/>
       <c r="G100" s="2"/>
-    </row>
-    <row r="101" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H100" s="2"/>
+    </row>
+    <row r="101" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D101" s="2"/>
+      <c r="F101" s="2"/>
       <c r="G101" s="2"/>
-    </row>
-    <row r="102" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H101" s="2"/>
+    </row>
+    <row r="102" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D102" s="2"/>
+      <c r="F102" s="2"/>
       <c r="G102" s="2"/>
-    </row>
-    <row r="103" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H102" s="2"/>
+    </row>
+    <row r="103" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D103" s="2"/>
+      <c r="F103" s="2"/>
       <c r="G103" s="2"/>
-    </row>
-    <row r="104" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H103" s="2"/>
+    </row>
+    <row r="104" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D104" s="2"/>
+      <c r="F104" s="2"/>
       <c r="G104" s="2"/>
-    </row>
-    <row r="105" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H104" s="2"/>
+    </row>
+    <row r="105" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D105" s="2"/>
+      <c r="F105" s="2"/>
       <c r="G105" s="2"/>
-    </row>
-    <row r="106" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H105" s="2"/>
+    </row>
+    <row r="106" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D106" s="2"/>
+      <c r="F106" s="2"/>
       <c r="G106" s="2"/>
-    </row>
-    <row r="107" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H106" s="2"/>
+    </row>
+    <row r="107" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D107" s="2"/>
+      <c r="F107" s="2"/>
       <c r="G107" s="2"/>
-    </row>
-    <row r="108" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H107" s="2"/>
+    </row>
+    <row r="108" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D108" s="2"/>
+      <c r="F108" s="2"/>
       <c r="G108" s="2"/>
-    </row>
-    <row r="109" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H108" s="2"/>
+    </row>
+    <row r="109" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D109" s="2"/>
+      <c r="F109" s="2"/>
       <c r="G109" s="2"/>
-    </row>
-    <row r="110" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H109" s="2"/>
+    </row>
+    <row r="110" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D110" s="2"/>
+      <c r="F110" s="2"/>
       <c r="G110" s="2"/>
-    </row>
-    <row r="111" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H110" s="2"/>
+    </row>
+    <row r="111" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D111" s="2"/>
+      <c r="F111" s="2"/>
       <c r="G111" s="2"/>
-    </row>
-    <row r="112" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H111" s="2"/>
+    </row>
+    <row r="112" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D112" s="2"/>
+      <c r="F112" s="2"/>
       <c r="G112" s="2"/>
-    </row>
-    <row r="113" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H112" s="2"/>
+    </row>
+    <row r="113" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D113" s="2"/>
+      <c r="F113" s="2"/>
       <c r="G113" s="2"/>
-    </row>
-    <row r="114" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H113" s="2"/>
+    </row>
+    <row r="114" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D114" s="2"/>
+      <c r="F114" s="2"/>
       <c r="G114" s="2"/>
-    </row>
-    <row r="115" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H114" s="2"/>
+    </row>
+    <row r="115" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D115" s="2"/>
+      <c r="F115" s="2"/>
       <c r="G115" s="2"/>
-    </row>
-    <row r="116" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H115" s="2"/>
+    </row>
+    <row r="116" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D116" s="2"/>
+      <c r="F116" s="2"/>
       <c r="G116" s="2"/>
-    </row>
-    <row r="117" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H116" s="2"/>
+    </row>
+    <row r="117" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D117" s="2"/>
+      <c r="F117" s="2"/>
       <c r="G117" s="2"/>
-    </row>
-    <row r="118" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H117" s="2"/>
+    </row>
+    <row r="118" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D118" s="2"/>
+      <c r="F118" s="2"/>
       <c r="G118" s="2"/>
-    </row>
-    <row r="119" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H118" s="2"/>
+    </row>
+    <row r="119" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D119" s="2"/>
+      <c r="F119" s="2"/>
       <c r="G119" s="2"/>
-    </row>
-    <row r="120" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H119" s="2"/>
+    </row>
+    <row r="120" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D120" s="2"/>
+      <c r="F120" s="2"/>
       <c r="G120" s="2"/>
-    </row>
-    <row r="121" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H120" s="2"/>
+    </row>
+    <row r="121" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D121" s="2"/>
+      <c r="F121" s="2"/>
       <c r="G121" s="2"/>
-    </row>
-    <row r="122" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H121" s="2"/>
+    </row>
+    <row r="122" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D122" s="2"/>
+      <c r="F122" s="2"/>
       <c r="G122" s="2"/>
-    </row>
-    <row r="123" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H122" s="2"/>
+    </row>
+    <row r="123" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D123" s="2"/>
+      <c r="F123" s="2"/>
       <c r="G123" s="2"/>
-    </row>
-    <row r="124" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H123" s="2"/>
+    </row>
+    <row r="124" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D124" s="2"/>
+      <c r="F124" s="2"/>
       <c r="G124" s="2"/>
-    </row>
-    <row r="125" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H124" s="2"/>
+    </row>
+    <row r="125" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D125" s="2"/>
+      <c r="F125" s="2"/>
       <c r="G125" s="2"/>
-    </row>
-    <row r="126" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H125" s="2"/>
+    </row>
+    <row r="126" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D126" s="2"/>
+      <c r="F126" s="2"/>
       <c r="G126" s="2"/>
-    </row>
-    <row r="127" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H126" s="2"/>
+    </row>
+    <row r="127" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D127" s="2"/>
+      <c r="F127" s="2"/>
       <c r="G127" s="2"/>
-    </row>
-    <row r="128" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H127" s="2"/>
+    </row>
+    <row r="128" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D128" s="2"/>
+      <c r="F128" s="2"/>
       <c r="G128" s="2"/>
-    </row>
-    <row r="129" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H128" s="2"/>
+    </row>
+    <row r="129" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D129" s="2"/>
+      <c r="F129" s="2"/>
       <c r="G129" s="2"/>
-    </row>
-    <row r="130" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H129" s="2"/>
+    </row>
+    <row r="130" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D130" s="2"/>
+      <c r="F130" s="2"/>
       <c r="G130" s="2"/>
-    </row>
-    <row r="131" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H130" s="2"/>
+    </row>
+    <row r="131" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D131" s="2"/>
+      <c r="F131" s="2"/>
       <c r="G131" s="2"/>
-    </row>
-    <row r="132" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H131" s="2"/>
+    </row>
+    <row r="132" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D132" s="2"/>
+      <c r="F132" s="2"/>
       <c r="G132" s="2"/>
-    </row>
-    <row r="133" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H132" s="2"/>
+    </row>
+    <row r="133" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D133" s="2"/>
+      <c r="F133" s="2"/>
       <c r="G133" s="2"/>
-    </row>
-    <row r="134" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H133" s="2"/>
+    </row>
+    <row r="134" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D134" s="2"/>
+      <c r="F134" s="2"/>
       <c r="G134" s="2"/>
-    </row>
-    <row r="135" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H134" s="2"/>
+    </row>
+    <row r="135" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D135" s="2"/>
+      <c r="F135" s="2"/>
       <c r="G135" s="2"/>
-    </row>
-    <row r="136" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H135" s="2"/>
+    </row>
+    <row r="136" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D136" s="2"/>
+      <c r="F136" s="2"/>
       <c r="G136" s="2"/>
-    </row>
-    <row r="137" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H136" s="2"/>
+    </row>
+    <row r="137" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D137" s="2"/>
+      <c r="F137" s="2"/>
       <c r="G137" s="2"/>
-    </row>
-    <row r="138" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H137" s="2"/>
+    </row>
+    <row r="138" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D138" s="2"/>
+      <c r="F138" s="2"/>
       <c r="G138" s="2"/>
-    </row>
-    <row r="139" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H138" s="2"/>
+    </row>
+    <row r="139" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D139" s="2"/>
+      <c r="F139" s="2"/>
       <c r="G139" s="2"/>
-    </row>
-    <row r="140" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H139" s="2"/>
+    </row>
+    <row r="140" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D140" s="2"/>
+      <c r="F140" s="2"/>
       <c r="G140" s="2"/>
-    </row>
-    <row r="141" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H140" s="2"/>
+    </row>
+    <row r="141" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D141" s="2"/>
+      <c r="F141" s="2"/>
       <c r="G141" s="2"/>
-    </row>
-    <row r="142" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H141" s="2"/>
+    </row>
+    <row r="142" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D142" s="2"/>
+      <c r="F142" s="2"/>
       <c r="G142" s="2"/>
-    </row>
-    <row r="143" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H142" s="2"/>
+    </row>
+    <row r="143" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D143" s="2"/>
+      <c r="F143" s="2"/>
       <c r="G143" s="2"/>
-    </row>
-    <row r="144" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H143" s="2"/>
+    </row>
+    <row r="144" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D144" s="2"/>
+      <c r="F144" s="2"/>
       <c r="G144" s="2"/>
-    </row>
-    <row r="145" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H144" s="2"/>
+    </row>
+    <row r="145" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D145" s="2"/>
+      <c r="F145" s="2"/>
       <c r="G145" s="2"/>
-    </row>
-    <row r="146" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H145" s="2"/>
+    </row>
+    <row r="146" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D146" s="2"/>
+      <c r="F146" s="2"/>
       <c r="G146" s="2"/>
-    </row>
-    <row r="147" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H146" s="2"/>
+    </row>
+    <row r="147" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D147" s="2"/>
+      <c r="F147" s="2"/>
       <c r="G147" s="2"/>
-    </row>
-    <row r="148" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H147" s="2"/>
+    </row>
+    <row r="148" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D148" s="2"/>
+      <c r="F148" s="2"/>
       <c r="G148" s="2"/>
-    </row>
-    <row r="149" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H148" s="2"/>
+    </row>
+    <row r="149" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D149" s="2"/>
+      <c r="F149" s="2"/>
       <c r="G149" s="2"/>
-    </row>
-    <row r="150" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H149" s="2"/>
+    </row>
+    <row r="150" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D150" s="2"/>
+      <c r="F150" s="2"/>
       <c r="G150" s="2"/>
-    </row>
-    <row r="151" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H150" s="2"/>
+    </row>
+    <row r="151" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D151" s="2"/>
+      <c r="F151" s="2"/>
       <c r="G151" s="2"/>
-    </row>
-    <row r="152" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H151" s="2"/>
+    </row>
+    <row r="152" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D152" s="2"/>
+      <c r="F152" s="2"/>
       <c r="G152" s="2"/>
-    </row>
-    <row r="153" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H152" s="2"/>
+    </row>
+    <row r="153" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D153" s="2"/>
+      <c r="F153" s="2"/>
       <c r="G153" s="2"/>
-    </row>
-    <row r="154" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H153" s="2"/>
+    </row>
+    <row r="154" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D154" s="2"/>
+      <c r="F154" s="2"/>
       <c r="G154" s="2"/>
-    </row>
-    <row r="155" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H154" s="2"/>
+    </row>
+    <row r="155" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D155" s="2"/>
+      <c r="F155" s="2"/>
       <c r="G155" s="2"/>
-    </row>
-    <row r="156" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H155" s="2"/>
+    </row>
+    <row r="156" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D156" s="2"/>
+      <c r="F156" s="2"/>
       <c r="G156" s="2"/>
-    </row>
-    <row r="157" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H156" s="2"/>
+    </row>
+    <row r="157" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D157" s="2"/>
+      <c r="F157" s="2"/>
       <c r="G157" s="2"/>
-    </row>
-    <row r="158" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H157" s="2"/>
+    </row>
+    <row r="158" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D158" s="2"/>
+      <c r="F158" s="2"/>
       <c r="G158" s="2"/>
-    </row>
-    <row r="159" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H158" s="2"/>
+    </row>
+    <row r="159" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D159" s="2"/>
+      <c r="F159" s="2"/>
       <c r="G159" s="2"/>
-    </row>
-    <row r="160" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H159" s="2"/>
+    </row>
+    <row r="160" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D160" s="2"/>
+      <c r="F160" s="2"/>
       <c r="G160" s="2"/>
-    </row>
-    <row r="161" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H160" s="2"/>
+    </row>
+    <row r="161" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D161" s="2"/>
+      <c r="F161" s="2"/>
       <c r="G161" s="2"/>
-    </row>
-    <row r="162" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H161" s="2"/>
+    </row>
+    <row r="162" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D162" s="2"/>
+      <c r="F162" s="2"/>
       <c r="G162" s="2"/>
-    </row>
-    <row r="163" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H162" s="2"/>
+    </row>
+    <row r="163" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D163" s="2"/>
+      <c r="F163" s="2"/>
       <c r="G163" s="2"/>
-    </row>
-    <row r="164" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H163" s="2"/>
+    </row>
+    <row r="164" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D164" s="2"/>
+      <c r="F164" s="2"/>
       <c r="G164" s="2"/>
-    </row>
-    <row r="165" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H164" s="2"/>
+    </row>
+    <row r="165" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D165" s="2"/>
+      <c r="F165" s="2"/>
       <c r="G165" s="2"/>
-    </row>
-    <row r="166" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H165" s="2"/>
+    </row>
+    <row r="166" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D166" s="2"/>
+      <c r="F166" s="2"/>
       <c r="G166" s="2"/>
-    </row>
-    <row r="167" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H166" s="2"/>
+    </row>
+    <row r="167" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D167" s="2"/>
+      <c r="F167" s="2"/>
       <c r="G167" s="2"/>
-    </row>
-    <row r="168" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H167" s="2"/>
+    </row>
+    <row r="168" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D168" s="2"/>
+      <c r="F168" s="2"/>
       <c r="G168" s="2"/>
-    </row>
-    <row r="169" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H168" s="2"/>
+    </row>
+    <row r="169" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D169" s="2"/>
+      <c r="F169" s="2"/>
       <c r="G169" s="2"/>
-    </row>
-    <row r="170" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H169" s="2"/>
+    </row>
+    <row r="170" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D170" s="2"/>
+      <c r="F170" s="2"/>
       <c r="G170" s="2"/>
-    </row>
-    <row r="171" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H170" s="2"/>
+    </row>
+    <row r="171" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D171" s="2"/>
+      <c r="F171" s="2"/>
       <c r="G171" s="2"/>
-    </row>
-    <row r="172" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H171" s="2"/>
+    </row>
+    <row r="172" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D172" s="2"/>
+      <c r="F172" s="2"/>
       <c r="G172" s="2"/>
-    </row>
-    <row r="173" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H172" s="2"/>
+    </row>
+    <row r="173" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D173" s="2"/>
+      <c r="F173" s="2"/>
       <c r="G173" s="2"/>
-    </row>
-    <row r="174" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H173" s="2"/>
+    </row>
+    <row r="174" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D174" s="2"/>
+      <c r="F174" s="2"/>
       <c r="G174" s="2"/>
-    </row>
-    <row r="175" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H174" s="2"/>
+    </row>
+    <row r="175" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D175" s="2"/>
+      <c r="F175" s="2"/>
       <c r="G175" s="2"/>
-    </row>
-    <row r="176" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H175" s="2"/>
+    </row>
+    <row r="176" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D176" s="2"/>
+      <c r="F176" s="2"/>
       <c r="G176" s="2"/>
-    </row>
-    <row r="177" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H176" s="2"/>
+    </row>
+    <row r="177" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D177" s="2"/>
+      <c r="F177" s="2"/>
       <c r="G177" s="2"/>
-    </row>
-    <row r="178" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H177" s="2"/>
+    </row>
+    <row r="178" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D178" s="2"/>
+      <c r="F178" s="2"/>
       <c r="G178" s="2"/>
-    </row>
-    <row r="179" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H178" s="2"/>
+    </row>
+    <row r="179" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D179" s="2"/>
+      <c r="F179" s="2"/>
       <c r="G179" s="2"/>
-    </row>
-    <row r="180" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H179" s="2"/>
+    </row>
+    <row r="180" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D180" s="2"/>
+      <c r="F180" s="2"/>
       <c r="G180" s="2"/>
-    </row>
-    <row r="181" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H180" s="2"/>
+    </row>
+    <row r="181" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D181" s="2"/>
+      <c r="F181" s="2"/>
       <c r="G181" s="2"/>
-    </row>
-    <row r="182" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H181" s="2"/>
+    </row>
+    <row r="182" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D182" s="2"/>
+      <c r="F182" s="2"/>
       <c r="G182" s="2"/>
-    </row>
-    <row r="183" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H182" s="2"/>
+    </row>
+    <row r="183" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D183" s="2"/>
+      <c r="F183" s="2"/>
       <c r="G183" s="2"/>
-    </row>
-    <row r="184" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H183" s="2"/>
+    </row>
+    <row r="184" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D184" s="2"/>
+      <c r="F184" s="2"/>
       <c r="G184" s="2"/>
-    </row>
-    <row r="185" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H184" s="2"/>
+    </row>
+    <row r="185" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D185" s="2"/>
+      <c r="F185" s="2"/>
       <c r="G185" s="2"/>
-    </row>
-    <row r="186" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H185" s="2"/>
+    </row>
+    <row r="186" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D186" s="2"/>
+      <c r="F186" s="2"/>
       <c r="G186" s="2"/>
-    </row>
-    <row r="187" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H186" s="2"/>
+    </row>
+    <row r="187" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D187" s="2"/>
+      <c r="F187" s="2"/>
       <c r="G187" s="2"/>
-    </row>
-    <row r="188" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H187" s="2"/>
+    </row>
+    <row r="188" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D188" s="2"/>
+      <c r="F188" s="2"/>
       <c r="G188" s="2"/>
-    </row>
-    <row r="189" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H188" s="2"/>
+    </row>
+    <row r="189" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D189" s="2"/>
+      <c r="F189" s="2"/>
       <c r="G189" s="2"/>
-    </row>
-    <row r="190" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H189" s="2"/>
+    </row>
+    <row r="190" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D190" s="2"/>
+      <c r="F190" s="2"/>
       <c r="G190" s="2"/>
-    </row>
-    <row r="191" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H190" s="2"/>
+    </row>
+    <row r="191" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D191" s="2"/>
+      <c r="F191" s="2"/>
       <c r="G191" s="2"/>
-    </row>
-    <row r="192" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H191" s="2"/>
+    </row>
+    <row r="192" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D192" s="2"/>
+      <c r="F192" s="2"/>
       <c r="G192" s="2"/>
-    </row>
-    <row r="193" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H192" s="2"/>
+    </row>
+    <row r="193" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D193" s="2"/>
+      <c r="F193" s="2"/>
       <c r="G193" s="2"/>
-    </row>
-    <row r="194" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H193" s="2"/>
+    </row>
+    <row r="194" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D194" s="2"/>
+      <c r="F194" s="2"/>
       <c r="G194" s="2"/>
-    </row>
-    <row r="195" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H194" s="2"/>
+    </row>
+    <row r="195" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D195" s="2"/>
+      <c r="F195" s="2"/>
       <c r="G195" s="2"/>
-    </row>
-    <row r="196" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H195" s="2"/>
+    </row>
+    <row r="196" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D196" s="2"/>
+      <c r="F196" s="2"/>
       <c r="G196" s="2"/>
-    </row>
-    <row r="197" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H196" s="2"/>
+    </row>
+    <row r="197" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D197" s="2"/>
+      <c r="F197" s="2"/>
       <c r="G197" s="2"/>
-    </row>
-    <row r="198" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H197" s="2"/>
+    </row>
+    <row r="198" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D198" s="2"/>
+      <c r="F198" s="2"/>
       <c r="G198" s="2"/>
-    </row>
-    <row r="199" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H198" s="2"/>
+    </row>
+    <row r="199" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D199" s="2"/>
+      <c r="F199" s="2"/>
       <c r="G199" s="2"/>
-    </row>
-    <row r="200" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H199" s="2"/>
+    </row>
+    <row r="200" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D200" s="2"/>
+      <c r="F200" s="2"/>
       <c r="G200" s="2"/>
-    </row>
-    <row r="201" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H200" s="2"/>
+    </row>
+    <row r="201" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D201" s="2"/>
+      <c r="F201" s="2"/>
       <c r="G201" s="2"/>
-    </row>
-    <row r="202" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H201" s="2"/>
+    </row>
+    <row r="202" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D202" s="2"/>
+      <c r="F202" s="2"/>
       <c r="G202" s="2"/>
-    </row>
-    <row r="203" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H202" s="2"/>
+    </row>
+    <row r="203" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D203" s="2"/>
+      <c r="F203" s="2"/>
       <c r="G203" s="2"/>
-    </row>
-    <row r="204" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H203" s="2"/>
+    </row>
+    <row r="204" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D204" s="2"/>
+      <c r="F204" s="2"/>
       <c r="G204" s="2"/>
-    </row>
-    <row r="205" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H204" s="2"/>
+    </row>
+    <row r="205" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D205" s="2"/>
+      <c r="F205" s="2"/>
       <c r="G205" s="2"/>
-    </row>
-    <row r="206" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H205" s="2"/>
+    </row>
+    <row r="206" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D206" s="2"/>
+      <c r="F206" s="2"/>
       <c r="G206" s="2"/>
-    </row>
-    <row r="207" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H206" s="2"/>
+    </row>
+    <row r="207" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D207" s="2"/>
+      <c r="F207" s="2"/>
       <c r="G207" s="2"/>
-    </row>
-    <row r="208" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H207" s="2"/>
+    </row>
+    <row r="208" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D208" s="2"/>
+      <c r="F208" s="2"/>
       <c r="G208" s="2"/>
-    </row>
-    <row r="209" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H208" s="2"/>
+    </row>
+    <row r="209" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D209" s="2"/>
+      <c r="F209" s="2"/>
       <c r="G209" s="2"/>
-    </row>
-    <row r="210" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H209" s="2"/>
+    </row>
+    <row r="210" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D210" s="2"/>
+      <c r="F210" s="2"/>
       <c r="G210" s="2"/>
-    </row>
-    <row r="211" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H210" s="2"/>
+    </row>
+    <row r="211" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D211" s="2"/>
+      <c r="F211" s="2"/>
       <c r="G211" s="2"/>
-    </row>
-    <row r="212" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H211" s="2"/>
+    </row>
+    <row r="212" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D212" s="2"/>
+      <c r="F212" s="2"/>
       <c r="G212" s="2"/>
-    </row>
-    <row r="213" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H212" s="2"/>
+    </row>
+    <row r="213" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D213" s="2"/>
+      <c r="F213" s="2"/>
       <c r="G213" s="2"/>
-    </row>
-    <row r="214" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H213" s="2"/>
+    </row>
+    <row r="214" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D214" s="2"/>
+      <c r="F214" s="2"/>
       <c r="G214" s="2"/>
-    </row>
-    <row r="215" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H214" s="2"/>
+    </row>
+    <row r="215" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D215" s="2"/>
+      <c r="F215" s="2"/>
       <c r="G215" s="2"/>
-    </row>
-    <row r="216" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H215" s="2"/>
+    </row>
+    <row r="216" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D216" s="2"/>
+      <c r="F216" s="2"/>
       <c r="G216" s="2"/>
-    </row>
-    <row r="217" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H216" s="2"/>
+    </row>
+    <row r="217" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D217" s="2"/>
+      <c r="F217" s="2"/>
       <c r="G217" s="2"/>
-    </row>
-    <row r="218" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H217" s="2"/>
+    </row>
+    <row r="218" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D218" s="2"/>
+      <c r="F218" s="2"/>
       <c r="G218" s="2"/>
-    </row>
-    <row r="219" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H218" s="2"/>
+    </row>
+    <row r="219" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D219" s="2"/>
+      <c r="F219" s="2"/>
       <c r="G219" s="2"/>
-    </row>
-    <row r="220" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H219" s="2"/>
+    </row>
+    <row r="220" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D220" s="2"/>
+      <c r="F220" s="2"/>
       <c r="G220" s="2"/>
-    </row>
-    <row r="221" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H220" s="2"/>
+    </row>
+    <row r="221" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D221" s="2"/>
+      <c r="F221" s="2"/>
       <c r="G221" s="2"/>
-    </row>
-    <row r="222" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H221" s="2"/>
+    </row>
+    <row r="222" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D222" s="2"/>
+      <c r="F222" s="2"/>
       <c r="G222" s="2"/>
-    </row>
-    <row r="223" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H222" s="2"/>
+    </row>
+    <row r="223" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D223" s="2"/>
+      <c r="F223" s="2"/>
       <c r="G223" s="2"/>
-    </row>
-    <row r="224" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H223" s="2"/>
+    </row>
+    <row r="224" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D224" s="2"/>
+      <c r="F224" s="2"/>
       <c r="G224" s="2"/>
-    </row>
-    <row r="225" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H224" s="2"/>
+    </row>
+    <row r="225" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D225" s="2"/>
+      <c r="F225" s="2"/>
       <c r="G225" s="2"/>
-    </row>
-    <row r="226" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H225" s="2"/>
+    </row>
+    <row r="226" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D226" s="2"/>
+      <c r="F226" s="2"/>
       <c r="G226" s="2"/>
-    </row>
-    <row r="227" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H226" s="2"/>
+    </row>
+    <row r="227" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D227" s="2"/>
+      <c r="F227" s="2"/>
       <c r="G227" s="2"/>
-    </row>
-    <row r="228" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H227" s="2"/>
+    </row>
+    <row r="228" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D228" s="2"/>
+      <c r="F228" s="2"/>
       <c r="G228" s="2"/>
-    </row>
-    <row r="229" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H228" s="2"/>
+    </row>
+    <row r="229" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D229" s="2"/>
+      <c r="F229" s="2"/>
       <c r="G229" s="2"/>
-    </row>
-    <row r="230" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H229" s="2"/>
+    </row>
+    <row r="230" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D230" s="2"/>
+      <c r="F230" s="2"/>
       <c r="G230" s="2"/>
-    </row>
-    <row r="231" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H230" s="2"/>
+    </row>
+    <row r="231" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D231" s="2"/>
+      <c r="F231" s="2"/>
       <c r="G231" s="2"/>
-    </row>
-    <row r="232" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H231" s="2"/>
+    </row>
+    <row r="232" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D232" s="2"/>
+      <c r="F232" s="2"/>
       <c r="G232" s="2"/>
-    </row>
-    <row r="233" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H232" s="2"/>
+    </row>
+    <row r="233" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D233" s="2"/>
+      <c r="F233" s="2"/>
       <c r="G233" s="2"/>
-    </row>
-    <row r="234" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H233" s="2"/>
+    </row>
+    <row r="234" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D234" s="2"/>
+      <c r="F234" s="2"/>
       <c r="G234" s="2"/>
-    </row>
-    <row r="235" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H234" s="2"/>
+    </row>
+    <row r="235" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D235" s="2"/>
+      <c r="F235" s="2"/>
       <c r="G235" s="2"/>
-    </row>
-    <row r="236" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H235" s="2"/>
+    </row>
+    <row r="236" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D236" s="2"/>
+      <c r="F236" s="2"/>
       <c r="G236" s="2"/>
-    </row>
-    <row r="237" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H236" s="2"/>
+    </row>
+    <row r="237" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D237" s="2"/>
+      <c r="F237" s="2"/>
       <c r="G237" s="2"/>
-    </row>
-    <row r="238" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H237" s="2"/>
+    </row>
+    <row r="238" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D238" s="2"/>
+      <c r="F238" s="2"/>
       <c r="G238" s="2"/>
-    </row>
-    <row r="239" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H238" s="2"/>
+    </row>
+    <row r="239" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D239" s="2"/>
+      <c r="F239" s="2"/>
       <c r="G239" s="2"/>
-    </row>
-    <row r="240" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H239" s="2"/>
+    </row>
+    <row r="240" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D240" s="2"/>
+      <c r="F240" s="2"/>
       <c r="G240" s="2"/>
-    </row>
-    <row r="241" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H240" s="2"/>
+    </row>
+    <row r="241" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D241" s="2"/>
+      <c r="F241" s="2"/>
       <c r="G241" s="2"/>
-    </row>
-    <row r="242" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H241" s="2"/>
+    </row>
+    <row r="242" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D242" s="2"/>
+      <c r="F242" s="2"/>
       <c r="G242" s="2"/>
-    </row>
-    <row r="243" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H242" s="2"/>
+    </row>
+    <row r="243" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D243" s="2"/>
+      <c r="F243" s="2"/>
       <c r="G243" s="2"/>
-    </row>
-    <row r="244" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H243" s="2"/>
+    </row>
+    <row r="244" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D244" s="2"/>
+      <c r="F244" s="2"/>
       <c r="G244" s="2"/>
-    </row>
-    <row r="245" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H244" s="2"/>
+    </row>
+    <row r="245" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D245" s="2"/>
+      <c r="F245" s="2"/>
       <c r="G245" s="2"/>
-    </row>
-    <row r="246" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H245" s="2"/>
+    </row>
+    <row r="246" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D246" s="2"/>
+      <c r="F246" s="2"/>
       <c r="G246" s="2"/>
-    </row>
-    <row r="247" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H246" s="2"/>
+    </row>
+    <row r="247" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D247" s="2"/>
+      <c r="F247" s="2"/>
       <c r="G247" s="2"/>
-    </row>
-    <row r="248" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H247" s="2"/>
+    </row>
+    <row r="248" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D248" s="2"/>
+      <c r="F248" s="2"/>
       <c r="G248" s="2"/>
-    </row>
-    <row r="249" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H248" s="2"/>
+    </row>
+    <row r="249" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D249" s="2"/>
+      <c r="F249" s="2"/>
       <c r="G249" s="2"/>
-    </row>
-    <row r="250" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H249" s="2"/>
+    </row>
+    <row r="250" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D250" s="2"/>
+      <c r="F250" s="2"/>
       <c r="G250" s="2"/>
-    </row>
-    <row r="251" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H250" s="2"/>
+    </row>
+    <row r="251" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D251" s="2"/>
+      <c r="F251" s="2"/>
       <c r="G251" s="2"/>
-    </row>
-    <row r="252" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H251" s="2"/>
+    </row>
+    <row r="252" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D252" s="2"/>
+      <c r="F252" s="2"/>
       <c r="G252" s="2"/>
-    </row>
-    <row r="253" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H252" s="2"/>
+    </row>
+    <row r="253" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D253" s="2"/>
+      <c r="F253" s="2"/>
       <c r="G253" s="2"/>
-    </row>
-    <row r="254" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H253" s="2"/>
+    </row>
+    <row r="254" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D254" s="2"/>
+      <c r="F254" s="2"/>
       <c r="G254" s="2"/>
-    </row>
-    <row r="255" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H254" s="2"/>
+    </row>
+    <row r="255" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D255" s="2"/>
+      <c r="F255" s="2"/>
       <c r="G255" s="2"/>
-    </row>
-    <row r="256" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H255" s="2"/>
+    </row>
+    <row r="256" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D256" s="2"/>
+      <c r="F256" s="2"/>
       <c r="G256" s="2"/>
-    </row>
-    <row r="257" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H256" s="2"/>
+    </row>
+    <row r="257" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D257" s="2"/>
+      <c r="F257" s="2"/>
       <c r="G257" s="2"/>
-    </row>
-    <row r="258" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H257" s="2"/>
+    </row>
+    <row r="258" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D258" s="2"/>
+      <c r="F258" s="2"/>
       <c r="G258" s="2"/>
-    </row>
-    <row r="259" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H258" s="2"/>
+    </row>
+    <row r="259" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D259" s="2"/>
+      <c r="F259" s="2"/>
       <c r="G259" s="2"/>
-    </row>
-    <row r="260" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H259" s="2"/>
+    </row>
+    <row r="260" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D260" s="2"/>
+      <c r="F260" s="2"/>
       <c r="G260" s="2"/>
-    </row>
-    <row r="261" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H260" s="2"/>
+    </row>
+    <row r="261" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D261" s="2"/>
+      <c r="F261" s="2"/>
       <c r="G261" s="2"/>
-    </row>
-    <row r="262" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H261" s="2"/>
+    </row>
+    <row r="262" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D262" s="2"/>
+      <c r="F262" s="2"/>
       <c r="G262" s="2"/>
-    </row>
-    <row r="263" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H262" s="2"/>
+    </row>
+    <row r="263" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D263" s="2"/>
+      <c r="F263" s="2"/>
       <c r="G263" s="2"/>
-    </row>
-    <row r="264" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H263" s="2"/>
+    </row>
+    <row r="264" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D264" s="2"/>
+      <c r="F264" s="2"/>
       <c r="G264" s="2"/>
-    </row>
-    <row r="265" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H264" s="2"/>
+    </row>
+    <row r="265" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D265" s="2"/>
+      <c r="F265" s="2"/>
       <c r="G265" s="2"/>
-    </row>
-    <row r="266" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H265" s="2"/>
+    </row>
+    <row r="266" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D266" s="2"/>
+      <c r="F266" s="2"/>
       <c r="G266" s="2"/>
-    </row>
-    <row r="267" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H266" s="2"/>
+    </row>
+    <row r="267" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D267" s="2"/>
+      <c r="F267" s="2"/>
       <c r="G267" s="2"/>
-    </row>
-    <row r="268" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H267" s="2"/>
+    </row>
+    <row r="268" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D268" s="2"/>
+      <c r="F268" s="2"/>
       <c r="G268" s="2"/>
-    </row>
-    <row r="269" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H268" s="2"/>
+    </row>
+    <row r="269" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D269" s="2"/>
+      <c r="F269" s="2"/>
       <c r="G269" s="2"/>
-    </row>
-    <row r="270" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H269" s="2"/>
+    </row>
+    <row r="270" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D270" s="2"/>
+      <c r="F270" s="2"/>
       <c r="G270" s="2"/>
-    </row>
-    <row r="271" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H270" s="2"/>
+    </row>
+    <row r="271" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D271" s="2"/>
+      <c r="F271" s="2"/>
       <c r="G271" s="2"/>
-    </row>
-    <row r="272" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H271" s="2"/>
+    </row>
+    <row r="272" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D272" s="2"/>
+      <c r="F272" s="2"/>
       <c r="G272" s="2"/>
-    </row>
-    <row r="273" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H272" s="2"/>
+    </row>
+    <row r="273" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D273" s="2"/>
+      <c r="F273" s="2"/>
       <c r="G273" s="2"/>
-    </row>
-    <row r="274" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H273" s="2"/>
+    </row>
+    <row r="274" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D274" s="2"/>
+      <c r="F274" s="2"/>
       <c r="G274" s="2"/>
-    </row>
-    <row r="275" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H274" s="2"/>
+    </row>
+    <row r="275" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D275" s="2"/>
+      <c r="F275" s="2"/>
       <c r="G275" s="2"/>
-    </row>
-    <row r="276" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H275" s="2"/>
+    </row>
+    <row r="276" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D276" s="2"/>
+      <c r="F276" s="2"/>
       <c r="G276" s="2"/>
-    </row>
-    <row r="277" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H276" s="2"/>
+    </row>
+    <row r="277" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D277" s="2"/>
+      <c r="F277" s="2"/>
       <c r="G277" s="2"/>
-    </row>
-    <row r="278" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H277" s="2"/>
+    </row>
+    <row r="278" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D278" s="2"/>
+      <c r="F278" s="2"/>
       <c r="G278" s="2"/>
-    </row>
-    <row r="279" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H278" s="2"/>
+    </row>
+    <row r="279" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D279" s="2"/>
+      <c r="F279" s="2"/>
       <c r="G279" s="2"/>
-    </row>
-    <row r="280" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H279" s="2"/>
+    </row>
+    <row r="280" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D280" s="2"/>
+      <c r="F280" s="2"/>
       <c r="G280" s="2"/>
-    </row>
-    <row r="281" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H280" s="2"/>
+    </row>
+    <row r="281" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D281" s="2"/>
+      <c r="F281" s="2"/>
       <c r="G281" s="2"/>
-    </row>
-    <row r="282" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H281" s="2"/>
+    </row>
+    <row r="282" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D282" s="2"/>
+      <c r="F282" s="2"/>
       <c r="G282" s="2"/>
-    </row>
-    <row r="283" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H282" s="2"/>
+    </row>
+    <row r="283" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D283" s="2"/>
+      <c r="F283" s="2"/>
       <c r="G283" s="2"/>
-    </row>
-    <row r="284" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H283" s="2"/>
+    </row>
+    <row r="284" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D284" s="2"/>
+      <c r="F284" s="2"/>
       <c r="G284" s="2"/>
-    </row>
-    <row r="285" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H284" s="2"/>
+    </row>
+    <row r="285" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D285" s="2"/>
+      <c r="F285" s="2"/>
       <c r="G285" s="2"/>
-    </row>
-    <row r="286" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H285" s="2"/>
+    </row>
+    <row r="286" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D286" s="2"/>
+      <c r="F286" s="2"/>
       <c r="G286" s="2"/>
-    </row>
-    <row r="287" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H286" s="2"/>
+    </row>
+    <row r="287" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D287" s="2"/>
+      <c r="F287" s="2"/>
       <c r="G287" s="2"/>
-    </row>
-    <row r="288" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H287" s="2"/>
+    </row>
+    <row r="288" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D288" s="2"/>
+      <c r="F288" s="2"/>
       <c r="G288" s="2"/>
-    </row>
-    <row r="289" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H288" s="2"/>
+    </row>
+    <row r="289" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D289" s="2"/>
+      <c r="F289" s="2"/>
       <c r="G289" s="2"/>
-    </row>
-    <row r="290" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H289" s="2"/>
+    </row>
+    <row r="290" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D290" s="2"/>
+      <c r="F290" s="2"/>
       <c r="G290" s="2"/>
-    </row>
-    <row r="291" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H290" s="2"/>
+    </row>
+    <row r="291" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D291" s="2"/>
+      <c r="F291" s="2"/>
       <c r="G291" s="2"/>
-    </row>
-    <row r="292" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H291" s="2"/>
+    </row>
+    <row r="292" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D292" s="2"/>
+      <c r="F292" s="2"/>
       <c r="G292" s="2"/>
-    </row>
-    <row r="293" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H292" s="2"/>
+    </row>
+    <row r="293" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D293" s="2"/>
+      <c r="F293" s="2"/>
       <c r="G293" s="2"/>
-    </row>
-    <row r="294" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H293" s="2"/>
+    </row>
+    <row r="294" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D294" s="2"/>
+      <c r="F294" s="2"/>
       <c r="G294" s="2"/>
-    </row>
-    <row r="295" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H294" s="2"/>
+    </row>
+    <row r="295" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D295" s="2"/>
+      <c r="F295" s="2"/>
       <c r="G295" s="2"/>
-    </row>
-    <row r="296" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H295" s="2"/>
+    </row>
+    <row r="296" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D296" s="2"/>
+      <c r="F296" s="2"/>
       <c r="G296" s="2"/>
-    </row>
-    <row r="297" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H296" s="2"/>
+    </row>
+    <row r="297" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D297" s="2"/>
+      <c r="F297" s="2"/>
       <c r="G297" s="2"/>
-    </row>
-    <row r="298" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H297" s="2"/>
+    </row>
+    <row r="298" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D298" s="2"/>
+      <c r="F298" s="2"/>
       <c r="G298" s="2"/>
-    </row>
-    <row r="299" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H298" s="2"/>
+    </row>
+    <row r="299" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D299" s="2"/>
+      <c r="F299" s="2"/>
       <c r="G299" s="2"/>
-    </row>
-    <row r="300" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H299" s="2"/>
+    </row>
+    <row r="300" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D300" s="2"/>
+      <c r="F300" s="2"/>
       <c r="G300" s="2"/>
-    </row>
-    <row r="301" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H300" s="2"/>
+    </row>
+    <row r="301" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D301" s="2"/>
+      <c r="F301" s="2"/>
       <c r="G301" s="2"/>
-    </row>
-    <row r="302" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H301" s="2"/>
+    </row>
+    <row r="302" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D302" s="2"/>
+      <c r="F302" s="2"/>
       <c r="G302" s="2"/>
-    </row>
-    <row r="303" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H302" s="2"/>
+    </row>
+    <row r="303" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D303" s="2"/>
+      <c r="F303" s="2"/>
       <c r="G303" s="2"/>
-    </row>
-    <row r="304" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H303" s="2"/>
+    </row>
+    <row r="304" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D304" s="2"/>
+      <c r="F304" s="2"/>
       <c r="G304" s="2"/>
-    </row>
-    <row r="305" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H304" s="2"/>
+    </row>
+    <row r="305" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D305" s="2"/>
+      <c r="F305" s="2"/>
       <c r="G305" s="2"/>
-    </row>
-    <row r="306" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H305" s="2"/>
+    </row>
+    <row r="306" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D306" s="2"/>
+      <c r="F306" s="2"/>
       <c r="G306" s="2"/>
-    </row>
-    <row r="307" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H306" s="2"/>
+    </row>
+    <row r="307" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D307" s="2"/>
+      <c r="F307" s="2"/>
       <c r="G307" s="2"/>
-    </row>
-    <row r="308" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H307" s="2"/>
+    </row>
+    <row r="308" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D308" s="2"/>
+      <c r="F308" s="2"/>
       <c r="G308" s="2"/>
-    </row>
-    <row r="309" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H308" s="2"/>
+    </row>
+    <row r="309" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D309" s="2"/>
+      <c r="F309" s="2"/>
       <c r="G309" s="2"/>
-    </row>
-    <row r="310" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H309" s="2"/>
+    </row>
+    <row r="310" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D310" s="2"/>
+      <c r="F310" s="2"/>
       <c r="G310" s="2"/>
-    </row>
-    <row r="311" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H310" s="2"/>
+    </row>
+    <row r="311" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D311" s="2"/>
+      <c r="F311" s="2"/>
       <c r="G311" s="2"/>
-    </row>
-    <row r="312" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H311" s="2"/>
+    </row>
+    <row r="312" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D312" s="2"/>
+      <c r="F312" s="2"/>
       <c r="G312" s="2"/>
-    </row>
-    <row r="313" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H312" s="2"/>
+    </row>
+    <row r="313" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D313" s="2"/>
+      <c r="F313" s="2"/>
       <c r="G313" s="2"/>
-    </row>
-    <row r="314" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H313" s="2"/>
+    </row>
+    <row r="314" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D314" s="2"/>
+      <c r="F314" s="2"/>
       <c r="G314" s="2"/>
-    </row>
-    <row r="315" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H314" s="2"/>
+    </row>
+    <row r="315" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D315" s="2"/>
+      <c r="F315" s="2"/>
       <c r="G315" s="2"/>
-    </row>
-    <row r="316" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H315" s="2"/>
+    </row>
+    <row r="316" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D316" s="2"/>
+      <c r="F316" s="2"/>
       <c r="G316" s="2"/>
-    </row>
-    <row r="317" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H316" s="2"/>
+    </row>
+    <row r="317" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D317" s="2"/>
+      <c r="F317" s="2"/>
       <c r="G317" s="2"/>
-    </row>
-    <row r="318" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H317" s="2"/>
+    </row>
+    <row r="318" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D318" s="2"/>
+      <c r="F318" s="2"/>
       <c r="G318" s="2"/>
-    </row>
-    <row r="319" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H318" s="2"/>
+    </row>
+    <row r="319" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D319" s="2"/>
+      <c r="F319" s="2"/>
       <c r="G319" s="2"/>
-    </row>
-    <row r="320" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H319" s="2"/>
+    </row>
+    <row r="320" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D320" s="2"/>
+      <c r="F320" s="2"/>
       <c r="G320" s="2"/>
-    </row>
-    <row r="321" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H320" s="2"/>
+    </row>
+    <row r="321" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D321" s="2"/>
+      <c r="F321" s="2"/>
       <c r="G321" s="2"/>
-    </row>
-    <row r="322" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H321" s="2"/>
+    </row>
+    <row r="322" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D322" s="2"/>
+      <c r="F322" s="2"/>
       <c r="G322" s="2"/>
-    </row>
-    <row r="323" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H322" s="2"/>
+    </row>
+    <row r="323" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D323" s="2"/>
+      <c r="F323" s="2"/>
       <c r="G323" s="2"/>
-    </row>
-    <row r="324" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H323" s="2"/>
+    </row>
+    <row r="324" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D324" s="2"/>
+      <c r="F324" s="2"/>
       <c r="G324" s="2"/>
-    </row>
-    <row r="325" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H324" s="2"/>
+    </row>
+    <row r="325" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D325" s="2"/>
+      <c r="F325" s="2"/>
       <c r="G325" s="2"/>
-    </row>
-    <row r="326" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H325" s="2"/>
+    </row>
+    <row r="326" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D326" s="2"/>
+      <c r="F326" s="2"/>
       <c r="G326" s="2"/>
-    </row>
-    <row r="327" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H326" s="2"/>
+    </row>
+    <row r="327" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D327" s="2"/>
+      <c r="F327" s="2"/>
       <c r="G327" s="2"/>
-    </row>
-    <row r="328" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H327" s="2"/>
+    </row>
+    <row r="328" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D328" s="2"/>
+      <c r="F328" s="2"/>
       <c r="G328" s="2"/>
-    </row>
-    <row r="329" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H328" s="2"/>
+    </row>
+    <row r="329" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D329" s="2"/>
+      <c r="F329" s="2"/>
       <c r="G329" s="2"/>
-    </row>
-    <row r="330" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H329" s="2"/>
+    </row>
+    <row r="330" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D330" s="2"/>
+      <c r="F330" s="2"/>
       <c r="G330" s="2"/>
-    </row>
-    <row r="331" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H330" s="2"/>
+    </row>
+    <row r="331" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D331" s="2"/>
+      <c r="F331" s="2"/>
       <c r="G331" s="2"/>
-    </row>
-    <row r="332" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H331" s="2"/>
+    </row>
+    <row r="332" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D332" s="2"/>
+      <c r="F332" s="2"/>
       <c r="G332" s="2"/>
-    </row>
-    <row r="333" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H332" s="2"/>
+    </row>
+    <row r="333" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D333" s="2"/>
+      <c r="F333" s="2"/>
       <c r="G333" s="2"/>
-    </row>
-    <row r="334" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H333" s="2"/>
+    </row>
+    <row r="334" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D334" s="2"/>
+      <c r="F334" s="2"/>
       <c r="G334" s="2"/>
-    </row>
-    <row r="335" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H334" s="2"/>
+    </row>
+    <row r="335" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D335" s="2"/>
+      <c r="F335" s="2"/>
       <c r="G335" s="2"/>
-    </row>
-    <row r="336" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H335" s="2"/>
+    </row>
+    <row r="336" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D336" s="2"/>
+      <c r="F336" s="2"/>
       <c r="G336" s="2"/>
-    </row>
-    <row r="337" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H336" s="2"/>
+    </row>
+    <row r="337" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D337" s="2"/>
+      <c r="F337" s="2"/>
       <c r="G337" s="2"/>
-    </row>
-    <row r="338" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H337" s="2"/>
+    </row>
+    <row r="338" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D338" s="2"/>
+      <c r="F338" s="2"/>
       <c r="G338" s="2"/>
-    </row>
-    <row r="339" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H338" s="2"/>
+    </row>
+    <row r="339" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D339" s="2"/>
+      <c r="F339" s="2"/>
       <c r="G339" s="2"/>
-    </row>
-    <row r="340" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H339" s="2"/>
+    </row>
+    <row r="340" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D340" s="2"/>
+      <c r="F340" s="2"/>
       <c r="G340" s="2"/>
-    </row>
-    <row r="341" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H340" s="2"/>
+    </row>
+    <row r="341" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D341" s="2"/>
+      <c r="F341" s="2"/>
       <c r="G341" s="2"/>
-    </row>
-    <row r="342" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H341" s="2"/>
+    </row>
+    <row r="342" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D342" s="2"/>
+      <c r="F342" s="2"/>
       <c r="G342" s="2"/>
-    </row>
-    <row r="343" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H342" s="2"/>
+    </row>
+    <row r="343" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D343" s="2"/>
+      <c r="F343" s="2"/>
       <c r="G343" s="2"/>
-    </row>
-    <row r="344" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H343" s="2"/>
+    </row>
+    <row r="344" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D344" s="2"/>
+      <c r="F344" s="2"/>
       <c r="G344" s="2"/>
-    </row>
-    <row r="345" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H344" s="2"/>
+    </row>
+    <row r="345" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D345" s="2"/>
+      <c r="F345" s="2"/>
       <c r="G345" s="2"/>
-    </row>
-    <row r="346" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H345" s="2"/>
+    </row>
+    <row r="346" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D346" s="2"/>
+      <c r="F346" s="2"/>
       <c r="G346" s="2"/>
-    </row>
-    <row r="347" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H346" s="2"/>
+    </row>
+    <row r="347" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D347" s="2"/>
+      <c r="F347" s="2"/>
       <c r="G347" s="2"/>
-    </row>
-    <row r="348" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H347" s="2"/>
+    </row>
+    <row r="348" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D348" s="2"/>
+      <c r="F348" s="2"/>
       <c r="G348" s="2"/>
-    </row>
-    <row r="349" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H348" s="2"/>
+    </row>
+    <row r="349" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D349" s="2"/>
+      <c r="F349" s="2"/>
       <c r="G349" s="2"/>
-    </row>
-    <row r="350" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H349" s="2"/>
+    </row>
+    <row r="350" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D350" s="2"/>
+      <c r="F350" s="2"/>
       <c r="G350" s="2"/>
-    </row>
-    <row r="351" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H350" s="2"/>
+    </row>
+    <row r="351" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D351" s="2"/>
+      <c r="F351" s="2"/>
       <c r="G351" s="2"/>
-    </row>
-    <row r="352" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H351" s="2"/>
+    </row>
+    <row r="352" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D352" s="2"/>
+      <c r="F352" s="2"/>
       <c r="G352" s="2"/>
-    </row>
-    <row r="353" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H352" s="2"/>
+    </row>
+    <row r="353" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D353" s="2"/>
+      <c r="F353" s="2"/>
       <c r="G353" s="2"/>
-    </row>
-    <row r="354" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H353" s="2"/>
+    </row>
+    <row r="354" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D354" s="2"/>
+      <c r="F354" s="2"/>
       <c r="G354" s="2"/>
-    </row>
-    <row r="355" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H354" s="2"/>
+    </row>
+    <row r="355" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D355" s="2"/>
+      <c r="F355" s="2"/>
       <c r="G355" s="2"/>
-    </row>
-    <row r="356" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H355" s="2"/>
+    </row>
+    <row r="356" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D356" s="2"/>
+      <c r="F356" s="2"/>
       <c r="G356" s="2"/>
-    </row>
-    <row r="357" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H356" s="2"/>
+    </row>
+    <row r="357" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D357" s="2"/>
+      <c r="F357" s="2"/>
       <c r="G357" s="2"/>
-    </row>
-    <row r="358" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H357" s="2"/>
+    </row>
+    <row r="358" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D358" s="2"/>
+      <c r="F358" s="2"/>
       <c r="G358" s="2"/>
-    </row>
-    <row r="359" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H358" s="2"/>
+    </row>
+    <row r="359" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D359" s="2"/>
+      <c r="F359" s="2"/>
       <c r="G359" s="2"/>
-    </row>
-    <row r="360" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H359" s="2"/>
+    </row>
+    <row r="360" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D360" s="2"/>
+      <c r="F360" s="2"/>
       <c r="G360" s="2"/>
-    </row>
-    <row r="361" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H360" s="2"/>
+    </row>
+    <row r="361" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D361" s="2"/>
+      <c r="F361" s="2"/>
       <c r="G361" s="2"/>
-    </row>
-    <row r="362" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H361" s="2"/>
+    </row>
+    <row r="362" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D362" s="2"/>
+      <c r="F362" s="2"/>
       <c r="G362" s="2"/>
-    </row>
-    <row r="363" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H362" s="2"/>
+    </row>
+    <row r="363" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D363" s="2"/>
+      <c r="F363" s="2"/>
       <c r="G363" s="2"/>
-    </row>
-    <row r="364" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H363" s="2"/>
+    </row>
+    <row r="364" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D364" s="2"/>
+      <c r="F364" s="2"/>
       <c r="G364" s="2"/>
-    </row>
-    <row r="365" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H364" s="2"/>
+    </row>
+    <row r="365" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D365" s="2"/>
+      <c r="F365" s="2"/>
       <c r="G365" s="2"/>
-    </row>
-    <row r="366" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H365" s="2"/>
+    </row>
+    <row r="366" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D366" s="2"/>
+      <c r="F366" s="2"/>
       <c r="G366" s="2"/>
-    </row>
-    <row r="367" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H366" s="2"/>
+    </row>
+    <row r="367" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D367" s="2"/>
+      <c r="F367" s="2"/>
       <c r="G367" s="2"/>
-    </row>
-    <row r="368" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H367" s="2"/>
+    </row>
+    <row r="368" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D368" s="2"/>
+      <c r="F368" s="2"/>
       <c r="G368" s="2"/>
-    </row>
-    <row r="369" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H368" s="2"/>
+    </row>
+    <row r="369" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D369" s="2"/>
+      <c r="F369" s="2"/>
       <c r="G369" s="2"/>
-    </row>
-    <row r="370" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H369" s="2"/>
+    </row>
+    <row r="370" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D370" s="2"/>
+      <c r="F370" s="2"/>
       <c r="G370" s="2"/>
-    </row>
-    <row r="371" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H370" s="2"/>
+    </row>
+    <row r="371" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D371" s="2"/>
+      <c r="F371" s="2"/>
       <c r="G371" s="2"/>
-    </row>
-    <row r="372" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H371" s="2"/>
+    </row>
+    <row r="372" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D372" s="2"/>
+      <c r="F372" s="2"/>
       <c r="G372" s="2"/>
-    </row>
-    <row r="373" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H372" s="2"/>
+    </row>
+    <row r="373" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D373" s="2"/>
+      <c r="F373" s="2"/>
       <c r="G373" s="2"/>
-    </row>
-    <row r="374" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H373" s="2"/>
+    </row>
+    <row r="374" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D374" s="2"/>
+      <c r="F374" s="2"/>
       <c r="G374" s="2"/>
-    </row>
-    <row r="375" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H374" s="2"/>
+    </row>
+    <row r="375" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D375" s="2"/>
+      <c r="F375" s="2"/>
       <c r="G375" s="2"/>
-    </row>
-    <row r="376" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H375" s="2"/>
+    </row>
+    <row r="376" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D376" s="2"/>
+      <c r="F376" s="2"/>
       <c r="G376" s="2"/>
-    </row>
-    <row r="377" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H376" s="2"/>
+    </row>
+    <row r="377" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D377" s="2"/>
+      <c r="F377" s="2"/>
       <c r="G377" s="2"/>
-    </row>
-    <row r="378" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H377" s="2"/>
+    </row>
+    <row r="378" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D378" s="2"/>
+      <c r="F378" s="2"/>
       <c r="G378" s="2"/>
-    </row>
-    <row r="379" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H378" s="2"/>
+    </row>
+    <row r="379" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D379" s="2"/>
+      <c r="F379" s="2"/>
       <c r="G379" s="2"/>
-    </row>
-    <row r="380" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H379" s="2"/>
+    </row>
+    <row r="380" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D380" s="2"/>
+      <c r="F380" s="2"/>
       <c r="G380" s="2"/>
-    </row>
-    <row r="381" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H380" s="2"/>
+    </row>
+    <row r="381" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D381" s="2"/>
+      <c r="F381" s="2"/>
       <c r="G381" s="2"/>
-    </row>
-    <row r="382" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H381" s="2"/>
+    </row>
+    <row r="382" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D382" s="2"/>
+      <c r="F382" s="2"/>
       <c r="G382" s="2"/>
-    </row>
-    <row r="383" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H382" s="2"/>
+    </row>
+    <row r="383" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D383" s="2"/>
+      <c r="F383" s="2"/>
       <c r="G383" s="2"/>
-    </row>
-    <row r="384" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H383" s="2"/>
+    </row>
+    <row r="384" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D384" s="2"/>
+      <c r="F384" s="2"/>
       <c r="G384" s="2"/>
-    </row>
-    <row r="385" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H384" s="2"/>
+    </row>
+    <row r="385" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D385" s="2"/>
+      <c r="F385" s="2"/>
       <c r="G385" s="2"/>
-    </row>
-    <row r="386" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H385" s="2"/>
+    </row>
+    <row r="386" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D386" s="2"/>
+      <c r="F386" s="2"/>
       <c r="G386" s="2"/>
-    </row>
-    <row r="387" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H386" s="2"/>
+    </row>
+    <row r="387" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D387" s="2"/>
+      <c r="F387" s="2"/>
       <c r="G387" s="2"/>
-    </row>
-    <row r="388" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H387" s="2"/>
+    </row>
+    <row r="388" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D388" s="2"/>
+      <c r="F388" s="2"/>
       <c r="G388" s="2"/>
-    </row>
-    <row r="389" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H388" s="2"/>
+    </row>
+    <row r="389" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D389" s="2"/>
+      <c r="F389" s="2"/>
       <c r="G389" s="2"/>
-    </row>
-    <row r="390" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H389" s="2"/>
+    </row>
+    <row r="390" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D390" s="2"/>
+      <c r="F390" s="2"/>
       <c r="G390" s="2"/>
-    </row>
-    <row r="391" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H390" s="2"/>
+    </row>
+    <row r="391" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D391" s="2"/>
+      <c r="F391" s="2"/>
       <c r="G391" s="2"/>
-    </row>
-    <row r="392" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H391" s="2"/>
+    </row>
+    <row r="392" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D392" s="2"/>
+      <c r="F392" s="2"/>
       <c r="G392" s="2"/>
-    </row>
-    <row r="393" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H392" s="2"/>
+    </row>
+    <row r="393" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D393" s="2"/>
+      <c r="F393" s="2"/>
       <c r="G393" s="2"/>
-    </row>
-    <row r="394" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H393" s="2"/>
+    </row>
+    <row r="394" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D394" s="2"/>
+      <c r="F394" s="2"/>
       <c r="G394" s="2"/>
-    </row>
-    <row r="395" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H394" s="2"/>
+    </row>
+    <row r="395" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D395" s="2"/>
+      <c r="F395" s="2"/>
       <c r="G395" s="2"/>
-    </row>
-    <row r="396" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H395" s="2"/>
+    </row>
+    <row r="396" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D396" s="2"/>
+      <c r="F396" s="2"/>
       <c r="G396" s="2"/>
-    </row>
-    <row r="397" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H396" s="2"/>
+    </row>
+    <row r="397" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D397" s="2"/>
+      <c r="F397" s="2"/>
       <c r="G397" s="2"/>
-    </row>
-    <row r="398" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H397" s="2"/>
+    </row>
+    <row r="398" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D398" s="2"/>
+      <c r="F398" s="2"/>
       <c r="G398" s="2"/>
-    </row>
-    <row r="399" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H398" s="2"/>
+    </row>
+    <row r="399" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D399" s="2"/>
+      <c r="F399" s="2"/>
       <c r="G399" s="2"/>
-    </row>
-    <row r="400" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H399" s="2"/>
+    </row>
+    <row r="400" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D400" s="2"/>
+      <c r="F400" s="2"/>
       <c r="G400" s="2"/>
-    </row>
-    <row r="401" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H400" s="2"/>
+    </row>
+    <row r="401" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D401" s="2"/>
+      <c r="F401" s="2"/>
       <c r="G401" s="2"/>
-    </row>
-    <row r="402" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H401" s="2"/>
+    </row>
+    <row r="402" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D402" s="2"/>
+      <c r="F402" s="2"/>
       <c r="G402" s="2"/>
-    </row>
-    <row r="403" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H402" s="2"/>
+    </row>
+    <row r="403" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D403" s="2"/>
+      <c r="F403" s="2"/>
       <c r="G403" s="2"/>
-    </row>
-    <row r="404" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H403" s="2"/>
+    </row>
+    <row r="404" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D404" s="2"/>
+      <c r="F404" s="2"/>
       <c r="G404" s="2"/>
-    </row>
-    <row r="405" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H404" s="2"/>
+    </row>
+    <row r="405" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D405" s="2"/>
+      <c r="F405" s="2"/>
       <c r="G405" s="2"/>
-    </row>
-    <row r="406" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H405" s="2"/>
+    </row>
+    <row r="406" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D406" s="2"/>
+      <c r="F406" s="2"/>
       <c r="G406" s="2"/>
-    </row>
-    <row r="407" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H406" s="2"/>
+    </row>
+    <row r="407" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D407" s="2"/>
+      <c r="F407" s="2"/>
       <c r="G407" s="2"/>
-    </row>
-    <row r="408" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H407" s="2"/>
+    </row>
+    <row r="408" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D408" s="2"/>
+      <c r="F408" s="2"/>
       <c r="G408" s="2"/>
-    </row>
-    <row r="409" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H408" s="2"/>
+    </row>
+    <row r="409" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D409" s="2"/>
+      <c r="F409" s="2"/>
       <c r="G409" s="2"/>
-    </row>
-    <row r="410" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H409" s="2"/>
+    </row>
+    <row r="410" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D410" s="2"/>
+      <c r="F410" s="2"/>
       <c r="G410" s="2"/>
-    </row>
-    <row r="411" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H410" s="2"/>
+    </row>
+    <row r="411" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D411" s="2"/>
+      <c r="F411" s="2"/>
       <c r="G411" s="2"/>
-    </row>
-    <row r="412" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H411" s="2"/>
+    </row>
+    <row r="412" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D412" s="2"/>
+      <c r="F412" s="2"/>
       <c r="G412" s="2"/>
-    </row>
-    <row r="413" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H412" s="2"/>
+    </row>
+    <row r="413" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D413" s="2"/>
+      <c r="F413" s="2"/>
       <c r="G413" s="2"/>
-    </row>
-    <row r="414" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H413" s="2"/>
+    </row>
+    <row r="414" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D414" s="2"/>
+      <c r="F414" s="2"/>
       <c r="G414" s="2"/>
-    </row>
-    <row r="415" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H414" s="2"/>
+    </row>
+    <row r="415" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D415" s="2"/>
+      <c r="F415" s="2"/>
       <c r="G415" s="2"/>
-    </row>
-    <row r="416" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H415" s="2"/>
+    </row>
+    <row r="416" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D416" s="2"/>
+      <c r="F416" s="2"/>
       <c r="G416" s="2"/>
-    </row>
-    <row r="417" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H416" s="2"/>
+    </row>
+    <row r="417" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D417" s="2"/>
+      <c r="F417" s="2"/>
       <c r="G417" s="2"/>
-    </row>
-    <row r="418" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H417" s="2"/>
+    </row>
+    <row r="418" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D418" s="2"/>
+      <c r="F418" s="2"/>
       <c r="G418" s="2"/>
-    </row>
-    <row r="419" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H418" s="2"/>
+    </row>
+    <row r="419" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D419" s="2"/>
+      <c r="F419" s="2"/>
       <c r="G419" s="2"/>
-    </row>
-    <row r="420" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H419" s="2"/>
+    </row>
+    <row r="420" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D420" s="2"/>
+      <c r="F420" s="2"/>
       <c r="G420" s="2"/>
-    </row>
-    <row r="421" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H420" s="2"/>
+    </row>
+    <row r="421" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D421" s="2"/>
+      <c r="F421" s="2"/>
       <c r="G421" s="2"/>
-    </row>
-    <row r="422" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H421" s="2"/>
+    </row>
+    <row r="422" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D422" s="2"/>
+      <c r="F422" s="2"/>
       <c r="G422" s="2"/>
-    </row>
-    <row r="423" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H422" s="2"/>
+    </row>
+    <row r="423" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D423" s="2"/>
+      <c r="F423" s="2"/>
       <c r="G423" s="2"/>
-    </row>
-    <row r="424" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H423" s="2"/>
+    </row>
+    <row r="424" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D424" s="2"/>
+      <c r="F424" s="2"/>
       <c r="G424" s="2"/>
-    </row>
-    <row r="425" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H424" s="2"/>
+    </row>
+    <row r="425" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D425" s="2"/>
+      <c r="F425" s="2"/>
       <c r="G425" s="2"/>
-    </row>
-    <row r="426" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H425" s="2"/>
+    </row>
+    <row r="426" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D426" s="2"/>
+      <c r="F426" s="2"/>
       <c r="G426" s="2"/>
-    </row>
-    <row r="427" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H426" s="2"/>
+    </row>
+    <row r="427" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D427" s="2"/>
+      <c r="F427" s="2"/>
       <c r="G427" s="2"/>
-    </row>
-    <row r="428" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H427" s="2"/>
+    </row>
+    <row r="428" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D428" s="2"/>
+      <c r="F428" s="2"/>
       <c r="G428" s="2"/>
-    </row>
-    <row r="429" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H428" s="2"/>
+    </row>
+    <row r="429" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D429" s="2"/>
+      <c r="F429" s="2"/>
       <c r="G429" s="2"/>
-    </row>
-    <row r="430" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H429" s="2"/>
+    </row>
+    <row r="430" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D430" s="2"/>
+      <c r="F430" s="2"/>
       <c r="G430" s="2"/>
-    </row>
-    <row r="431" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H430" s="2"/>
+    </row>
+    <row r="431" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D431" s="2"/>
+      <c r="F431" s="2"/>
       <c r="G431" s="2"/>
-    </row>
-    <row r="432" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H431" s="2"/>
+    </row>
+    <row r="432" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D432" s="2"/>
+      <c r="F432" s="2"/>
       <c r="G432" s="2"/>
-    </row>
-    <row r="433" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H432" s="2"/>
+    </row>
+    <row r="433" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D433" s="2"/>
+      <c r="F433" s="2"/>
       <c r="G433" s="2"/>
-    </row>
-    <row r="434" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H433" s="2"/>
+    </row>
+    <row r="434" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D434" s="2"/>
+      <c r="F434" s="2"/>
       <c r="G434" s="2"/>
-    </row>
-    <row r="435" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H434" s="2"/>
+    </row>
+    <row r="435" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D435" s="2"/>
+      <c r="F435" s="2"/>
       <c r="G435" s="2"/>
-    </row>
-    <row r="436" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H435" s="2"/>
+    </row>
+    <row r="436" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D436" s="2"/>
+      <c r="F436" s="2"/>
       <c r="G436" s="2"/>
-    </row>
-    <row r="437" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H436" s="2"/>
+    </row>
+    <row r="437" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D437" s="2"/>
+      <c r="F437" s="2"/>
       <c r="G437" s="2"/>
-    </row>
-    <row r="438" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H437" s="2"/>
+    </row>
+    <row r="438" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D438" s="2"/>
+      <c r="F438" s="2"/>
       <c r="G438" s="2"/>
-    </row>
-    <row r="439" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H438" s="2"/>
+    </row>
+    <row r="439" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D439" s="2"/>
+      <c r="F439" s="2"/>
       <c r="G439" s="2"/>
-    </row>
-    <row r="440" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H439" s="2"/>
+    </row>
+    <row r="440" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D440" s="2"/>
+      <c r="F440" s="2"/>
       <c r="G440" s="2"/>
-    </row>
-    <row r="441" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H440" s="2"/>
+    </row>
+    <row r="441" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D441" s="2"/>
+      <c r="F441" s="2"/>
       <c r="G441" s="2"/>
-    </row>
-    <row r="442" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H441" s="2"/>
+    </row>
+    <row r="442" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D442" s="2"/>
+      <c r="F442" s="2"/>
       <c r="G442" s="2"/>
-    </row>
-    <row r="443" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H442" s="2"/>
+    </row>
+    <row r="443" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D443" s="2"/>
+      <c r="F443" s="2"/>
       <c r="G443" s="2"/>
-    </row>
-    <row r="444" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H443" s="2"/>
+    </row>
+    <row r="444" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D444" s="2"/>
+      <c r="F444" s="2"/>
       <c r="G444" s="2"/>
-    </row>
-    <row r="445" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H444" s="2"/>
+    </row>
+    <row r="445" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D445" s="2"/>
+      <c r="F445" s="2"/>
       <c r="G445" s="2"/>
-    </row>
-    <row r="446" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H445" s="2"/>
+    </row>
+    <row r="446" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D446" s="2"/>
+      <c r="F446" s="2"/>
       <c r="G446" s="2"/>
-    </row>
-    <row r="447" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H446" s="2"/>
+    </row>
+    <row r="447" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D447" s="2"/>
+      <c r="F447" s="2"/>
       <c r="G447" s="2"/>
-    </row>
-    <row r="448" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H447" s="2"/>
+    </row>
+    <row r="448" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D448" s="2"/>
+      <c r="F448" s="2"/>
       <c r="G448" s="2"/>
-    </row>
-    <row r="449" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H448" s="2"/>
+    </row>
+    <row r="449" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D449" s="2"/>
+      <c r="F449" s="2"/>
       <c r="G449" s="2"/>
-    </row>
-    <row r="450" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H449" s="2"/>
+    </row>
+    <row r="450" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D450" s="2"/>
+      <c r="F450" s="2"/>
       <c r="G450" s="2"/>
-    </row>
-    <row r="451" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H450" s="2"/>
+    </row>
+    <row r="451" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D451" s="2"/>
+      <c r="F451" s="2"/>
       <c r="G451" s="2"/>
-    </row>
-    <row r="452" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H451" s="2"/>
+    </row>
+    <row r="452" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D452" s="2"/>
+      <c r="F452" s="2"/>
       <c r="G452" s="2"/>
-    </row>
-    <row r="453" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H452" s="2"/>
+    </row>
+    <row r="453" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D453" s="2"/>
+      <c r="F453" s="2"/>
       <c r="G453" s="2"/>
-    </row>
-    <row r="454" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H453" s="2"/>
+    </row>
+    <row r="454" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D454" s="2"/>
+      <c r="F454" s="2"/>
       <c r="G454" s="2"/>
-    </row>
-    <row r="455" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H454" s="2"/>
+    </row>
+    <row r="455" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D455" s="2"/>
+      <c r="F455" s="2"/>
       <c r="G455" s="2"/>
-    </row>
-    <row r="456" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H455" s="2"/>
+    </row>
+    <row r="456" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D456" s="2"/>
+      <c r="F456" s="2"/>
       <c r="G456" s="2"/>
-    </row>
-    <row r="457" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H456" s="2"/>
+    </row>
+    <row r="457" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D457" s="2"/>
+      <c r="F457" s="2"/>
       <c r="G457" s="2"/>
-    </row>
-    <row r="458" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H457" s="2"/>
+    </row>
+    <row r="458" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D458" s="2"/>
+      <c r="F458" s="2"/>
       <c r="G458" s="2"/>
-    </row>
-    <row r="459" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H458" s="2"/>
+    </row>
+    <row r="459" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D459" s="2"/>
+      <c r="F459" s="2"/>
       <c r="G459" s="2"/>
-    </row>
-    <row r="460" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H459" s="2"/>
+    </row>
+    <row r="460" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D460" s="2"/>
+      <c r="F460" s="2"/>
       <c r="G460" s="2"/>
-    </row>
-    <row r="461" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H460" s="2"/>
+    </row>
+    <row r="461" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D461" s="2"/>
+      <c r="F461" s="2"/>
       <c r="G461" s="2"/>
-    </row>
-    <row r="462" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H461" s="2"/>
+    </row>
+    <row r="462" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D462" s="2"/>
+      <c r="F462" s="2"/>
       <c r="G462" s="2"/>
-    </row>
-    <row r="463" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H462" s="2"/>
+    </row>
+    <row r="463" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D463" s="2"/>
+      <c r="F463" s="2"/>
       <c r="G463" s="2"/>
-    </row>
-    <row r="464" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H463" s="2"/>
+    </row>
+    <row r="464" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D464" s="2"/>
+      <c r="F464" s="2"/>
       <c r="G464" s="2"/>
-    </row>
-    <row r="465" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H464" s="2"/>
+    </row>
+    <row r="465" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D465" s="2"/>
+      <c r="F465" s="2"/>
       <c r="G465" s="2"/>
-    </row>
-    <row r="466" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H465" s="2"/>
+    </row>
+    <row r="466" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D466" s="2"/>
+      <c r="F466" s="2"/>
       <c r="G466" s="2"/>
-    </row>
-    <row r="467" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H466" s="2"/>
+    </row>
+    <row r="467" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D467" s="2"/>
+      <c r="F467" s="2"/>
       <c r="G467" s="2"/>
-    </row>
-    <row r="468" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H467" s="2"/>
+    </row>
+    <row r="468" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D468" s="2"/>
+      <c r="F468" s="2"/>
       <c r="G468" s="2"/>
-    </row>
-    <row r="469" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H468" s="2"/>
+    </row>
+    <row r="469" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D469" s="2"/>
+      <c r="F469" s="2"/>
       <c r="G469" s="2"/>
-    </row>
-    <row r="470" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H469" s="2"/>
+    </row>
+    <row r="470" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D470" s="2"/>
+      <c r="F470" s="2"/>
       <c r="G470" s="2"/>
-    </row>
-    <row r="471" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H470" s="2"/>
+    </row>
+    <row r="471" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D471" s="2"/>
+      <c r="F471" s="2"/>
       <c r="G471" s="2"/>
-    </row>
-    <row r="472" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H471" s="2"/>
+    </row>
+    <row r="472" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D472" s="2"/>
+      <c r="F472" s="2"/>
       <c r="G472" s="2"/>
-    </row>
-    <row r="473" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H472" s="2"/>
+    </row>
+    <row r="473" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D473" s="2"/>
+      <c r="F473" s="2"/>
       <c r="G473" s="2"/>
-    </row>
-    <row r="474" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H473" s="2"/>
+    </row>
+    <row r="474" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D474" s="2"/>
+      <c r="F474" s="2"/>
       <c r="G474" s="2"/>
-    </row>
-    <row r="475" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H474" s="2"/>
+    </row>
+    <row r="475" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D475" s="2"/>
+      <c r="F475" s="2"/>
       <c r="G475" s="2"/>
-    </row>
-    <row r="476" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H475" s="2"/>
+    </row>
+    <row r="476" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D476" s="2"/>
+      <c r="F476" s="2"/>
       <c r="G476" s="2"/>
-    </row>
-    <row r="477" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H476" s="2"/>
+    </row>
+    <row r="477" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D477" s="2"/>
+      <c r="F477" s="2"/>
       <c r="G477" s="2"/>
-    </row>
-    <row r="478" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H477" s="2"/>
+    </row>
+    <row r="478" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D478" s="2"/>
+      <c r="F478" s="2"/>
       <c r="G478" s="2"/>
-    </row>
-    <row r="479" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H478" s="2"/>
+    </row>
+    <row r="479" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D479" s="2"/>
+      <c r="F479" s="2"/>
       <c r="G479" s="2"/>
-    </row>
-    <row r="480" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H479" s="2"/>
+    </row>
+    <row r="480" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D480" s="2"/>
+      <c r="F480" s="2"/>
       <c r="G480" s="2"/>
-    </row>
-    <row r="481" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H480" s="2"/>
+    </row>
+    <row r="481" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D481" s="2"/>
+      <c r="F481" s="2"/>
       <c r="G481" s="2"/>
-    </row>
-    <row r="482" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H481" s="2"/>
+    </row>
+    <row r="482" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D482" s="2"/>
+      <c r="F482" s="2"/>
       <c r="G482" s="2"/>
-    </row>
-    <row r="483" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H482" s="2"/>
+    </row>
+    <row r="483" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D483" s="2"/>
+      <c r="F483" s="2"/>
       <c r="G483" s="2"/>
-    </row>
-    <row r="484" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H483" s="2"/>
+    </row>
+    <row r="484" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D484" s="2"/>
+      <c r="F484" s="2"/>
       <c r="G484" s="2"/>
-    </row>
-    <row r="485" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H484" s="2"/>
+    </row>
+    <row r="485" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D485" s="2"/>
+      <c r="F485" s="2"/>
       <c r="G485" s="2"/>
-    </row>
-    <row r="486" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H485" s="2"/>
+    </row>
+    <row r="486" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D486" s="2"/>
+      <c r="F486" s="2"/>
       <c r="G486" s="2"/>
-    </row>
-    <row r="487" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H486" s="2"/>
+    </row>
+    <row r="487" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D487" s="2"/>
+      <c r="F487" s="2"/>
       <c r="G487" s="2"/>
-    </row>
-    <row r="488" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H487" s="2"/>
+    </row>
+    <row r="488" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D488" s="2"/>
+      <c r="F488" s="2"/>
       <c r="G488" s="2"/>
-    </row>
-    <row r="489" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H488" s="2"/>
+    </row>
+    <row r="489" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D489" s="2"/>
+      <c r="F489" s="2"/>
       <c r="G489" s="2"/>
-    </row>
-    <row r="490" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H489" s="2"/>
+    </row>
+    <row r="490" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D490" s="2"/>
+      <c r="F490" s="2"/>
       <c r="G490" s="2"/>
-    </row>
-    <row r="491" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H490" s="2"/>
+    </row>
+    <row r="491" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D491" s="2"/>
+      <c r="F491" s="2"/>
       <c r="G491" s="2"/>
-    </row>
-    <row r="492" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H491" s="2"/>
+    </row>
+    <row r="492" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D492" s="2"/>
+      <c r="F492" s="2"/>
       <c r="G492" s="2"/>
-    </row>
-    <row r="493" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H492" s="2"/>
+    </row>
+    <row r="493" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D493" s="2"/>
+      <c r="F493" s="2"/>
       <c r="G493" s="2"/>
-    </row>
-    <row r="494" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H493" s="2"/>
+    </row>
+    <row r="494" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D494" s="2"/>
+      <c r="F494" s="2"/>
       <c r="G494" s="2"/>
-    </row>
-    <row r="495" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H494" s="2"/>
+    </row>
+    <row r="495" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D495" s="2"/>
+      <c r="F495" s="2"/>
       <c r="G495" s="2"/>
-    </row>
-    <row r="496" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H495" s="2"/>
+    </row>
+    <row r="496" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D496" s="2"/>
+      <c r="F496" s="2"/>
       <c r="G496" s="2"/>
-    </row>
-    <row r="497" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H496" s="2"/>
+    </row>
+    <row r="497" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D497" s="2"/>
+      <c r="F497" s="2"/>
       <c r="G497" s="2"/>
-    </row>
-    <row r="498" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H497" s="2"/>
+    </row>
+    <row r="498" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D498" s="2"/>
+      <c r="F498" s="2"/>
       <c r="G498" s="2"/>
-    </row>
-    <row r="499" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H498" s="2"/>
+    </row>
+    <row r="499" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D499" s="2"/>
+      <c r="F499" s="2"/>
       <c r="G499" s="2"/>
-    </row>
-    <row r="500" spans="4:7" x14ac:dyDescent="0.25">
+      <c r="H499" s="2"/>
+    </row>
+    <row r="500" spans="4:8" x14ac:dyDescent="0.25">
       <c r="D500" s="2"/>
+      <c r="F500" s="2"/>
       <c r="G500" s="2"/>
+      <c r="H500" s="2"/>
     </row>
   </sheetData>
   <dataValidations count="2">
@@ -3275,42 +4292,42 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>
@@ -3321,7 +4338,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A39"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="140" customWidth="1"/>
@@ -3329,92 +4346,197 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>140</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Treatments: update Co2 content from spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/content/treatments.xlsx
+++ b/src/content/treatments.xlsx
@@ -1,19 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30602"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="11_CD8CFCFBC2BCBCE8A5A932D356D42070557EB562" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B41ED63-4E26-40D8-95A5-A9436EBD30BA}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Treatments" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="Treatment Types" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="Instructions" state="visible" r:id="rId6"/>
+    <sheet name="Treatments" sheetId="1" r:id="rId1"/>
+    <sheet name="Treatment Types" sheetId="2" r:id="rId2"/>
+    <sheet name="Instructions" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191028"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="149">
   <si>
     <t>Title</t>
   </si>
@@ -309,7 +329,16 @@
     <t>co2</t>
   </si>
   <si>
-    <t>Irure dolor in reprehenderit in voluptate velit esse cillum dolore eu fugiat nulla pariatur lorem ipsum dolor sit amet consectetur adipiscing.</t>
+    <t>The effects of CO2 laser include improved skin texture, reduced wrinkles and scars, enhanced skin firmness, and overall skin rejuvenation.</t>
+  </si>
+  <si>
+    <t>It treats wrinkles, fine lines, acne scars, sun damage, and uneven skin tone.</t>
+  </si>
+  <si>
+    <t>Benefits include improved skin texture, reduced wrinkles and scars, skin tightening, and overall rejuvenation.</t>
+  </si>
+  <si>
+    <t>CO2 laser works by emitting a concentrated beam of carbon dioxide light to vaporize the top layers of skin, promoting collagen production and skin resurfacing.</t>
   </si>
   <si>
     <t>Miim Laser</t>
@@ -456,21 +485,24 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
       <b/>
-    </font>
-    <font>
-      <b/>
       <sz val="14"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -493,13 +525,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -838,9 +876,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:H500"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
@@ -851,3696 +889,3742 @@
     <col min="8" max="8" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:8" s="1" customFormat="1">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" ht="45.75">
+      <c r="A2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
       </c>
+      <c r="E2" s="5"/>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="3" spans="1:8" ht="45.75">
+      <c r="A3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C3" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="E3" s="5"/>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:8" ht="45.75">
+      <c r="A4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C4" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>17</v>
       </c>
+      <c r="E4" s="5"/>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="5" spans="1:8" ht="45.75">
+      <c r="A5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C5" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="E5" s="5"/>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="6" spans="1:8" ht="45.75">
+      <c r="A6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>23</v>
       </c>
+      <c r="E6" s="5"/>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:8" ht="45.75">
+      <c r="A7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D7" s="2" t="s">
         <v>26</v>
       </c>
+      <c r="E7" s="5"/>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:8" ht="45.75">
+      <c r="A8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>30</v>
       </c>
+      <c r="E8" s="5"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:8" ht="45.75">
+      <c r="A9" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>33</v>
       </c>
+      <c r="E9" s="5"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:8" ht="45.75">
+      <c r="A10" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>36</v>
       </c>
+      <c r="E10" s="5"/>
       <c r="F10" s="2"/>
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:8" ht="30.75">
+      <c r="A11" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>39</v>
       </c>
+      <c r="E11" s="5"/>
       <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:8" ht="45.75">
+      <c r="A12" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>42</v>
       </c>
+      <c r="E12" s="5"/>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:8" ht="45.75">
+      <c r="A13" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>45</v>
       </c>
+      <c r="E13" s="5"/>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:8" ht="45.75">
+      <c r="A14" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>48</v>
       </c>
+      <c r="E14" s="5"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:8" ht="45.75">
+      <c r="A15" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>51</v>
       </c>
+      <c r="E15" s="5"/>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:8" ht="45.75">
+      <c r="A16" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>54</v>
       </c>
+      <c r="E16" s="5"/>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:8" ht="45.75">
+      <c r="A17" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>58</v>
       </c>
+      <c r="E17" s="5"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:8" ht="45.75">
+      <c r="A18" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>61</v>
       </c>
+      <c r="E18" s="5"/>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:8" ht="45.75">
+      <c r="A19" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>63</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>64</v>
       </c>
+      <c r="E19" s="5"/>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:8" ht="45.75">
+      <c r="A20" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>67</v>
       </c>
+      <c r="E20" s="5"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:8" ht="45.75">
+      <c r="A21" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>70</v>
       </c>
+      <c r="E21" s="5"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:8" ht="30.75">
+      <c r="A22" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>73</v>
       </c>
+      <c r="E22" s="5"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:8" ht="45.75">
+      <c r="A23" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>76</v>
       </c>
+      <c r="E23" s="5"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:8" ht="45.75">
+      <c r="A24" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>79</v>
       </c>
+      <c r="E24" s="5"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:8" ht="45.75">
+      <c r="A25" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D25" s="2" t="s">
         <v>82</v>
       </c>
+      <c r="E25" s="5"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:8" ht="45.75">
+      <c r="A26" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>86</v>
       </c>
+      <c r="E26" s="5"/>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
       <c r="H26" s="2"/>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:8" ht="30.75">
+      <c r="A27" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D27" s="2" t="s">
         <v>89</v>
       </c>
+      <c r="E27" s="5"/>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
       <c r="H27" s="2"/>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:8" ht="45.75">
+      <c r="A28" s="5" t="s">
         <v>90</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>92</v>
       </c>
+      <c r="E28" s="5"/>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2"/>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:8" ht="45.75">
+      <c r="A29" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="5" t="s">
         <v>85</v>
       </c>
       <c r="D29" s="2" t="s">
         <v>95</v>
       </c>
+      <c r="E29" s="5"/>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2"/>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:8" ht="45.75">
+      <c r="A30" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F30" s="2"/>
-      <c r="G30" s="2"/>
-      <c r="H30" s="2"/>
-    </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="E30" s="5"/>
+      <c r="F30" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B31" t="s">
+      <c r="G30" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="C31" t="s">
+      <c r="H30" s="2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8" ht="45.75">
+      <c r="A31" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>103</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>101</v>
-      </c>
+        <v>104</v>
+      </c>
+      <c r="E31" s="5"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>102</v>
-      </c>
-      <c r="B32" t="s">
-        <v>103</v>
-      </c>
-      <c r="C32" t="s">
+    <row r="32" spans="1:8" ht="45.75">
+      <c r="A32" s="5" t="s">
+        <v>105</v>
+      </c>
+      <c r="B32" s="5" t="s">
+        <v>106</v>
+      </c>
+      <c r="C32" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>104</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="E32" s="5"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
       <c r="H32" s="2"/>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>105</v>
-      </c>
-      <c r="B33" t="s">
-        <v>106</v>
-      </c>
-      <c r="C33" t="s">
+    <row r="33" spans="1:8" ht="45.75">
+      <c r="A33" s="5" t="s">
+        <v>108</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>109</v>
+      </c>
+      <c r="C33" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>107</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="E33" s="5"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>108</v>
-      </c>
-      <c r="B34" t="s">
-        <v>109</v>
-      </c>
-      <c r="C34" t="s">
+    <row r="34" spans="1:8" ht="45.75">
+      <c r="A34" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="B34" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="C34" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D34" s="2" t="s">
-        <v>110</v>
-      </c>
+        <v>113</v>
+      </c>
+      <c r="E34" s="5"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>111</v>
-      </c>
-      <c r="B35" t="s">
-        <v>112</v>
-      </c>
-      <c r="C35" t="s">
+    <row r="35" spans="1:8" ht="45.75">
+      <c r="A35" s="5" t="s">
+        <v>114</v>
+      </c>
+      <c r="B35" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="C35" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>113</v>
-      </c>
+        <v>116</v>
+      </c>
+      <c r="E35" s="5"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>114</v>
-      </c>
-      <c r="B36" t="s">
-        <v>115</v>
-      </c>
-      <c r="C36" t="s">
+    <row r="36" spans="1:8" ht="45.75">
+      <c r="A36" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="B36" s="5" t="s">
+        <v>118</v>
+      </c>
+      <c r="C36" s="5" t="s">
         <v>57</v>
       </c>
       <c r="D36" s="2" t="s">
-        <v>116</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="E36" s="5"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>117</v>
-      </c>
-      <c r="B37" t="s">
-        <v>118</v>
-      </c>
-      <c r="C37" t="s">
+    <row r="37" spans="1:8" ht="45.75">
+      <c r="A37" s="5" t="s">
+        <v>120</v>
+      </c>
+      <c r="B37" s="5" t="s">
+        <v>121</v>
+      </c>
+      <c r="C37" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>119</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="E37" s="5"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
     </row>
-    <row r="38" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8">
       <c r="D38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
       <c r="H38" s="2"/>
     </row>
-    <row r="39" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8">
       <c r="D39" s="2"/>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
       <c r="H39" s="2"/>
     </row>
-    <row r="40" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8">
       <c r="D40" s="2"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
       <c r="H40" s="2"/>
     </row>
-    <row r="41" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8">
       <c r="D41" s="2"/>
       <c r="F41" s="2"/>
       <c r="G41" s="2"/>
       <c r="H41" s="2"/>
     </row>
-    <row r="42" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8">
       <c r="D42" s="2"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
       <c r="H42" s="2"/>
     </row>
-    <row r="43" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8">
       <c r="D43" s="2"/>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
       <c r="H43" s="2"/>
     </row>
-    <row r="44" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8">
       <c r="D44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
       <c r="H44" s="2"/>
     </row>
-    <row r="45" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8">
       <c r="D45" s="2"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
       <c r="H45" s="2"/>
     </row>
-    <row r="46" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8">
       <c r="D46" s="2"/>
       <c r="F46" s="2"/>
       <c r="G46" s="2"/>
       <c r="H46" s="2"/>
     </row>
-    <row r="47" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8">
       <c r="D47" s="2"/>
       <c r="F47" s="2"/>
       <c r="G47" s="2"/>
       <c r="H47" s="2"/>
     </row>
-    <row r="48" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8">
       <c r="D48" s="2"/>
       <c r="F48" s="2"/>
       <c r="G48" s="2"/>
       <c r="H48" s="2"/>
     </row>
-    <row r="49" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="4:8">
       <c r="D49" s="2"/>
       <c r="F49" s="2"/>
       <c r="G49" s="2"/>
       <c r="H49" s="2"/>
     </row>
-    <row r="50" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="4:8">
       <c r="D50" s="2"/>
       <c r="F50" s="2"/>
       <c r="G50" s="2"/>
       <c r="H50" s="2"/>
     </row>
-    <row r="51" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="51" spans="4:8">
       <c r="D51" s="2"/>
       <c r="F51" s="2"/>
       <c r="G51" s="2"/>
       <c r="H51" s="2"/>
     </row>
-    <row r="52" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="52" spans="4:8">
       <c r="D52" s="2"/>
       <c r="F52" s="2"/>
       <c r="G52" s="2"/>
       <c r="H52" s="2"/>
     </row>
-    <row r="53" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="53" spans="4:8">
       <c r="D53" s="2"/>
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
       <c r="H53" s="2"/>
     </row>
-    <row r="54" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="54" spans="4:8">
       <c r="D54" s="2"/>
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
       <c r="H54" s="2"/>
     </row>
-    <row r="55" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="4:8">
       <c r="D55" s="2"/>
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
       <c r="H55" s="2"/>
     </row>
-    <row r="56" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="4:8">
       <c r="D56" s="2"/>
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
       <c r="H56" s="2"/>
     </row>
-    <row r="57" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="4:8">
       <c r="D57" s="2"/>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
       <c r="H57" s="2"/>
     </row>
-    <row r="58" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="4:8">
       <c r="D58" s="2"/>
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
       <c r="H58" s="2"/>
     </row>
-    <row r="59" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="4:8">
       <c r="D59" s="2"/>
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
       <c r="H59" s="2"/>
     </row>
-    <row r="60" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="60" spans="4:8">
       <c r="D60" s="2"/>
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
       <c r="H60" s="2"/>
     </row>
-    <row r="61" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="61" spans="4:8">
       <c r="D61" s="2"/>
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
       <c r="H61" s="2"/>
     </row>
-    <row r="62" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="62" spans="4:8">
       <c r="D62" s="2"/>
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
       <c r="H62" s="2"/>
     </row>
-    <row r="63" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="63" spans="4:8">
       <c r="D63" s="2"/>
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
       <c r="H63" s="2"/>
     </row>
-    <row r="64" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="4:8">
       <c r="D64" s="2"/>
       <c r="F64" s="2"/>
       <c r="G64" s="2"/>
       <c r="H64" s="2"/>
     </row>
-    <row r="65" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="4:8">
       <c r="D65" s="2"/>
       <c r="F65" s="2"/>
       <c r="G65" s="2"/>
       <c r="H65" s="2"/>
     </row>
-    <row r="66" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="4:8">
       <c r="D66" s="2"/>
       <c r="F66" s="2"/>
       <c r="G66" s="2"/>
       <c r="H66" s="2"/>
     </row>
-    <row r="67" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="67" spans="4:8">
       <c r="D67" s="2"/>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
       <c r="H67" s="2"/>
     </row>
-    <row r="68" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="68" spans="4:8">
       <c r="D68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
       <c r="H68" s="2"/>
     </row>
-    <row r="69" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="69" spans="4:8">
       <c r="D69" s="2"/>
       <c r="F69" s="2"/>
       <c r="G69" s="2"/>
       <c r="H69" s="2"/>
     </row>
-    <row r="70" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="70" spans="4:8">
       <c r="D70" s="2"/>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
       <c r="H70" s="2"/>
     </row>
-    <row r="71" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="4:8">
       <c r="D71" s="2"/>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
       <c r="H71" s="2"/>
     </row>
-    <row r="72" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="4:8">
       <c r="D72" s="2"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
       <c r="H72" s="2"/>
     </row>
-    <row r="73" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="4:8">
       <c r="D73" s="2"/>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
     </row>
-    <row r="74" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="74" spans="4:8">
       <c r="D74" s="2"/>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
     </row>
-    <row r="75" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="75" spans="4:8">
       <c r="D75" s="2"/>
       <c r="F75" s="2"/>
       <c r="G75" s="2"/>
       <c r="H75" s="2"/>
     </row>
-    <row r="76" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="76" spans="4:8">
       <c r="D76" s="2"/>
       <c r="F76" s="2"/>
       <c r="G76" s="2"/>
       <c r="H76" s="2"/>
     </row>
-    <row r="77" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="77" spans="4:8">
       <c r="D77" s="2"/>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
     </row>
-    <row r="78" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="4:8">
       <c r="D78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
     </row>
-    <row r="79" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="4:8">
       <c r="D79" s="2"/>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
     </row>
-    <row r="80" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="80" spans="4:8">
       <c r="D80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
     </row>
-    <row r="81" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="81" spans="4:8">
       <c r="D81" s="2"/>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
     </row>
-    <row r="82" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="82" spans="4:8">
       <c r="D82" s="2"/>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
       <c r="H82" s="2"/>
     </row>
-    <row r="83" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="83" spans="4:8">
       <c r="D83" s="2"/>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
     </row>
-    <row r="84" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="4:8">
       <c r="D84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
     </row>
-    <row r="85" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="85" spans="4:8">
       <c r="D85" s="2"/>
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
     </row>
-    <row r="86" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="86" spans="4:8">
       <c r="D86" s="2"/>
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
     </row>
-    <row r="87" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="87" spans="4:8">
       <c r="D87" s="2"/>
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
     </row>
-    <row r="88" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="88" spans="4:8">
       <c r="D88" s="2"/>
       <c r="F88" s="2"/>
       <c r="G88" s="2"/>
       <c r="H88" s="2"/>
     </row>
-    <row r="89" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="89" spans="4:8">
       <c r="D89" s="2"/>
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
     </row>
-    <row r="90" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="90" spans="4:8">
       <c r="D90" s="2"/>
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
     </row>
-    <row r="91" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="91" spans="4:8">
       <c r="D91" s="2"/>
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
     </row>
-    <row r="92" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="92" spans="4:8">
       <c r="D92" s="2"/>
       <c r="F92" s="2"/>
       <c r="G92" s="2"/>
       <c r="H92" s="2"/>
     </row>
-    <row r="93" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="93" spans="4:8">
       <c r="D93" s="2"/>
       <c r="F93" s="2"/>
       <c r="G93" s="2"/>
       <c r="H93" s="2"/>
     </row>
-    <row r="94" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="94" spans="4:8">
       <c r="D94" s="2"/>
       <c r="F94" s="2"/>
       <c r="G94" s="2"/>
       <c r="H94" s="2"/>
     </row>
-    <row r="95" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="95" spans="4:8">
       <c r="D95" s="2"/>
       <c r="F95" s="2"/>
       <c r="G95" s="2"/>
       <c r="H95" s="2"/>
     </row>
-    <row r="96" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="96" spans="4:8">
       <c r="D96" s="2"/>
       <c r="F96" s="2"/>
       <c r="G96" s="2"/>
       <c r="H96" s="2"/>
     </row>
-    <row r="97" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="97" spans="4:8">
       <c r="D97" s="2"/>
       <c r="F97" s="2"/>
       <c r="G97" s="2"/>
       <c r="H97" s="2"/>
     </row>
-    <row r="98" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="98" spans="4:8">
       <c r="D98" s="2"/>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
       <c r="H98" s="2"/>
     </row>
-    <row r="99" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="99" spans="4:8">
       <c r="D99" s="2"/>
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
       <c r="H99" s="2"/>
     </row>
-    <row r="100" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="100" spans="4:8">
       <c r="D100" s="2"/>
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
       <c r="H100" s="2"/>
     </row>
-    <row r="101" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="101" spans="4:8">
       <c r="D101" s="2"/>
       <c r="F101" s="2"/>
       <c r="G101" s="2"/>
       <c r="H101" s="2"/>
     </row>
-    <row r="102" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="102" spans="4:8">
       <c r="D102" s="2"/>
       <c r="F102" s="2"/>
       <c r="G102" s="2"/>
       <c r="H102" s="2"/>
     </row>
-    <row r="103" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="103" spans="4:8">
       <c r="D103" s="2"/>
       <c r="F103" s="2"/>
       <c r="G103" s="2"/>
       <c r="H103" s="2"/>
     </row>
-    <row r="104" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="104" spans="4:8">
       <c r="D104" s="2"/>
       <c r="F104" s="2"/>
       <c r="G104" s="2"/>
       <c r="H104" s="2"/>
     </row>
-    <row r="105" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="105" spans="4:8">
       <c r="D105" s="2"/>
       <c r="F105" s="2"/>
       <c r="G105" s="2"/>
       <c r="H105" s="2"/>
     </row>
-    <row r="106" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="106" spans="4:8">
       <c r="D106" s="2"/>
       <c r="F106" s="2"/>
       <c r="G106" s="2"/>
       <c r="H106" s="2"/>
     </row>
-    <row r="107" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="107" spans="4:8">
       <c r="D107" s="2"/>
       <c r="F107" s="2"/>
       <c r="G107" s="2"/>
       <c r="H107" s="2"/>
     </row>
-    <row r="108" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="108" spans="4:8">
       <c r="D108" s="2"/>
       <c r="F108" s="2"/>
       <c r="G108" s="2"/>
       <c r="H108" s="2"/>
     </row>
-    <row r="109" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="109" spans="4:8">
       <c r="D109" s="2"/>
       <c r="F109" s="2"/>
       <c r="G109" s="2"/>
       <c r="H109" s="2"/>
     </row>
-    <row r="110" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="110" spans="4:8">
       <c r="D110" s="2"/>
       <c r="F110" s="2"/>
       <c r="G110" s="2"/>
       <c r="H110" s="2"/>
     </row>
-    <row r="111" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="111" spans="4:8">
       <c r="D111" s="2"/>
       <c r="F111" s="2"/>
       <c r="G111" s="2"/>
       <c r="H111" s="2"/>
     </row>
-    <row r="112" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="112" spans="4:8">
       <c r="D112" s="2"/>
       <c r="F112" s="2"/>
       <c r="G112" s="2"/>
       <c r="H112" s="2"/>
     </row>
-    <row r="113" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="113" spans="4:8">
       <c r="D113" s="2"/>
       <c r="F113" s="2"/>
       <c r="G113" s="2"/>
       <c r="H113" s="2"/>
     </row>
-    <row r="114" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="114" spans="4:8">
       <c r="D114" s="2"/>
       <c r="F114" s="2"/>
       <c r="G114" s="2"/>
       <c r="H114" s="2"/>
     </row>
-    <row r="115" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="115" spans="4:8">
       <c r="D115" s="2"/>
       <c r="F115" s="2"/>
       <c r="G115" s="2"/>
       <c r="H115" s="2"/>
     </row>
-    <row r="116" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="116" spans="4:8">
       <c r="D116" s="2"/>
       <c r="F116" s="2"/>
       <c r="G116" s="2"/>
       <c r="H116" s="2"/>
     </row>
-    <row r="117" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="117" spans="4:8">
       <c r="D117" s="2"/>
       <c r="F117" s="2"/>
       <c r="G117" s="2"/>
       <c r="H117" s="2"/>
     </row>
-    <row r="118" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="118" spans="4:8">
       <c r="D118" s="2"/>
       <c r="F118" s="2"/>
       <c r="G118" s="2"/>
       <c r="H118" s="2"/>
     </row>
-    <row r="119" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="119" spans="4:8">
       <c r="D119" s="2"/>
       <c r="F119" s="2"/>
       <c r="G119" s="2"/>
       <c r="H119" s="2"/>
     </row>
-    <row r="120" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="120" spans="4:8">
       <c r="D120" s="2"/>
       <c r="F120" s="2"/>
       <c r="G120" s="2"/>
       <c r="H120" s="2"/>
     </row>
-    <row r="121" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="121" spans="4:8">
       <c r="D121" s="2"/>
       <c r="F121" s="2"/>
       <c r="G121" s="2"/>
       <c r="H121" s="2"/>
     </row>
-    <row r="122" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="122" spans="4:8">
       <c r="D122" s="2"/>
       <c r="F122" s="2"/>
       <c r="G122" s="2"/>
       <c r="H122" s="2"/>
     </row>
-    <row r="123" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="123" spans="4:8">
       <c r="D123" s="2"/>
       <c r="F123" s="2"/>
       <c r="G123" s="2"/>
       <c r="H123" s="2"/>
     </row>
-    <row r="124" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="124" spans="4:8">
       <c r="D124" s="2"/>
       <c r="F124" s="2"/>
       <c r="G124" s="2"/>
       <c r="H124" s="2"/>
     </row>
-    <row r="125" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="125" spans="4:8">
       <c r="D125" s="2"/>
       <c r="F125" s="2"/>
       <c r="G125" s="2"/>
       <c r="H125" s="2"/>
     </row>
-    <row r="126" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="126" spans="4:8">
       <c r="D126" s="2"/>
       <c r="F126" s="2"/>
       <c r="G126" s="2"/>
       <c r="H126" s="2"/>
     </row>
-    <row r="127" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="127" spans="4:8">
       <c r="D127" s="2"/>
       <c r="F127" s="2"/>
       <c r="G127" s="2"/>
       <c r="H127" s="2"/>
     </row>
-    <row r="128" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="128" spans="4:8">
       <c r="D128" s="2"/>
       <c r="F128" s="2"/>
       <c r="G128" s="2"/>
       <c r="H128" s="2"/>
     </row>
-    <row r="129" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="129" spans="4:8">
       <c r="D129" s="2"/>
       <c r="F129" s="2"/>
       <c r="G129" s="2"/>
       <c r="H129" s="2"/>
     </row>
-    <row r="130" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="130" spans="4:8">
       <c r="D130" s="2"/>
       <c r="F130" s="2"/>
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
     </row>
-    <row r="131" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="131" spans="4:8">
       <c r="D131" s="2"/>
       <c r="F131" s="2"/>
       <c r="G131" s="2"/>
       <c r="H131" s="2"/>
     </row>
-    <row r="132" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="132" spans="4:8">
       <c r="D132" s="2"/>
       <c r="F132" s="2"/>
       <c r="G132" s="2"/>
       <c r="H132" s="2"/>
     </row>
-    <row r="133" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="133" spans="4:8">
       <c r="D133" s="2"/>
       <c r="F133" s="2"/>
       <c r="G133" s="2"/>
       <c r="H133" s="2"/>
     </row>
-    <row r="134" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="134" spans="4:8">
       <c r="D134" s="2"/>
       <c r="F134" s="2"/>
       <c r="G134" s="2"/>
       <c r="H134" s="2"/>
     </row>
-    <row r="135" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="135" spans="4:8">
       <c r="D135" s="2"/>
       <c r="F135" s="2"/>
       <c r="G135" s="2"/>
       <c r="H135" s="2"/>
     </row>
-    <row r="136" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="136" spans="4:8">
       <c r="D136" s="2"/>
       <c r="F136" s="2"/>
       <c r="G136" s="2"/>
       <c r="H136" s="2"/>
     </row>
-    <row r="137" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="137" spans="4:8">
       <c r="D137" s="2"/>
       <c r="F137" s="2"/>
       <c r="G137" s="2"/>
       <c r="H137" s="2"/>
     </row>
-    <row r="138" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="138" spans="4:8">
       <c r="D138" s="2"/>
       <c r="F138" s="2"/>
       <c r="G138" s="2"/>
       <c r="H138" s="2"/>
     </row>
-    <row r="139" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="139" spans="4:8">
       <c r="D139" s="2"/>
       <c r="F139" s="2"/>
       <c r="G139" s="2"/>
       <c r="H139" s="2"/>
     </row>
-    <row r="140" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="140" spans="4:8">
       <c r="D140" s="2"/>
       <c r="F140" s="2"/>
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
     </row>
-    <row r="141" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="141" spans="4:8">
       <c r="D141" s="2"/>
       <c r="F141" s="2"/>
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
     </row>
-    <row r="142" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="142" spans="4:8">
       <c r="D142" s="2"/>
       <c r="F142" s="2"/>
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
     </row>
-    <row r="143" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="143" spans="4:8">
       <c r="D143" s="2"/>
       <c r="F143" s="2"/>
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
     </row>
-    <row r="144" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="144" spans="4:8">
       <c r="D144" s="2"/>
       <c r="F144" s="2"/>
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
     </row>
-    <row r="145" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="145" spans="4:8">
       <c r="D145" s="2"/>
       <c r="F145" s="2"/>
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
     </row>
-    <row r="146" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="146" spans="4:8">
       <c r="D146" s="2"/>
       <c r="F146" s="2"/>
       <c r="G146" s="2"/>
       <c r="H146" s="2"/>
     </row>
-    <row r="147" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="147" spans="4:8">
       <c r="D147" s="2"/>
       <c r="F147" s="2"/>
       <c r="G147" s="2"/>
       <c r="H147" s="2"/>
     </row>
-    <row r="148" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="148" spans="4:8">
       <c r="D148" s="2"/>
       <c r="F148" s="2"/>
       <c r="G148" s="2"/>
       <c r="H148" s="2"/>
     </row>
-    <row r="149" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="149" spans="4:8">
       <c r="D149" s="2"/>
       <c r="F149" s="2"/>
       <c r="G149" s="2"/>
       <c r="H149" s="2"/>
     </row>
-    <row r="150" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="150" spans="4:8">
       <c r="D150" s="2"/>
       <c r="F150" s="2"/>
       <c r="G150" s="2"/>
       <c r="H150" s="2"/>
     </row>
-    <row r="151" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="151" spans="4:8">
       <c r="D151" s="2"/>
       <c r="F151" s="2"/>
       <c r="G151" s="2"/>
       <c r="H151" s="2"/>
     </row>
-    <row r="152" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="152" spans="4:8">
       <c r="D152" s="2"/>
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
       <c r="H152" s="2"/>
     </row>
-    <row r="153" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="153" spans="4:8">
       <c r="D153" s="2"/>
       <c r="F153" s="2"/>
       <c r="G153" s="2"/>
       <c r="H153" s="2"/>
     </row>
-    <row r="154" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="154" spans="4:8">
       <c r="D154" s="2"/>
       <c r="F154" s="2"/>
       <c r="G154" s="2"/>
       <c r="H154" s="2"/>
     </row>
-    <row r="155" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="155" spans="4:8">
       <c r="D155" s="2"/>
       <c r="F155" s="2"/>
       <c r="G155" s="2"/>
       <c r="H155" s="2"/>
     </row>
-    <row r="156" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="156" spans="4:8">
       <c r="D156" s="2"/>
       <c r="F156" s="2"/>
       <c r="G156" s="2"/>
       <c r="H156" s="2"/>
     </row>
-    <row r="157" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="157" spans="4:8">
       <c r="D157" s="2"/>
       <c r="F157" s="2"/>
       <c r="G157" s="2"/>
       <c r="H157" s="2"/>
     </row>
-    <row r="158" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="158" spans="4:8">
       <c r="D158" s="2"/>
       <c r="F158" s="2"/>
       <c r="G158" s="2"/>
       <c r="H158" s="2"/>
     </row>
-    <row r="159" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="159" spans="4:8">
       <c r="D159" s="2"/>
       <c r="F159" s="2"/>
       <c r="G159" s="2"/>
       <c r="H159" s="2"/>
     </row>
-    <row r="160" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="160" spans="4:8">
       <c r="D160" s="2"/>
       <c r="F160" s="2"/>
       <c r="G160" s="2"/>
       <c r="H160" s="2"/>
     </row>
-    <row r="161" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="161" spans="4:8">
       <c r="D161" s="2"/>
       <c r="F161" s="2"/>
       <c r="G161" s="2"/>
       <c r="H161" s="2"/>
     </row>
-    <row r="162" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="162" spans="4:8">
       <c r="D162" s="2"/>
       <c r="F162" s="2"/>
       <c r="G162" s="2"/>
       <c r="H162" s="2"/>
     </row>
-    <row r="163" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="163" spans="4:8">
       <c r="D163" s="2"/>
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
       <c r="H163" s="2"/>
     </row>
-    <row r="164" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="164" spans="4:8">
       <c r="D164" s="2"/>
       <c r="F164" s="2"/>
       <c r="G164" s="2"/>
       <c r="H164" s="2"/>
     </row>
-    <row r="165" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="165" spans="4:8">
       <c r="D165" s="2"/>
       <c r="F165" s="2"/>
       <c r="G165" s="2"/>
       <c r="H165" s="2"/>
     </row>
-    <row r="166" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="166" spans="4:8">
       <c r="D166" s="2"/>
       <c r="F166" s="2"/>
       <c r="G166" s="2"/>
       <c r="H166" s="2"/>
     </row>
-    <row r="167" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="167" spans="4:8">
       <c r="D167" s="2"/>
       <c r="F167" s="2"/>
       <c r="G167" s="2"/>
       <c r="H167" s="2"/>
     </row>
-    <row r="168" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="168" spans="4:8">
       <c r="D168" s="2"/>
       <c r="F168" s="2"/>
       <c r="G168" s="2"/>
       <c r="H168" s="2"/>
     </row>
-    <row r="169" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="169" spans="4:8">
       <c r="D169" s="2"/>
       <c r="F169" s="2"/>
       <c r="G169" s="2"/>
       <c r="H169" s="2"/>
     </row>
-    <row r="170" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="170" spans="4:8">
       <c r="D170" s="2"/>
       <c r="F170" s="2"/>
       <c r="G170" s="2"/>
       <c r="H170" s="2"/>
     </row>
-    <row r="171" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="171" spans="4:8">
       <c r="D171" s="2"/>
       <c r="F171" s="2"/>
       <c r="G171" s="2"/>
       <c r="H171" s="2"/>
     </row>
-    <row r="172" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="172" spans="4:8">
       <c r="D172" s="2"/>
       <c r="F172" s="2"/>
       <c r="G172" s="2"/>
       <c r="H172" s="2"/>
     </row>
-    <row r="173" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="173" spans="4:8">
       <c r="D173" s="2"/>
       <c r="F173" s="2"/>
       <c r="G173" s="2"/>
       <c r="H173" s="2"/>
     </row>
-    <row r="174" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="174" spans="4:8">
       <c r="D174" s="2"/>
       <c r="F174" s="2"/>
       <c r="G174" s="2"/>
       <c r="H174" s="2"/>
     </row>
-    <row r="175" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="175" spans="4:8">
       <c r="D175" s="2"/>
       <c r="F175" s="2"/>
       <c r="G175" s="2"/>
       <c r="H175" s="2"/>
     </row>
-    <row r="176" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="176" spans="4:8">
       <c r="D176" s="2"/>
       <c r="F176" s="2"/>
       <c r="G176" s="2"/>
       <c r="H176" s="2"/>
     </row>
-    <row r="177" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="177" spans="4:8">
       <c r="D177" s="2"/>
       <c r="F177" s="2"/>
       <c r="G177" s="2"/>
       <c r="H177" s="2"/>
     </row>
-    <row r="178" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="178" spans="4:8">
       <c r="D178" s="2"/>
       <c r="F178" s="2"/>
       <c r="G178" s="2"/>
       <c r="H178" s="2"/>
     </row>
-    <row r="179" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="179" spans="4:8">
       <c r="D179" s="2"/>
       <c r="F179" s="2"/>
       <c r="G179" s="2"/>
       <c r="H179" s="2"/>
     </row>
-    <row r="180" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="180" spans="4:8">
       <c r="D180" s="2"/>
       <c r="F180" s="2"/>
       <c r="G180" s="2"/>
       <c r="H180" s="2"/>
     </row>
-    <row r="181" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="181" spans="4:8">
       <c r="D181" s="2"/>
       <c r="F181" s="2"/>
       <c r="G181" s="2"/>
       <c r="H181" s="2"/>
     </row>
-    <row r="182" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="182" spans="4:8">
       <c r="D182" s="2"/>
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
       <c r="H182" s="2"/>
     </row>
-    <row r="183" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="183" spans="4:8">
       <c r="D183" s="2"/>
       <c r="F183" s="2"/>
       <c r="G183" s="2"/>
       <c r="H183" s="2"/>
     </row>
-    <row r="184" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="184" spans="4:8">
       <c r="D184" s="2"/>
       <c r="F184" s="2"/>
       <c r="G184" s="2"/>
       <c r="H184" s="2"/>
     </row>
-    <row r="185" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="185" spans="4:8">
       <c r="D185" s="2"/>
       <c r="F185" s="2"/>
       <c r="G185" s="2"/>
       <c r="H185" s="2"/>
     </row>
-    <row r="186" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="186" spans="4:8">
       <c r="D186" s="2"/>
       <c r="F186" s="2"/>
       <c r="G186" s="2"/>
       <c r="H186" s="2"/>
     </row>
-    <row r="187" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="187" spans="4:8">
       <c r="D187" s="2"/>
       <c r="F187" s="2"/>
       <c r="G187" s="2"/>
       <c r="H187" s="2"/>
     </row>
-    <row r="188" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="188" spans="4:8">
       <c r="D188" s="2"/>
       <c r="F188" s="2"/>
       <c r="G188" s="2"/>
       <c r="H188" s="2"/>
     </row>
-    <row r="189" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="189" spans="4:8">
       <c r="D189" s="2"/>
       <c r="F189" s="2"/>
       <c r="G189" s="2"/>
       <c r="H189" s="2"/>
     </row>
-    <row r="190" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="190" spans="4:8">
       <c r="D190" s="2"/>
       <c r="F190" s="2"/>
       <c r="G190" s="2"/>
       <c r="H190" s="2"/>
     </row>
-    <row r="191" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="191" spans="4:8">
       <c r="D191" s="2"/>
       <c r="F191" s="2"/>
       <c r="G191" s="2"/>
       <c r="H191" s="2"/>
     </row>
-    <row r="192" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="192" spans="4:8">
       <c r="D192" s="2"/>
       <c r="F192" s="2"/>
       <c r="G192" s="2"/>
       <c r="H192" s="2"/>
     </row>
-    <row r="193" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="193" spans="4:8">
       <c r="D193" s="2"/>
       <c r="F193" s="2"/>
       <c r="G193" s="2"/>
       <c r="H193" s="2"/>
     </row>
-    <row r="194" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="194" spans="4:8">
       <c r="D194" s="2"/>
       <c r="F194" s="2"/>
       <c r="G194" s="2"/>
       <c r="H194" s="2"/>
     </row>
-    <row r="195" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="195" spans="4:8">
       <c r="D195" s="2"/>
       <c r="F195" s="2"/>
       <c r="G195" s="2"/>
       <c r="H195" s="2"/>
     </row>
-    <row r="196" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="196" spans="4:8">
       <c r="D196" s="2"/>
       <c r="F196" s="2"/>
       <c r="G196" s="2"/>
       <c r="H196" s="2"/>
     </row>
-    <row r="197" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="197" spans="4:8">
       <c r="D197" s="2"/>
       <c r="F197" s="2"/>
       <c r="G197" s="2"/>
       <c r="H197" s="2"/>
     </row>
-    <row r="198" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="198" spans="4:8">
       <c r="D198" s="2"/>
       <c r="F198" s="2"/>
       <c r="G198" s="2"/>
       <c r="H198" s="2"/>
     </row>
-    <row r="199" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="199" spans="4:8">
       <c r="D199" s="2"/>
       <c r="F199" s="2"/>
       <c r="G199" s="2"/>
       <c r="H199" s="2"/>
     </row>
-    <row r="200" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="200" spans="4:8">
       <c r="D200" s="2"/>
       <c r="F200" s="2"/>
       <c r="G200" s="2"/>
       <c r="H200" s="2"/>
     </row>
-    <row r="201" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="201" spans="4:8">
       <c r="D201" s="2"/>
       <c r="F201" s="2"/>
       <c r="G201" s="2"/>
       <c r="H201" s="2"/>
     </row>
-    <row r="202" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="202" spans="4:8">
       <c r="D202" s="2"/>
       <c r="F202" s="2"/>
       <c r="G202" s="2"/>
       <c r="H202" s="2"/>
     </row>
-    <row r="203" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="203" spans="4:8">
       <c r="D203" s="2"/>
       <c r="F203" s="2"/>
       <c r="G203" s="2"/>
       <c r="H203" s="2"/>
     </row>
-    <row r="204" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="204" spans="4:8">
       <c r="D204" s="2"/>
       <c r="F204" s="2"/>
       <c r="G204" s="2"/>
       <c r="H204" s="2"/>
     </row>
-    <row r="205" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="205" spans="4:8">
       <c r="D205" s="2"/>
       <c r="F205" s="2"/>
       <c r="G205" s="2"/>
       <c r="H205" s="2"/>
     </row>
-    <row r="206" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="206" spans="4:8">
       <c r="D206" s="2"/>
       <c r="F206" s="2"/>
       <c r="G206" s="2"/>
       <c r="H206" s="2"/>
     </row>
-    <row r="207" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="207" spans="4:8">
       <c r="D207" s="2"/>
       <c r="F207" s="2"/>
       <c r="G207" s="2"/>
       <c r="H207" s="2"/>
     </row>
-    <row r="208" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="208" spans="4:8">
       <c r="D208" s="2"/>
       <c r="F208" s="2"/>
       <c r="G208" s="2"/>
       <c r="H208" s="2"/>
     </row>
-    <row r="209" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="209" spans="4:8">
       <c r="D209" s="2"/>
       <c r="F209" s="2"/>
       <c r="G209" s="2"/>
       <c r="H209" s="2"/>
     </row>
-    <row r="210" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="210" spans="4:8">
       <c r="D210" s="2"/>
       <c r="F210" s="2"/>
       <c r="G210" s="2"/>
       <c r="H210" s="2"/>
     </row>
-    <row r="211" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="211" spans="4:8">
       <c r="D211" s="2"/>
       <c r="F211" s="2"/>
       <c r="G211" s="2"/>
       <c r="H211" s="2"/>
     </row>
-    <row r="212" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="212" spans="4:8">
       <c r="D212" s="2"/>
       <c r="F212" s="2"/>
       <c r="G212" s="2"/>
       <c r="H212" s="2"/>
     </row>
-    <row r="213" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="213" spans="4:8">
       <c r="D213" s="2"/>
       <c r="F213" s="2"/>
       <c r="G213" s="2"/>
       <c r="H213" s="2"/>
     </row>
-    <row r="214" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="214" spans="4:8">
       <c r="D214" s="2"/>
       <c r="F214" s="2"/>
       <c r="G214" s="2"/>
       <c r="H214" s="2"/>
     </row>
-    <row r="215" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="215" spans="4:8">
       <c r="D215" s="2"/>
       <c r="F215" s="2"/>
       <c r="G215" s="2"/>
       <c r="H215" s="2"/>
     </row>
-    <row r="216" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="216" spans="4:8">
       <c r="D216" s="2"/>
       <c r="F216" s="2"/>
       <c r="G216" s="2"/>
       <c r="H216" s="2"/>
     </row>
-    <row r="217" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="217" spans="4:8">
       <c r="D217" s="2"/>
       <c r="F217" s="2"/>
       <c r="G217" s="2"/>
       <c r="H217" s="2"/>
     </row>
-    <row r="218" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="218" spans="4:8">
       <c r="D218" s="2"/>
       <c r="F218" s="2"/>
       <c r="G218" s="2"/>
       <c r="H218" s="2"/>
     </row>
-    <row r="219" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="219" spans="4:8">
       <c r="D219" s="2"/>
       <c r="F219" s="2"/>
       <c r="G219" s="2"/>
       <c r="H219" s="2"/>
     </row>
-    <row r="220" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="220" spans="4:8">
       <c r="D220" s="2"/>
       <c r="F220" s="2"/>
       <c r="G220" s="2"/>
       <c r="H220" s="2"/>
     </row>
-    <row r="221" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="221" spans="4:8">
       <c r="D221" s="2"/>
       <c r="F221" s="2"/>
       <c r="G221" s="2"/>
       <c r="H221" s="2"/>
     </row>
-    <row r="222" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="222" spans="4:8">
       <c r="D222" s="2"/>
       <c r="F222" s="2"/>
       <c r="G222" s="2"/>
       <c r="H222" s="2"/>
     </row>
-    <row r="223" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="223" spans="4:8">
       <c r="D223" s="2"/>
       <c r="F223" s="2"/>
       <c r="G223" s="2"/>
       <c r="H223" s="2"/>
     </row>
-    <row r="224" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="224" spans="4:8">
       <c r="D224" s="2"/>
       <c r="F224" s="2"/>
       <c r="G224" s="2"/>
       <c r="H224" s="2"/>
     </row>
-    <row r="225" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="225" spans="4:8">
       <c r="D225" s="2"/>
       <c r="F225" s="2"/>
       <c r="G225" s="2"/>
       <c r="H225" s="2"/>
     </row>
-    <row r="226" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="226" spans="4:8">
       <c r="D226" s="2"/>
       <c r="F226" s="2"/>
       <c r="G226" s="2"/>
       <c r="H226" s="2"/>
     </row>
-    <row r="227" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="227" spans="4:8">
       <c r="D227" s="2"/>
       <c r="F227" s="2"/>
       <c r="G227" s="2"/>
       <c r="H227" s="2"/>
     </row>
-    <row r="228" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="228" spans="4:8">
       <c r="D228" s="2"/>
       <c r="F228" s="2"/>
       <c r="G228" s="2"/>
       <c r="H228" s="2"/>
     </row>
-    <row r="229" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="229" spans="4:8">
       <c r="D229" s="2"/>
       <c r="F229" s="2"/>
       <c r="G229" s="2"/>
       <c r="H229" s="2"/>
     </row>
-    <row r="230" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="230" spans="4:8">
       <c r="D230" s="2"/>
       <c r="F230" s="2"/>
       <c r="G230" s="2"/>
       <c r="H230" s="2"/>
     </row>
-    <row r="231" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="231" spans="4:8">
       <c r="D231" s="2"/>
       <c r="F231" s="2"/>
       <c r="G231" s="2"/>
       <c r="H231" s="2"/>
     </row>
-    <row r="232" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="232" spans="4:8">
       <c r="D232" s="2"/>
       <c r="F232" s="2"/>
       <c r="G232" s="2"/>
       <c r="H232" s="2"/>
     </row>
-    <row r="233" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="233" spans="4:8">
       <c r="D233" s="2"/>
       <c r="F233" s="2"/>
       <c r="G233" s="2"/>
       <c r="H233" s="2"/>
     </row>
-    <row r="234" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="234" spans="4:8">
       <c r="D234" s="2"/>
       <c r="F234" s="2"/>
       <c r="G234" s="2"/>
       <c r="H234" s="2"/>
     </row>
-    <row r="235" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="235" spans="4:8">
       <c r="D235" s="2"/>
       <c r="F235" s="2"/>
       <c r="G235" s="2"/>
       <c r="H235" s="2"/>
     </row>
-    <row r="236" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="236" spans="4:8">
       <c r="D236" s="2"/>
       <c r="F236" s="2"/>
       <c r="G236" s="2"/>
       <c r="H236" s="2"/>
     </row>
-    <row r="237" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="237" spans="4:8">
       <c r="D237" s="2"/>
       <c r="F237" s="2"/>
       <c r="G237" s="2"/>
       <c r="H237" s="2"/>
     </row>
-    <row r="238" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="238" spans="4:8">
       <c r="D238" s="2"/>
       <c r="F238" s="2"/>
       <c r="G238" s="2"/>
       <c r="H238" s="2"/>
     </row>
-    <row r="239" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="239" spans="4:8">
       <c r="D239" s="2"/>
       <c r="F239" s="2"/>
       <c r="G239" s="2"/>
       <c r="H239" s="2"/>
     </row>
-    <row r="240" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="240" spans="4:8">
       <c r="D240" s="2"/>
       <c r="F240" s="2"/>
       <c r="G240" s="2"/>
       <c r="H240" s="2"/>
     </row>
-    <row r="241" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="241" spans="4:8">
       <c r="D241" s="2"/>
       <c r="F241" s="2"/>
       <c r="G241" s="2"/>
       <c r="H241" s="2"/>
     </row>
-    <row r="242" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="242" spans="4:8">
       <c r="D242" s="2"/>
       <c r="F242" s="2"/>
       <c r="G242" s="2"/>
       <c r="H242" s="2"/>
     </row>
-    <row r="243" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="243" spans="4:8">
       <c r="D243" s="2"/>
       <c r="F243" s="2"/>
       <c r="G243" s="2"/>
       <c r="H243" s="2"/>
     </row>
-    <row r="244" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="244" spans="4:8">
       <c r="D244" s="2"/>
       <c r="F244" s="2"/>
       <c r="G244" s="2"/>
       <c r="H244" s="2"/>
     </row>
-    <row r="245" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="245" spans="4:8">
       <c r="D245" s="2"/>
       <c r="F245" s="2"/>
       <c r="G245" s="2"/>
       <c r="H245" s="2"/>
     </row>
-    <row r="246" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="246" spans="4:8">
       <c r="D246" s="2"/>
       <c r="F246" s="2"/>
       <c r="G246" s="2"/>
       <c r="H246" s="2"/>
     </row>
-    <row r="247" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="247" spans="4:8">
       <c r="D247" s="2"/>
       <c r="F247" s="2"/>
       <c r="G247" s="2"/>
       <c r="H247" s="2"/>
     </row>
-    <row r="248" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="248" spans="4:8">
       <c r="D248" s="2"/>
       <c r="F248" s="2"/>
       <c r="G248" s="2"/>
       <c r="H248" s="2"/>
     </row>
-    <row r="249" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="249" spans="4:8">
       <c r="D249" s="2"/>
       <c r="F249" s="2"/>
       <c r="G249" s="2"/>
       <c r="H249" s="2"/>
     </row>
-    <row r="250" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="250" spans="4:8">
       <c r="D250" s="2"/>
       <c r="F250" s="2"/>
       <c r="G250" s="2"/>
       <c r="H250" s="2"/>
     </row>
-    <row r="251" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="251" spans="4:8">
       <c r="D251" s="2"/>
       <c r="F251" s="2"/>
       <c r="G251" s="2"/>
       <c r="H251" s="2"/>
     </row>
-    <row r="252" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="252" spans="4:8">
       <c r="D252" s="2"/>
       <c r="F252" s="2"/>
       <c r="G252" s="2"/>
       <c r="H252" s="2"/>
     </row>
-    <row r="253" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="253" spans="4:8">
       <c r="D253" s="2"/>
       <c r="F253" s="2"/>
       <c r="G253" s="2"/>
       <c r="H253" s="2"/>
     </row>
-    <row r="254" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="254" spans="4:8">
       <c r="D254" s="2"/>
       <c r="F254" s="2"/>
       <c r="G254" s="2"/>
       <c r="H254" s="2"/>
     </row>
-    <row r="255" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="255" spans="4:8">
       <c r="D255" s="2"/>
       <c r="F255" s="2"/>
       <c r="G255" s="2"/>
       <c r="H255" s="2"/>
     </row>
-    <row r="256" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="256" spans="4:8">
       <c r="D256" s="2"/>
       <c r="F256" s="2"/>
       <c r="G256" s="2"/>
       <c r="H256" s="2"/>
     </row>
-    <row r="257" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="257" spans="4:8">
       <c r="D257" s="2"/>
       <c r="F257" s="2"/>
       <c r="G257" s="2"/>
       <c r="H257" s="2"/>
     </row>
-    <row r="258" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="258" spans="4:8">
       <c r="D258" s="2"/>
       <c r="F258" s="2"/>
       <c r="G258" s="2"/>
       <c r="H258" s="2"/>
     </row>
-    <row r="259" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="259" spans="4:8">
       <c r="D259" s="2"/>
       <c r="F259" s="2"/>
       <c r="G259" s="2"/>
       <c r="H259" s="2"/>
     </row>
-    <row r="260" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="260" spans="4:8">
       <c r="D260" s="2"/>
       <c r="F260" s="2"/>
       <c r="G260" s="2"/>
       <c r="H260" s="2"/>
     </row>
-    <row r="261" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="261" spans="4:8">
       <c r="D261" s="2"/>
       <c r="F261" s="2"/>
       <c r="G261" s="2"/>
       <c r="H261" s="2"/>
     </row>
-    <row r="262" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="262" spans="4:8">
       <c r="D262" s="2"/>
       <c r="F262" s="2"/>
       <c r="G262" s="2"/>
       <c r="H262" s="2"/>
     </row>
-    <row r="263" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="263" spans="4:8">
       <c r="D263" s="2"/>
       <c r="F263" s="2"/>
       <c r="G263" s="2"/>
       <c r="H263" s="2"/>
     </row>
-    <row r="264" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="264" spans="4:8">
       <c r="D264" s="2"/>
       <c r="F264" s="2"/>
       <c r="G264" s="2"/>
       <c r="H264" s="2"/>
     </row>
-    <row r="265" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="265" spans="4:8">
       <c r="D265" s="2"/>
       <c r="F265" s="2"/>
       <c r="G265" s="2"/>
       <c r="H265" s="2"/>
     </row>
-    <row r="266" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="266" spans="4:8">
       <c r="D266" s="2"/>
       <c r="F266" s="2"/>
       <c r="G266" s="2"/>
       <c r="H266" s="2"/>
     </row>
-    <row r="267" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="267" spans="4:8">
       <c r="D267" s="2"/>
       <c r="F267" s="2"/>
       <c r="G267" s="2"/>
       <c r="H267" s="2"/>
     </row>
-    <row r="268" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="268" spans="4:8">
       <c r="D268" s="2"/>
       <c r="F268" s="2"/>
       <c r="G268" s="2"/>
       <c r="H268" s="2"/>
     </row>
-    <row r="269" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="269" spans="4:8">
       <c r="D269" s="2"/>
       <c r="F269" s="2"/>
       <c r="G269" s="2"/>
       <c r="H269" s="2"/>
     </row>
-    <row r="270" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="270" spans="4:8">
       <c r="D270" s="2"/>
       <c r="F270" s="2"/>
       <c r="G270" s="2"/>
       <c r="H270" s="2"/>
     </row>
-    <row r="271" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="271" spans="4:8">
       <c r="D271" s="2"/>
       <c r="F271" s="2"/>
       <c r="G271" s="2"/>
       <c r="H271" s="2"/>
     </row>
-    <row r="272" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="272" spans="4:8">
       <c r="D272" s="2"/>
       <c r="F272" s="2"/>
       <c r="G272" s="2"/>
       <c r="H272" s="2"/>
     </row>
-    <row r="273" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="273" spans="4:8">
       <c r="D273" s="2"/>
       <c r="F273" s="2"/>
       <c r="G273" s="2"/>
       <c r="H273" s="2"/>
     </row>
-    <row r="274" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="274" spans="4:8">
       <c r="D274" s="2"/>
       <c r="F274" s="2"/>
       <c r="G274" s="2"/>
       <c r="H274" s="2"/>
     </row>
-    <row r="275" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="275" spans="4:8">
       <c r="D275" s="2"/>
       <c r="F275" s="2"/>
       <c r="G275" s="2"/>
       <c r="H275" s="2"/>
     </row>
-    <row r="276" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="276" spans="4:8">
       <c r="D276" s="2"/>
       <c r="F276" s="2"/>
       <c r="G276" s="2"/>
       <c r="H276" s="2"/>
     </row>
-    <row r="277" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="277" spans="4:8">
       <c r="D277" s="2"/>
       <c r="F277" s="2"/>
       <c r="G277" s="2"/>
       <c r="H277" s="2"/>
     </row>
-    <row r="278" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="278" spans="4:8">
       <c r="D278" s="2"/>
       <c r="F278" s="2"/>
       <c r="G278" s="2"/>
       <c r="H278" s="2"/>
     </row>
-    <row r="279" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="279" spans="4:8">
       <c r="D279" s="2"/>
       <c r="F279" s="2"/>
       <c r="G279" s="2"/>
       <c r="H279" s="2"/>
     </row>
-    <row r="280" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="280" spans="4:8">
       <c r="D280" s="2"/>
       <c r="F280" s="2"/>
       <c r="G280" s="2"/>
       <c r="H280" s="2"/>
     </row>
-    <row r="281" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="281" spans="4:8">
       <c r="D281" s="2"/>
       <c r="F281" s="2"/>
       <c r="G281" s="2"/>
       <c r="H281" s="2"/>
     </row>
-    <row r="282" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="282" spans="4:8">
       <c r="D282" s="2"/>
       <c r="F282" s="2"/>
       <c r="G282" s="2"/>
       <c r="H282" s="2"/>
     </row>
-    <row r="283" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="283" spans="4:8">
       <c r="D283" s="2"/>
       <c r="F283" s="2"/>
       <c r="G283" s="2"/>
       <c r="H283" s="2"/>
     </row>
-    <row r="284" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="284" spans="4:8">
       <c r="D284" s="2"/>
       <c r="F284" s="2"/>
       <c r="G284" s="2"/>
       <c r="H284" s="2"/>
     </row>
-    <row r="285" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="285" spans="4:8">
       <c r="D285" s="2"/>
       <c r="F285" s="2"/>
       <c r="G285" s="2"/>
       <c r="H285" s="2"/>
     </row>
-    <row r="286" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="286" spans="4:8">
       <c r="D286" s="2"/>
       <c r="F286" s="2"/>
       <c r="G286" s="2"/>
       <c r="H286" s="2"/>
     </row>
-    <row r="287" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="287" spans="4:8">
       <c r="D287" s="2"/>
       <c r="F287" s="2"/>
       <c r="G287" s="2"/>
       <c r="H287" s="2"/>
     </row>
-    <row r="288" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="288" spans="4:8">
       <c r="D288" s="2"/>
       <c r="F288" s="2"/>
       <c r="G288" s="2"/>
       <c r="H288" s="2"/>
     </row>
-    <row r="289" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="289" spans="4:8">
       <c r="D289" s="2"/>
       <c r="F289" s="2"/>
       <c r="G289" s="2"/>
       <c r="H289" s="2"/>
     </row>
-    <row r="290" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="290" spans="4:8">
       <c r="D290" s="2"/>
       <c r="F290" s="2"/>
       <c r="G290" s="2"/>
       <c r="H290" s="2"/>
     </row>
-    <row r="291" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="291" spans="4:8">
       <c r="D291" s="2"/>
       <c r="F291" s="2"/>
       <c r="G291" s="2"/>
       <c r="H291" s="2"/>
     </row>
-    <row r="292" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="292" spans="4:8">
       <c r="D292" s="2"/>
       <c r="F292" s="2"/>
       <c r="G292" s="2"/>
       <c r="H292" s="2"/>
     </row>
-    <row r="293" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="293" spans="4:8">
       <c r="D293" s="2"/>
       <c r="F293" s="2"/>
       <c r="G293" s="2"/>
       <c r="H293" s="2"/>
     </row>
-    <row r="294" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="294" spans="4:8">
       <c r="D294" s="2"/>
       <c r="F294" s="2"/>
       <c r="G294" s="2"/>
       <c r="H294" s="2"/>
     </row>
-    <row r="295" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="295" spans="4:8">
       <c r="D295" s="2"/>
       <c r="F295" s="2"/>
       <c r="G295" s="2"/>
       <c r="H295" s="2"/>
     </row>
-    <row r="296" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="296" spans="4:8">
       <c r="D296" s="2"/>
       <c r="F296" s="2"/>
       <c r="G296" s="2"/>
       <c r="H296" s="2"/>
     </row>
-    <row r="297" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="297" spans="4:8">
       <c r="D297" s="2"/>
       <c r="F297" s="2"/>
       <c r="G297" s="2"/>
       <c r="H297" s="2"/>
     </row>
-    <row r="298" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="298" spans="4:8">
       <c r="D298" s="2"/>
       <c r="F298" s="2"/>
       <c r="G298" s="2"/>
       <c r="H298" s="2"/>
     </row>
-    <row r="299" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="299" spans="4:8">
       <c r="D299" s="2"/>
       <c r="F299" s="2"/>
       <c r="G299" s="2"/>
       <c r="H299" s="2"/>
     </row>
-    <row r="300" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="300" spans="4:8">
       <c r="D300" s="2"/>
       <c r="F300" s="2"/>
       <c r="G300" s="2"/>
       <c r="H300" s="2"/>
     </row>
-    <row r="301" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="301" spans="4:8">
       <c r="D301" s="2"/>
       <c r="F301" s="2"/>
       <c r="G301" s="2"/>
       <c r="H301" s="2"/>
     </row>
-    <row r="302" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="302" spans="4:8">
       <c r="D302" s="2"/>
       <c r="F302" s="2"/>
       <c r="G302" s="2"/>
       <c r="H302" s="2"/>
     </row>
-    <row r="303" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="303" spans="4:8">
       <c r="D303" s="2"/>
       <c r="F303" s="2"/>
       <c r="G303" s="2"/>
       <c r="H303" s="2"/>
     </row>
-    <row r="304" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="304" spans="4:8">
       <c r="D304" s="2"/>
       <c r="F304" s="2"/>
       <c r="G304" s="2"/>
       <c r="H304" s="2"/>
     </row>
-    <row r="305" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="305" spans="4:8">
       <c r="D305" s="2"/>
       <c r="F305" s="2"/>
       <c r="G305" s="2"/>
       <c r="H305" s="2"/>
     </row>
-    <row r="306" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="306" spans="4:8">
       <c r="D306" s="2"/>
       <c r="F306" s="2"/>
       <c r="G306" s="2"/>
       <c r="H306" s="2"/>
     </row>
-    <row r="307" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="307" spans="4:8">
       <c r="D307" s="2"/>
       <c r="F307" s="2"/>
       <c r="G307" s="2"/>
       <c r="H307" s="2"/>
     </row>
-    <row r="308" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="308" spans="4:8">
       <c r="D308" s="2"/>
       <c r="F308" s="2"/>
       <c r="G308" s="2"/>
       <c r="H308" s="2"/>
     </row>
-    <row r="309" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="309" spans="4:8">
       <c r="D309" s="2"/>
       <c r="F309" s="2"/>
       <c r="G309" s="2"/>
       <c r="H309" s="2"/>
     </row>
-    <row r="310" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="310" spans="4:8">
       <c r="D310" s="2"/>
       <c r="F310" s="2"/>
       <c r="G310" s="2"/>
       <c r="H310" s="2"/>
     </row>
-    <row r="311" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="311" spans="4:8">
       <c r="D311" s="2"/>
       <c r="F311" s="2"/>
       <c r="G311" s="2"/>
       <c r="H311" s="2"/>
     </row>
-    <row r="312" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="312" spans="4:8">
       <c r="D312" s="2"/>
       <c r="F312" s="2"/>
       <c r="G312" s="2"/>
       <c r="H312" s="2"/>
     </row>
-    <row r="313" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="313" spans="4:8">
       <c r="D313" s="2"/>
       <c r="F313" s="2"/>
       <c r="G313" s="2"/>
       <c r="H313" s="2"/>
     </row>
-    <row r="314" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="314" spans="4:8">
       <c r="D314" s="2"/>
       <c r="F314" s="2"/>
       <c r="G314" s="2"/>
       <c r="H314" s="2"/>
     </row>
-    <row r="315" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="315" spans="4:8">
       <c r="D315" s="2"/>
       <c r="F315" s="2"/>
       <c r="G315" s="2"/>
       <c r="H315" s="2"/>
     </row>
-    <row r="316" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="316" spans="4:8">
       <c r="D316" s="2"/>
       <c r="F316" s="2"/>
       <c r="G316" s="2"/>
       <c r="H316" s="2"/>
     </row>
-    <row r="317" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="317" spans="4:8">
       <c r="D317" s="2"/>
       <c r="F317" s="2"/>
       <c r="G317" s="2"/>
       <c r="H317" s="2"/>
     </row>
-    <row r="318" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="318" spans="4:8">
       <c r="D318" s="2"/>
       <c r="F318" s="2"/>
       <c r="G318" s="2"/>
       <c r="H318" s="2"/>
     </row>
-    <row r="319" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="319" spans="4:8">
       <c r="D319" s="2"/>
       <c r="F319" s="2"/>
       <c r="G319" s="2"/>
       <c r="H319" s="2"/>
     </row>
-    <row r="320" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="320" spans="4:8">
       <c r="D320" s="2"/>
       <c r="F320" s="2"/>
       <c r="G320" s="2"/>
       <c r="H320" s="2"/>
     </row>
-    <row r="321" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="321" spans="4:8">
       <c r="D321" s="2"/>
       <c r="F321" s="2"/>
       <c r="G321" s="2"/>
       <c r="H321" s="2"/>
     </row>
-    <row r="322" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="322" spans="4:8">
       <c r="D322" s="2"/>
       <c r="F322" s="2"/>
       <c r="G322" s="2"/>
       <c r="H322" s="2"/>
     </row>
-    <row r="323" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="323" spans="4:8">
       <c r="D323" s="2"/>
       <c r="F323" s="2"/>
       <c r="G323" s="2"/>
       <c r="H323" s="2"/>
     </row>
-    <row r="324" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="324" spans="4:8">
       <c r="D324" s="2"/>
       <c r="F324" s="2"/>
       <c r="G324" s="2"/>
       <c r="H324" s="2"/>
     </row>
-    <row r="325" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="325" spans="4:8">
       <c r="D325" s="2"/>
       <c r="F325" s="2"/>
       <c r="G325" s="2"/>
       <c r="H325" s="2"/>
     </row>
-    <row r="326" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="326" spans="4:8">
       <c r="D326" s="2"/>
       <c r="F326" s="2"/>
       <c r="G326" s="2"/>
       <c r="H326" s="2"/>
     </row>
-    <row r="327" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="327" spans="4:8">
       <c r="D327" s="2"/>
       <c r="F327" s="2"/>
       <c r="G327" s="2"/>
       <c r="H327" s="2"/>
     </row>
-    <row r="328" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="328" spans="4:8">
       <c r="D328" s="2"/>
       <c r="F328" s="2"/>
       <c r="G328" s="2"/>
       <c r="H328" s="2"/>
     </row>
-    <row r="329" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="329" spans="4:8">
       <c r="D329" s="2"/>
       <c r="F329" s="2"/>
       <c r="G329" s="2"/>
       <c r="H329" s="2"/>
     </row>
-    <row r="330" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="330" spans="4:8">
       <c r="D330" s="2"/>
       <c r="F330" s="2"/>
       <c r="G330" s="2"/>
       <c r="H330" s="2"/>
     </row>
-    <row r="331" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="331" spans="4:8">
       <c r="D331" s="2"/>
       <c r="F331" s="2"/>
       <c r="G331" s="2"/>
       <c r="H331" s="2"/>
     </row>
-    <row r="332" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="332" spans="4:8">
       <c r="D332" s="2"/>
       <c r="F332" s="2"/>
       <c r="G332" s="2"/>
       <c r="H332" s="2"/>
     </row>
-    <row r="333" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="333" spans="4:8">
       <c r="D333" s="2"/>
       <c r="F333" s="2"/>
       <c r="G333" s="2"/>
       <c r="H333" s="2"/>
     </row>
-    <row r="334" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="334" spans="4:8">
       <c r="D334" s="2"/>
       <c r="F334" s="2"/>
       <c r="G334" s="2"/>
       <c r="H334" s="2"/>
     </row>
-    <row r="335" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="335" spans="4:8">
       <c r="D335" s="2"/>
       <c r="F335" s="2"/>
       <c r="G335" s="2"/>
       <c r="H335" s="2"/>
     </row>
-    <row r="336" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="336" spans="4:8">
       <c r="D336" s="2"/>
       <c r="F336" s="2"/>
       <c r="G336" s="2"/>
       <c r="H336" s="2"/>
     </row>
-    <row r="337" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="337" spans="4:8">
       <c r="D337" s="2"/>
       <c r="F337" s="2"/>
       <c r="G337" s="2"/>
       <c r="H337" s="2"/>
     </row>
-    <row r="338" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="338" spans="4:8">
       <c r="D338" s="2"/>
       <c r="F338" s="2"/>
       <c r="G338" s="2"/>
       <c r="H338" s="2"/>
     </row>
-    <row r="339" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="339" spans="4:8">
       <c r="D339" s="2"/>
       <c r="F339" s="2"/>
       <c r="G339" s="2"/>
       <c r="H339" s="2"/>
     </row>
-    <row r="340" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="340" spans="4:8">
       <c r="D340" s="2"/>
       <c r="F340" s="2"/>
       <c r="G340" s="2"/>
       <c r="H340" s="2"/>
     </row>
-    <row r="341" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="341" spans="4:8">
       <c r="D341" s="2"/>
       <c r="F341" s="2"/>
       <c r="G341" s="2"/>
       <c r="H341" s="2"/>
     </row>
-    <row r="342" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="342" spans="4:8">
       <c r="D342" s="2"/>
       <c r="F342" s="2"/>
       <c r="G342" s="2"/>
       <c r="H342" s="2"/>
     </row>
-    <row r="343" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="343" spans="4:8">
       <c r="D343" s="2"/>
       <c r="F343" s="2"/>
       <c r="G343" s="2"/>
       <c r="H343" s="2"/>
     </row>
-    <row r="344" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="344" spans="4:8">
       <c r="D344" s="2"/>
       <c r="F344" s="2"/>
       <c r="G344" s="2"/>
       <c r="H344" s="2"/>
     </row>
-    <row r="345" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="345" spans="4:8">
       <c r="D345" s="2"/>
       <c r="F345" s="2"/>
       <c r="G345" s="2"/>
       <c r="H345" s="2"/>
     </row>
-    <row r="346" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="346" spans="4:8">
       <c r="D346" s="2"/>
       <c r="F346" s="2"/>
       <c r="G346" s="2"/>
       <c r="H346" s="2"/>
     </row>
-    <row r="347" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="347" spans="4:8">
       <c r="D347" s="2"/>
       <c r="F347" s="2"/>
       <c r="G347" s="2"/>
       <c r="H347" s="2"/>
     </row>
-    <row r="348" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="348" spans="4:8">
       <c r="D348" s="2"/>
       <c r="F348" s="2"/>
       <c r="G348" s="2"/>
       <c r="H348" s="2"/>
     </row>
-    <row r="349" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="349" spans="4:8">
       <c r="D349" s="2"/>
       <c r="F349" s="2"/>
       <c r="G349" s="2"/>
       <c r="H349" s="2"/>
     </row>
-    <row r="350" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="350" spans="4:8">
       <c r="D350" s="2"/>
       <c r="F350" s="2"/>
       <c r="G350" s="2"/>
       <c r="H350" s="2"/>
     </row>
-    <row r="351" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="351" spans="4:8">
       <c r="D351" s="2"/>
       <c r="F351" s="2"/>
       <c r="G351" s="2"/>
       <c r="H351" s="2"/>
     </row>
-    <row r="352" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="352" spans="4:8">
       <c r="D352" s="2"/>
       <c r="F352" s="2"/>
       <c r="G352" s="2"/>
       <c r="H352" s="2"/>
     </row>
-    <row r="353" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="353" spans="4:8">
       <c r="D353" s="2"/>
       <c r="F353" s="2"/>
       <c r="G353" s="2"/>
       <c r="H353" s="2"/>
     </row>
-    <row r="354" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="354" spans="4:8">
       <c r="D354" s="2"/>
       <c r="F354" s="2"/>
       <c r="G354" s="2"/>
       <c r="H354" s="2"/>
     </row>
-    <row r="355" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="355" spans="4:8">
       <c r="D355" s="2"/>
       <c r="F355" s="2"/>
       <c r="G355" s="2"/>
       <c r="H355" s="2"/>
     </row>
-    <row r="356" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="356" spans="4:8">
       <c r="D356" s="2"/>
       <c r="F356" s="2"/>
       <c r="G356" s="2"/>
       <c r="H356" s="2"/>
     </row>
-    <row r="357" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="357" spans="4:8">
       <c r="D357" s="2"/>
       <c r="F357" s="2"/>
       <c r="G357" s="2"/>
       <c r="H357" s="2"/>
     </row>
-    <row r="358" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="358" spans="4:8">
       <c r="D358" s="2"/>
       <c r="F358" s="2"/>
       <c r="G358" s="2"/>
       <c r="H358" s="2"/>
     </row>
-    <row r="359" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="359" spans="4:8">
       <c r="D359" s="2"/>
       <c r="F359" s="2"/>
       <c r="G359" s="2"/>
       <c r="H359" s="2"/>
     </row>
-    <row r="360" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="360" spans="4:8">
       <c r="D360" s="2"/>
       <c r="F360" s="2"/>
       <c r="G360" s="2"/>
       <c r="H360" s="2"/>
     </row>
-    <row r="361" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="361" spans="4:8">
       <c r="D361" s="2"/>
       <c r="F361" s="2"/>
       <c r="G361" s="2"/>
       <c r="H361" s="2"/>
     </row>
-    <row r="362" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="362" spans="4:8">
       <c r="D362" s="2"/>
       <c r="F362" s="2"/>
       <c r="G362" s="2"/>
       <c r="H362" s="2"/>
     </row>
-    <row r="363" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="363" spans="4:8">
       <c r="D363" s="2"/>
       <c r="F363" s="2"/>
       <c r="G363" s="2"/>
       <c r="H363" s="2"/>
     </row>
-    <row r="364" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="364" spans="4:8">
       <c r="D364" s="2"/>
       <c r="F364" s="2"/>
       <c r="G364" s="2"/>
       <c r="H364" s="2"/>
     </row>
-    <row r="365" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="365" spans="4:8">
       <c r="D365" s="2"/>
       <c r="F365" s="2"/>
       <c r="G365" s="2"/>
       <c r="H365" s="2"/>
     </row>
-    <row r="366" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="366" spans="4:8">
       <c r="D366" s="2"/>
       <c r="F366" s="2"/>
       <c r="G366" s="2"/>
       <c r="H366" s="2"/>
     </row>
-    <row r="367" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="367" spans="4:8">
       <c r="D367" s="2"/>
       <c r="F367" s="2"/>
       <c r="G367" s="2"/>
       <c r="H367" s="2"/>
     </row>
-    <row r="368" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="368" spans="4:8">
       <c r="D368" s="2"/>
       <c r="F368" s="2"/>
       <c r="G368" s="2"/>
       <c r="H368" s="2"/>
     </row>
-    <row r="369" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="369" spans="4:8">
       <c r="D369" s="2"/>
       <c r="F369" s="2"/>
       <c r="G369" s="2"/>
       <c r="H369" s="2"/>
     </row>
-    <row r="370" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="370" spans="4:8">
       <c r="D370" s="2"/>
       <c r="F370" s="2"/>
       <c r="G370" s="2"/>
       <c r="H370" s="2"/>
     </row>
-    <row r="371" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="371" spans="4:8">
       <c r="D371" s="2"/>
       <c r="F371" s="2"/>
       <c r="G371" s="2"/>
       <c r="H371" s="2"/>
     </row>
-    <row r="372" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="372" spans="4:8">
       <c r="D372" s="2"/>
       <c r="F372" s="2"/>
       <c r="G372" s="2"/>
       <c r="H372" s="2"/>
     </row>
-    <row r="373" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="373" spans="4:8">
       <c r="D373" s="2"/>
       <c r="F373" s="2"/>
       <c r="G373" s="2"/>
       <c r="H373" s="2"/>
     </row>
-    <row r="374" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="374" spans="4:8">
       <c r="D374" s="2"/>
       <c r="F374" s="2"/>
       <c r="G374" s="2"/>
       <c r="H374" s="2"/>
     </row>
-    <row r="375" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="375" spans="4:8">
       <c r="D375" s="2"/>
       <c r="F375" s="2"/>
       <c r="G375" s="2"/>
       <c r="H375" s="2"/>
     </row>
-    <row r="376" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="376" spans="4:8">
       <c r="D376" s="2"/>
       <c r="F376" s="2"/>
       <c r="G376" s="2"/>
       <c r="H376" s="2"/>
     </row>
-    <row r="377" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="377" spans="4:8">
       <c r="D377" s="2"/>
       <c r="F377" s="2"/>
       <c r="G377" s="2"/>
       <c r="H377" s="2"/>
     </row>
-    <row r="378" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="378" spans="4:8">
       <c r="D378" s="2"/>
       <c r="F378" s="2"/>
       <c r="G378" s="2"/>
       <c r="H378" s="2"/>
     </row>
-    <row r="379" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="379" spans="4:8">
       <c r="D379" s="2"/>
       <c r="F379" s="2"/>
       <c r="G379" s="2"/>
       <c r="H379" s="2"/>
     </row>
-    <row r="380" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="380" spans="4:8">
       <c r="D380" s="2"/>
       <c r="F380" s="2"/>
       <c r="G380" s="2"/>
       <c r="H380" s="2"/>
     </row>
-    <row r="381" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="381" spans="4:8">
       <c r="D381" s="2"/>
       <c r="F381" s="2"/>
       <c r="G381" s="2"/>
       <c r="H381" s="2"/>
     </row>
-    <row r="382" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="382" spans="4:8">
       <c r="D382" s="2"/>
       <c r="F382" s="2"/>
       <c r="G382" s="2"/>
       <c r="H382" s="2"/>
     </row>
-    <row r="383" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="383" spans="4:8">
       <c r="D383" s="2"/>
       <c r="F383" s="2"/>
       <c r="G383" s="2"/>
       <c r="H383" s="2"/>
     </row>
-    <row r="384" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="384" spans="4:8">
       <c r="D384" s="2"/>
       <c r="F384" s="2"/>
       <c r="G384" s="2"/>
       <c r="H384" s="2"/>
     </row>
-    <row r="385" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="385" spans="4:8">
       <c r="D385" s="2"/>
       <c r="F385" s="2"/>
       <c r="G385" s="2"/>
       <c r="H385" s="2"/>
     </row>
-    <row r="386" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="386" spans="4:8">
       <c r="D386" s="2"/>
       <c r="F386" s="2"/>
       <c r="G386" s="2"/>
       <c r="H386" s="2"/>
     </row>
-    <row r="387" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="387" spans="4:8">
       <c r="D387" s="2"/>
       <c r="F387" s="2"/>
       <c r="G387" s="2"/>
       <c r="H387" s="2"/>
     </row>
-    <row r="388" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="388" spans="4:8">
       <c r="D388" s="2"/>
       <c r="F388" s="2"/>
       <c r="G388" s="2"/>
       <c r="H388" s="2"/>
     </row>
-    <row r="389" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="389" spans="4:8">
       <c r="D389" s="2"/>
       <c r="F389" s="2"/>
       <c r="G389" s="2"/>
       <c r="H389" s="2"/>
     </row>
-    <row r="390" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="390" spans="4:8">
       <c r="D390" s="2"/>
       <c r="F390" s="2"/>
       <c r="G390" s="2"/>
       <c r="H390" s="2"/>
     </row>
-    <row r="391" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="391" spans="4:8">
       <c r="D391" s="2"/>
       <c r="F391" s="2"/>
       <c r="G391" s="2"/>
       <c r="H391" s="2"/>
     </row>
-    <row r="392" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="392" spans="4:8">
       <c r="D392" s="2"/>
       <c r="F392" s="2"/>
       <c r="G392" s="2"/>
       <c r="H392" s="2"/>
     </row>
-    <row r="393" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="393" spans="4:8">
       <c r="D393" s="2"/>
       <c r="F393" s="2"/>
       <c r="G393" s="2"/>
       <c r="H393" s="2"/>
     </row>
-    <row r="394" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="394" spans="4:8">
       <c r="D394" s="2"/>
       <c r="F394" s="2"/>
       <c r="G394" s="2"/>
       <c r="H394" s="2"/>
     </row>
-    <row r="395" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="395" spans="4:8">
       <c r="D395" s="2"/>
       <c r="F395" s="2"/>
       <c r="G395" s="2"/>
       <c r="H395" s="2"/>
     </row>
-    <row r="396" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="396" spans="4:8">
       <c r="D396" s="2"/>
       <c r="F396" s="2"/>
       <c r="G396" s="2"/>
       <c r="H396" s="2"/>
     </row>
-    <row r="397" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="397" spans="4:8">
       <c r="D397" s="2"/>
       <c r="F397" s="2"/>
       <c r="G397" s="2"/>
       <c r="H397" s="2"/>
     </row>
-    <row r="398" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="398" spans="4:8">
       <c r="D398" s="2"/>
       <c r="F398" s="2"/>
       <c r="G398" s="2"/>
       <c r="H398" s="2"/>
     </row>
-    <row r="399" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="399" spans="4:8">
       <c r="D399" s="2"/>
       <c r="F399" s="2"/>
       <c r="G399" s="2"/>
       <c r="H399" s="2"/>
     </row>
-    <row r="400" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="400" spans="4:8">
       <c r="D400" s="2"/>
       <c r="F400" s="2"/>
       <c r="G400" s="2"/>
       <c r="H400" s="2"/>
     </row>
-    <row r="401" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="401" spans="4:8">
       <c r="D401" s="2"/>
       <c r="F401" s="2"/>
       <c r="G401" s="2"/>
       <c r="H401" s="2"/>
     </row>
-    <row r="402" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="402" spans="4:8">
       <c r="D402" s="2"/>
       <c r="F402" s="2"/>
       <c r="G402" s="2"/>
       <c r="H402" s="2"/>
     </row>
-    <row r="403" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="403" spans="4:8">
       <c r="D403" s="2"/>
       <c r="F403" s="2"/>
       <c r="G403" s="2"/>
       <c r="H403" s="2"/>
     </row>
-    <row r="404" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="404" spans="4:8">
       <c r="D404" s="2"/>
       <c r="F404" s="2"/>
       <c r="G404" s="2"/>
       <c r="H404" s="2"/>
     </row>
-    <row r="405" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="405" spans="4:8">
       <c r="D405" s="2"/>
       <c r="F405" s="2"/>
       <c r="G405" s="2"/>
       <c r="H405" s="2"/>
     </row>
-    <row r="406" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="406" spans="4:8">
       <c r="D406" s="2"/>
       <c r="F406" s="2"/>
       <c r="G406" s="2"/>
       <c r="H406" s="2"/>
     </row>
-    <row r="407" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="407" spans="4:8">
       <c r="D407" s="2"/>
       <c r="F407" s="2"/>
       <c r="G407" s="2"/>
       <c r="H407" s="2"/>
     </row>
-    <row r="408" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="408" spans="4:8">
       <c r="D408" s="2"/>
       <c r="F408" s="2"/>
       <c r="G408" s="2"/>
       <c r="H408" s="2"/>
     </row>
-    <row r="409" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="409" spans="4:8">
       <c r="D409" s="2"/>
       <c r="F409" s="2"/>
       <c r="G409" s="2"/>
       <c r="H409" s="2"/>
     </row>
-    <row r="410" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="410" spans="4:8">
       <c r="D410" s="2"/>
       <c r="F410" s="2"/>
       <c r="G410" s="2"/>
       <c r="H410" s="2"/>
     </row>
-    <row r="411" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="411" spans="4:8">
       <c r="D411" s="2"/>
       <c r="F411" s="2"/>
       <c r="G411" s="2"/>
       <c r="H411" s="2"/>
     </row>
-    <row r="412" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="412" spans="4:8">
       <c r="D412" s="2"/>
       <c r="F412" s="2"/>
       <c r="G412" s="2"/>
       <c r="H412" s="2"/>
     </row>
-    <row r="413" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="413" spans="4:8">
       <c r="D413" s="2"/>
       <c r="F413" s="2"/>
       <c r="G413" s="2"/>
       <c r="H413" s="2"/>
     </row>
-    <row r="414" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="414" spans="4:8">
       <c r="D414" s="2"/>
       <c r="F414" s="2"/>
       <c r="G414" s="2"/>
       <c r="H414" s="2"/>
     </row>
-    <row r="415" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="415" spans="4:8">
       <c r="D415" s="2"/>
       <c r="F415" s="2"/>
       <c r="G415" s="2"/>
       <c r="H415" s="2"/>
     </row>
-    <row r="416" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="416" spans="4:8">
       <c r="D416" s="2"/>
       <c r="F416" s="2"/>
       <c r="G416" s="2"/>
       <c r="H416" s="2"/>
     </row>
-    <row r="417" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="417" spans="4:8">
       <c r="D417" s="2"/>
       <c r="F417" s="2"/>
       <c r="G417" s="2"/>
       <c r="H417" s="2"/>
     </row>
-    <row r="418" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="418" spans="4:8">
       <c r="D418" s="2"/>
       <c r="F418" s="2"/>
       <c r="G418" s="2"/>
       <c r="H418" s="2"/>
     </row>
-    <row r="419" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="419" spans="4:8">
       <c r="D419" s="2"/>
       <c r="F419" s="2"/>
       <c r="G419" s="2"/>
       <c r="H419" s="2"/>
     </row>
-    <row r="420" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="420" spans="4:8">
       <c r="D420" s="2"/>
       <c r="F420" s="2"/>
       <c r="G420" s="2"/>
       <c r="H420" s="2"/>
     </row>
-    <row r="421" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="421" spans="4:8">
       <c r="D421" s="2"/>
       <c r="F421" s="2"/>
       <c r="G421" s="2"/>
       <c r="H421" s="2"/>
     </row>
-    <row r="422" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="422" spans="4:8">
       <c r="D422" s="2"/>
       <c r="F422" s="2"/>
       <c r="G422" s="2"/>
       <c r="H422" s="2"/>
     </row>
-    <row r="423" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="423" spans="4:8">
       <c r="D423" s="2"/>
       <c r="F423" s="2"/>
       <c r="G423" s="2"/>
       <c r="H423" s="2"/>
     </row>
-    <row r="424" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="424" spans="4:8">
       <c r="D424" s="2"/>
       <c r="F424" s="2"/>
       <c r="G424" s="2"/>
       <c r="H424" s="2"/>
     </row>
-    <row r="425" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="425" spans="4:8">
       <c r="D425" s="2"/>
       <c r="F425" s="2"/>
       <c r="G425" s="2"/>
       <c r="H425" s="2"/>
     </row>
-    <row r="426" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="426" spans="4:8">
       <c r="D426" s="2"/>
       <c r="F426" s="2"/>
       <c r="G426" s="2"/>
       <c r="H426" s="2"/>
     </row>
-    <row r="427" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="427" spans="4:8">
       <c r="D427" s="2"/>
       <c r="F427" s="2"/>
       <c r="G427" s="2"/>
       <c r="H427" s="2"/>
     </row>
-    <row r="428" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="428" spans="4:8">
       <c r="D428" s="2"/>
       <c r="F428" s="2"/>
       <c r="G428" s="2"/>
       <c r="H428" s="2"/>
     </row>
-    <row r="429" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="429" spans="4:8">
       <c r="D429" s="2"/>
       <c r="F429" s="2"/>
       <c r="G429" s="2"/>
       <c r="H429" s="2"/>
     </row>
-    <row r="430" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="430" spans="4:8">
       <c r="D430" s="2"/>
       <c r="F430" s="2"/>
       <c r="G430" s="2"/>
       <c r="H430" s="2"/>
     </row>
-    <row r="431" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="431" spans="4:8">
       <c r="D431" s="2"/>
       <c r="F431" s="2"/>
       <c r="G431" s="2"/>
       <c r="H431" s="2"/>
     </row>
-    <row r="432" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="432" spans="4:8">
       <c r="D432" s="2"/>
       <c r="F432" s="2"/>
       <c r="G432" s="2"/>
       <c r="H432" s="2"/>
     </row>
-    <row r="433" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="433" spans="4:8">
       <c r="D433" s="2"/>
       <c r="F433" s="2"/>
       <c r="G433" s="2"/>
       <c r="H433" s="2"/>
     </row>
-    <row r="434" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="434" spans="4:8">
       <c r="D434" s="2"/>
       <c r="F434" s="2"/>
       <c r="G434" s="2"/>
       <c r="H434" s="2"/>
     </row>
-    <row r="435" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="435" spans="4:8">
       <c r="D435" s="2"/>
       <c r="F435" s="2"/>
       <c r="G435" s="2"/>
       <c r="H435" s="2"/>
     </row>
-    <row r="436" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="436" spans="4:8">
       <c r="D436" s="2"/>
       <c r="F436" s="2"/>
       <c r="G436" s="2"/>
       <c r="H436" s="2"/>
     </row>
-    <row r="437" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="437" spans="4:8">
       <c r="D437" s="2"/>
       <c r="F437" s="2"/>
       <c r="G437" s="2"/>
       <c r="H437" s="2"/>
     </row>
-    <row r="438" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="438" spans="4:8">
       <c r="D438" s="2"/>
       <c r="F438" s="2"/>
       <c r="G438" s="2"/>
       <c r="H438" s="2"/>
     </row>
-    <row r="439" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="439" spans="4:8">
       <c r="D439" s="2"/>
       <c r="F439" s="2"/>
       <c r="G439" s="2"/>
       <c r="H439" s="2"/>
     </row>
-    <row r="440" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="440" spans="4:8">
       <c r="D440" s="2"/>
       <c r="F440" s="2"/>
       <c r="G440" s="2"/>
       <c r="H440" s="2"/>
     </row>
-    <row r="441" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="441" spans="4:8">
       <c r="D441" s="2"/>
       <c r="F441" s="2"/>
       <c r="G441" s="2"/>
       <c r="H441" s="2"/>
     </row>
-    <row r="442" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="442" spans="4:8">
       <c r="D442" s="2"/>
       <c r="F442" s="2"/>
       <c r="G442" s="2"/>
       <c r="H442" s="2"/>
     </row>
-    <row r="443" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="443" spans="4:8">
       <c r="D443" s="2"/>
       <c r="F443" s="2"/>
       <c r="G443" s="2"/>
       <c r="H443" s="2"/>
     </row>
-    <row r="444" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="444" spans="4:8">
       <c r="D444" s="2"/>
       <c r="F444" s="2"/>
       <c r="G444" s="2"/>
       <c r="H444" s="2"/>
     </row>
-    <row r="445" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="445" spans="4:8">
       <c r="D445" s="2"/>
       <c r="F445" s="2"/>
       <c r="G445" s="2"/>
       <c r="H445" s="2"/>
     </row>
-    <row r="446" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="446" spans="4:8">
       <c r="D446" s="2"/>
       <c r="F446" s="2"/>
       <c r="G446" s="2"/>
       <c r="H446" s="2"/>
     </row>
-    <row r="447" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="447" spans="4:8">
       <c r="D447" s="2"/>
       <c r="F447" s="2"/>
       <c r="G447" s="2"/>
       <c r="H447" s="2"/>
     </row>
-    <row r="448" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="448" spans="4:8">
       <c r="D448" s="2"/>
       <c r="F448" s="2"/>
       <c r="G448" s="2"/>
       <c r="H448" s="2"/>
     </row>
-    <row r="449" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="449" spans="4:8">
       <c r="D449" s="2"/>
       <c r="F449" s="2"/>
       <c r="G449" s="2"/>
       <c r="H449" s="2"/>
     </row>
-    <row r="450" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="450" spans="4:8">
       <c r="D450" s="2"/>
       <c r="F450" s="2"/>
       <c r="G450" s="2"/>
       <c r="H450" s="2"/>
     </row>
-    <row r="451" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="451" spans="4:8">
       <c r="D451" s="2"/>
       <c r="F451" s="2"/>
       <c r="G451" s="2"/>
       <c r="H451" s="2"/>
     </row>
-    <row r="452" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="452" spans="4:8">
       <c r="D452" s="2"/>
       <c r="F452" s="2"/>
       <c r="G452" s="2"/>
       <c r="H452" s="2"/>
     </row>
-    <row r="453" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="453" spans="4:8">
       <c r="D453" s="2"/>
       <c r="F453" s="2"/>
       <c r="G453" s="2"/>
       <c r="H453" s="2"/>
     </row>
-    <row r="454" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="454" spans="4:8">
       <c r="D454" s="2"/>
       <c r="F454" s="2"/>
       <c r="G454" s="2"/>
       <c r="H454" s="2"/>
     </row>
-    <row r="455" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="455" spans="4:8">
       <c r="D455" s="2"/>
       <c r="F455" s="2"/>
       <c r="G455" s="2"/>
       <c r="H455" s="2"/>
     </row>
-    <row r="456" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="456" spans="4:8">
       <c r="D456" s="2"/>
       <c r="F456" s="2"/>
       <c r="G456" s="2"/>
       <c r="H456" s="2"/>
     </row>
-    <row r="457" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="457" spans="4:8">
       <c r="D457" s="2"/>
       <c r="F457" s="2"/>
       <c r="G457" s="2"/>
       <c r="H457" s="2"/>
     </row>
-    <row r="458" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="458" spans="4:8">
       <c r="D458" s="2"/>
       <c r="F458" s="2"/>
       <c r="G458" s="2"/>
       <c r="H458" s="2"/>
     </row>
-    <row r="459" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="459" spans="4:8">
       <c r="D459" s="2"/>
       <c r="F459" s="2"/>
       <c r="G459" s="2"/>
       <c r="H459" s="2"/>
     </row>
-    <row r="460" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="460" spans="4:8">
       <c r="D460" s="2"/>
       <c r="F460" s="2"/>
       <c r="G460" s="2"/>
       <c r="H460" s="2"/>
     </row>
-    <row r="461" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="461" spans="4:8">
       <c r="D461" s="2"/>
       <c r="F461" s="2"/>
       <c r="G461" s="2"/>
       <c r="H461" s="2"/>
     </row>
-    <row r="462" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="462" spans="4:8">
       <c r="D462" s="2"/>
       <c r="F462" s="2"/>
       <c r="G462" s="2"/>
       <c r="H462" s="2"/>
     </row>
-    <row r="463" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="463" spans="4:8">
       <c r="D463" s="2"/>
       <c r="F463" s="2"/>
       <c r="G463" s="2"/>
       <c r="H463" s="2"/>
     </row>
-    <row r="464" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="464" spans="4:8">
       <c r="D464" s="2"/>
       <c r="F464" s="2"/>
       <c r="G464" s="2"/>
       <c r="H464" s="2"/>
     </row>
-    <row r="465" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="465" spans="4:8">
       <c r="D465" s="2"/>
       <c r="F465" s="2"/>
       <c r="G465" s="2"/>
       <c r="H465" s="2"/>
     </row>
-    <row r="466" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="466" spans="4:8">
       <c r="D466" s="2"/>
       <c r="F466" s="2"/>
       <c r="G466" s="2"/>
       <c r="H466" s="2"/>
     </row>
-    <row r="467" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="467" spans="4:8">
       <c r="D467" s="2"/>
       <c r="F467" s="2"/>
       <c r="G467" s="2"/>
       <c r="H467" s="2"/>
     </row>
-    <row r="468" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="468" spans="4:8">
       <c r="D468" s="2"/>
       <c r="F468" s="2"/>
       <c r="G468" s="2"/>
       <c r="H468" s="2"/>
     </row>
-    <row r="469" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="469" spans="4:8">
       <c r="D469" s="2"/>
       <c r="F469" s="2"/>
       <c r="G469" s="2"/>
       <c r="H469" s="2"/>
     </row>
-    <row r="470" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="470" spans="4:8">
       <c r="D470" s="2"/>
       <c r="F470" s="2"/>
       <c r="G470" s="2"/>
       <c r="H470" s="2"/>
     </row>
-    <row r="471" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="471" spans="4:8">
       <c r="D471" s="2"/>
       <c r="F471" s="2"/>
       <c r="G471" s="2"/>
       <c r="H471" s="2"/>
     </row>
-    <row r="472" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="472" spans="4:8">
       <c r="D472" s="2"/>
       <c r="F472" s="2"/>
       <c r="G472" s="2"/>
       <c r="H472" s="2"/>
     </row>
-    <row r="473" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="473" spans="4:8">
       <c r="D473" s="2"/>
       <c r="F473" s="2"/>
       <c r="G473" s="2"/>
       <c r="H473" s="2"/>
     </row>
-    <row r="474" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="474" spans="4:8">
       <c r="D474" s="2"/>
       <c r="F474" s="2"/>
       <c r="G474" s="2"/>
       <c r="H474" s="2"/>
     </row>
-    <row r="475" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="475" spans="4:8">
       <c r="D475" s="2"/>
       <c r="F475" s="2"/>
       <c r="G475" s="2"/>
       <c r="H475" s="2"/>
     </row>
-    <row r="476" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="476" spans="4:8">
       <c r="D476" s="2"/>
       <c r="F476" s="2"/>
       <c r="G476" s="2"/>
       <c r="H476" s="2"/>
     </row>
-    <row r="477" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="477" spans="4:8">
       <c r="D477" s="2"/>
       <c r="F477" s="2"/>
       <c r="G477" s="2"/>
       <c r="H477" s="2"/>
     </row>
-    <row r="478" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="478" spans="4:8">
       <c r="D478" s="2"/>
       <c r="F478" s="2"/>
       <c r="G478" s="2"/>
       <c r="H478" s="2"/>
     </row>
-    <row r="479" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="479" spans="4:8">
       <c r="D479" s="2"/>
       <c r="F479" s="2"/>
       <c r="G479" s="2"/>
       <c r="H479" s="2"/>
     </row>
-    <row r="480" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="480" spans="4:8">
       <c r="D480" s="2"/>
       <c r="F480" s="2"/>
       <c r="G480" s="2"/>
       <c r="H480" s="2"/>
     </row>
-    <row r="481" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="481" spans="4:8">
       <c r="D481" s="2"/>
       <c r="F481" s="2"/>
       <c r="G481" s="2"/>
       <c r="H481" s="2"/>
     </row>
-    <row r="482" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="482" spans="4:8">
       <c r="D482" s="2"/>
       <c r="F482" s="2"/>
       <c r="G482" s="2"/>
       <c r="H482" s="2"/>
     </row>
-    <row r="483" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="483" spans="4:8">
       <c r="D483" s="2"/>
       <c r="F483" s="2"/>
       <c r="G483" s="2"/>
       <c r="H483" s="2"/>
     </row>
-    <row r="484" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="484" spans="4:8">
       <c r="D484" s="2"/>
       <c r="F484" s="2"/>
       <c r="G484" s="2"/>
       <c r="H484" s="2"/>
     </row>
-    <row r="485" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="485" spans="4:8">
       <c r="D485" s="2"/>
       <c r="F485" s="2"/>
       <c r="G485" s="2"/>
       <c r="H485" s="2"/>
     </row>
-    <row r="486" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="486" spans="4:8">
       <c r="D486" s="2"/>
       <c r="F486" s="2"/>
       <c r="G486" s="2"/>
       <c r="H486" s="2"/>
     </row>
-    <row r="487" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="487" spans="4:8">
       <c r="D487" s="2"/>
       <c r="F487" s="2"/>
       <c r="G487" s="2"/>
       <c r="H487" s="2"/>
     </row>
-    <row r="488" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="488" spans="4:8">
       <c r="D488" s="2"/>
       <c r="F488" s="2"/>
       <c r="G488" s="2"/>
       <c r="H488" s="2"/>
     </row>
-    <row r="489" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="489" spans="4:8">
       <c r="D489" s="2"/>
       <c r="F489" s="2"/>
       <c r="G489" s="2"/>
       <c r="H489" s="2"/>
     </row>
-    <row r="490" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="490" spans="4:8">
       <c r="D490" s="2"/>
       <c r="F490" s="2"/>
       <c r="G490" s="2"/>
       <c r="H490" s="2"/>
     </row>
-    <row r="491" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="491" spans="4:8">
       <c r="D491" s="2"/>
       <c r="F491" s="2"/>
       <c r="G491" s="2"/>
       <c r="H491" s="2"/>
     </row>
-    <row r="492" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="492" spans="4:8">
       <c r="D492" s="2"/>
       <c r="F492" s="2"/>
       <c r="G492" s="2"/>
       <c r="H492" s="2"/>
     </row>
-    <row r="493" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="493" spans="4:8">
       <c r="D493" s="2"/>
       <c r="F493" s="2"/>
       <c r="G493" s="2"/>
       <c r="H493" s="2"/>
     </row>
-    <row r="494" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="494" spans="4:8">
       <c r="D494" s="2"/>
       <c r="F494" s="2"/>
       <c r="G494" s="2"/>
       <c r="H494" s="2"/>
     </row>
-    <row r="495" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="495" spans="4:8">
       <c r="D495" s="2"/>
       <c r="F495" s="2"/>
       <c r="G495" s="2"/>
       <c r="H495" s="2"/>
     </row>
-    <row r="496" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="496" spans="4:8">
       <c r="D496" s="2"/>
       <c r="F496" s="2"/>
       <c r="G496" s="2"/>
       <c r="H496" s="2"/>
     </row>
-    <row r="497" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="497" spans="4:8">
       <c r="D497" s="2"/>
       <c r="F497" s="2"/>
       <c r="G497" s="2"/>
       <c r="H497" s="2"/>
     </row>
-    <row r="498" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="498" spans="4:8">
       <c r="D498" s="2"/>
       <c r="F498" s="2"/>
       <c r="G498" s="2"/>
       <c r="H498" s="2"/>
     </row>
-    <row r="499" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="499" spans="4:8">
       <c r="D499" s="2"/>
       <c r="F499" s="2"/>
       <c r="G499" s="2"/>
       <c r="H499" s="2"/>
     </row>
-    <row r="500" spans="4:8" x14ac:dyDescent="0.25">
+    <row r="500" spans="4:8">
       <c r="D500" s="2"/>
       <c r="F500" s="2"/>
       <c r="G500" s="2"/>
       <c r="H500" s="2"/>
     </row>
   </sheetData>
-  <dataValidations count="2">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Unknown treatment type" error="Pick a type from the list (edit types on the &quot;Treatment Types&quot; sheet)." sqref="C10:C500">
-      <formula1>'Treatment Types'!$A$2:$A$30</formula1>
-    </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="Unknown treatment type" error="Pick a type from the list (edit types on the &quot;Treatment Types&quot; sheet)." sqref="C2:C500">
-      <formula1>'Treatment Types'!$A$2:$A$30</formula1>
-    </dataValidation>
-  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" showErrorMessage="1" errorTitle="Unknown treatment type" error="Pick a type from the list (edit types on the &quot;Treatment Types&quot; sheet)." xr:uid="{00000000-0002-0000-0000-000000000000}">
+          <x14:formula1>
+            <xm:f>'Treatment Types'!$A$2:$A$30</xm:f>
+          </x14:formula1>
+          <xm:sqref>C2:C500</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>10</v>
       </c>
       <c r="B2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>29</v>
       </c>
       <c r="B3" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>85</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A39"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="140" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1">
       <c r="A1" s="3" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
       <c r="A3" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
       <c r="A4" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1">
+      <c r="A10" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1">
+      <c r="A11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1">
+      <c r="A12" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1">
+      <c r="A13" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1">
+      <c r="A14" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1">
+      <c r="A15" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1">
+      <c r="A16" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1">
+      <c r="A17" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1">
+      <c r="A18" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1">
+      <c r="A19" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="20" spans="1:1">
+      <c r="A20" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="21" spans="1:1">
+      <c r="A21" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="22" spans="1:1">
+      <c r="A22" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="23" spans="1:1">
+      <c r="A23" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="24" spans="1:1">
+      <c r="A24" t="s">
         <v>134</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="25" spans="1:1">
+      <c r="A25" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="26" spans="1:1">
+      <c r="A26" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1">
+      <c r="A27" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1">
+      <c r="A28" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1">
+      <c r="A29" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="30" spans="1:1">
+      <c r="A30" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1">
+      <c r="A31" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="32" spans="1:1">
+      <c r="A32" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1">
+      <c r="A33" t="s">
         <v>139</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="34" spans="1:1">
+      <c r="A34" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="35" spans="1:1">
+      <c r="A35" t="s">
         <v>141</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="36" spans="1:1">
+      <c r="A36" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1">
+      <c r="A37" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="38" spans="1:1">
+      <c r="A38" t="s">
         <v>143</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="39" spans="1:1">
+      <c r="A39" t="s">
         <v>144</v>
-      </c>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Treatments: fix PRP image filenames
Intro image prp.png -> PRP.jpg, before/after pRP-ba.png -> PRP-ba.png
to match the files in src/assets/images/treatments/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/content/treatments.xlsx
+++ b/src/content/treatments.xlsx
@@ -433,7 +433,7 @@
     <t xml:space="preserve">  • Short Name (optional): a shorter label for compact places. Leave blank to use the Title.</t>
   </si>
   <si>
-    <t>prp.png</t>
+    <t>PRP.jpg</t>
   </si>
   <si>
     <t>PRP</t>
@@ -452,7 +452,7 @@
     <t>PRP Injections are an incredibly effective anti-aging treatment used to eliminate the appearance of fine lines, wrinkles, and to aid in volume loss.</t>
   </si>
   <si>
-    <t>pRP-ba.png</t>
+    <t>PRP-ba.png</t>
   </si>
 </sst>
 </file>

</xml_diff>